<commit_message>
The material table shows before/after/delta for the December re-dispatch
Owner (2026-08-27): 'clearly show how much extra tonnage — what was the
old SAP, what is the new SAP after reallocation, and how much percent
changed.'

Each scenario's 'tonnage by material' table now reads: BEFORE re-dispatch
t/mo · AFTER t/mo · delta t/mo · Change % · Dec sales share · Coverage
after. SAP and LIM-TOS show +0.0% (untouched by design — the cut never
takes a targeted row below its line); LIM-LD shows its reduction (e.g.
3.0.1: 1,903,679 -> 1,819,328, -4.4%, still 105.8% of its share); STOCK
shows NEW +99,120..228,303 t; TOTAL-moved row shows the net effect (the
re-dispatch trades a small LD surplus for a larger stock build — net
tonnage UP in every scenario because the freed trucks work long hauls
instead of overshooting short ones).
</commit_message>
<xml_diff>
--- a/reports/scenario_comparison_dec_options.xlsx
+++ b/reports/scenario_comparison_dec_options.xlsx
@@ -18,10 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="+0.0%;-0.0%"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -126,6 +127,24 @@
       <color rgb="001B7A41"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00A52929"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001B7A41"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000F4C81"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -150,7 +169,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -172,11 +191,12 @@
         <color rgb="00DBE4EE"/>
       </bottom>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -250,6 +270,28 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1059,16 +1101,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H133"/>
+  <dimension ref="A1:H135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1086,6 +1128,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="18" t="inlineStr">
         <is>
@@ -1186,6 +1229,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
@@ -1675,6 +1719,7 @@
         <v>5231542</v>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>
@@ -1690,19 +1735,35 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>t/month (new plan)</t>
+          <t>BEFORE re-dispatch t/mo</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>December sales share</t>
+          <t>AFTER re-dispatch t/mo</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Coverage</t>
-        </is>
-      </c>
+          <t>Δ t/mo</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Change %</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Dec sales share</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Coverage after</t>
+        </is>
+      </c>
+      <c r="H29" s="31" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
@@ -1710,15 +1771,25 @@
           <t>SAP</t>
         </is>
       </c>
-      <c r="B30" s="5" t="n">
+      <c r="B30" s="15" t="n">
         <v>2311732</v>
       </c>
-      <c r="C30" s="5" t="n">
+      <c r="C30" s="32" t="n">
+        <v>2311732</v>
+      </c>
+      <c r="D30" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="15" t="n">
         <v>2311213</v>
       </c>
-      <c r="D30" s="7" t="n">
+      <c r="G30" s="34" t="n">
         <v>1.000224557407734</v>
       </c>
+      <c r="H30" s="31" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
@@ -1726,15 +1797,25 @@
           <t>LIM-TOS</t>
         </is>
       </c>
-      <c r="B31" s="5" t="n">
+      <c r="B31" s="15" t="n">
         <v>1001362</v>
       </c>
-      <c r="C31" s="5" t="n">
+      <c r="C31" s="32" t="n">
+        <v>1001362</v>
+      </c>
+      <c r="D31" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="15" t="n">
         <v>996084</v>
       </c>
-      <c r="D31" s="7" t="n">
+      <c r="G31" s="34" t="n">
         <v>1.005298749904626</v>
       </c>
+      <c r="H31" s="31" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
@@ -1742,35 +1823,87 @@
           <t>LIM-LD</t>
         </is>
       </c>
-      <c r="B32" s="5" t="n">
+      <c r="B32" s="15" t="n">
+        <v>1903679</v>
+      </c>
+      <c r="C32" s="32" t="n">
         <v>1819328</v>
       </c>
-      <c r="C32" s="5" t="n">
+      <c r="D32" s="35" t="n">
+        <v>-84351</v>
+      </c>
+      <c r="E32" s="36" t="n">
+        <v>-0.04430946603917992</v>
+      </c>
+      <c r="F32" s="15" t="n">
         <v>1719964</v>
       </c>
-      <c r="D32" s="7" t="n">
+      <c r="G32" s="34" t="n">
         <v>1.057770976601836</v>
       </c>
+      <c r="H32" s="31" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="26" t="inlineStr">
+      <c r="A33" s="28" t="inlineStr">
         <is>
           <t>STOCK (kilnable, FeNi KM0)</t>
         </is>
       </c>
-      <c r="B33" s="5" t="n">
+      <c r="B33" s="15" t="n"/>
+      <c r="C33" s="32" t="n">
         <v>99120</v>
       </c>
-      <c r="C33" s="30" t="inlineStr">
+      <c r="D33" s="27" t="n">
+        <v>99120</v>
+      </c>
+      <c r="E33" s="26" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="F33" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D33" s="26" t="inlineStr">
+      <c r="G33" s="37" t="inlineStr">
         <is>
           <t>on top of the met sales lines</t>
         </is>
       </c>
+      <c r="H33" s="31" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="38" t="inlineStr">
+        <is>
+          <t>TOTAL moved</t>
+        </is>
+      </c>
+      <c r="B34" s="32" t="n">
+        <v>5216773</v>
+      </c>
+      <c r="C34" s="32" t="n">
+        <v>5231542</v>
+      </c>
+      <c r="D34" s="27" t="n">
+        <v>14769</v>
+      </c>
+      <c r="E34" s="33" t="n">
+        <v>0.002831060504261926</v>
+      </c>
+      <c r="F34" s="31" t="n"/>
+      <c r="G34" s="31" t="n"/>
+      <c r="H34" s="31" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="31" t="n"/>
+      <c r="B35" s="31" t="n"/>
+      <c r="C35" s="31" t="n"/>
+      <c r="D35" s="31" t="n"/>
+      <c r="E35" s="31" t="n"/>
+      <c r="F35" s="31" t="n"/>
+      <c r="G35" s="31" t="n"/>
+      <c r="H35" s="31" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="18" t="inlineStr">
@@ -1872,6 +2005,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="16" t="inlineStr">
         <is>
@@ -2425,6 +2559,7 @@
         <v>5336733</v>
       </c>
     </row>
+    <row r="61"/>
     <row r="62">
       <c r="A62" s="16" t="inlineStr">
         <is>
@@ -2440,19 +2575,35 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>t/month (new plan)</t>
+          <t>BEFORE re-dispatch t/mo</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>December sales share</t>
+          <t>AFTER re-dispatch t/mo</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Coverage</t>
-        </is>
-      </c>
+          <t>Δ t/mo</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Change %</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Dec sales share</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>Coverage after</t>
+        </is>
+      </c>
+      <c r="H63" s="31" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="14" t="inlineStr">
@@ -2460,15 +2611,25 @@
           <t>SAP</t>
         </is>
       </c>
-      <c r="B64" s="5" t="n">
+      <c r="B64" s="15" t="n">
         <v>2311732</v>
       </c>
-      <c r="C64" s="5" t="n">
+      <c r="C64" s="32" t="n">
+        <v>2311732</v>
+      </c>
+      <c r="D64" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" s="15" t="n">
         <v>2311213</v>
       </c>
-      <c r="D64" s="7" t="n">
+      <c r="G64" s="34" t="n">
         <v>1.000224557407734</v>
       </c>
+      <c r="H64" s="31" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="14" t="inlineStr">
@@ -2476,15 +2637,25 @@
           <t>LIM-TOS</t>
         </is>
       </c>
-      <c r="B65" s="5" t="n">
+      <c r="B65" s="15" t="n">
         <v>1000556</v>
       </c>
-      <c r="C65" s="5" t="n">
+      <c r="C65" s="32" t="n">
+        <v>1000556</v>
+      </c>
+      <c r="D65" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" s="15" t="n">
         <v>996084</v>
       </c>
-      <c r="D65" s="7" t="n">
+      <c r="G65" s="34" t="n">
         <v>1.004489581199979</v>
       </c>
+      <c r="H65" s="31" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="14" t="inlineStr">
@@ -2492,35 +2663,87 @@
           <t>LIM-LD</t>
         </is>
       </c>
-      <c r="B66" s="5" t="n">
+      <c r="B66" s="15" t="n">
+        <v>2031523</v>
+      </c>
+      <c r="C66" s="32" t="n">
         <v>1818903</v>
       </c>
-      <c r="C66" s="5" t="n">
+      <c r="D66" s="35" t="n">
+        <v>-212620</v>
+      </c>
+      <c r="E66" s="36" t="n">
+        <v>-0.1046603951813492</v>
+      </c>
+      <c r="F66" s="15" t="n">
         <v>1719964</v>
       </c>
-      <c r="D66" s="7" t="n">
+      <c r="G66" s="34" t="n">
         <v>1.057523878406757</v>
       </c>
+      <c r="H66" s="31" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="26" t="inlineStr">
+      <c r="A67" s="28" t="inlineStr">
         <is>
           <t>STOCK (kilnable, FeNi KM0)</t>
         </is>
       </c>
-      <c r="B67" s="5" t="n">
+      <c r="B67" s="15" t="n"/>
+      <c r="C67" s="32" t="n">
         <v>205542</v>
       </c>
-      <c r="C67" s="30" t="inlineStr">
+      <c r="D67" s="27" t="n">
+        <v>205542</v>
+      </c>
+      <c r="E67" s="26" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="F67" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D67" s="26" t="inlineStr">
+      <c r="G67" s="37" t="inlineStr">
         <is>
           <t>on top of the met sales lines</t>
         </is>
       </c>
+      <c r="H67" s="31" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="38" t="inlineStr">
+        <is>
+          <t>TOTAL moved</t>
+        </is>
+      </c>
+      <c r="B68" s="32" t="n">
+        <v>5343811</v>
+      </c>
+      <c r="C68" s="32" t="n">
+        <v>5336733</v>
+      </c>
+      <c r="D68" s="35" t="n">
+        <v>-7078</v>
+      </c>
+      <c r="E68" s="36" t="n">
+        <v>-0.001324522891995993</v>
+      </c>
+      <c r="F68" s="31" t="n"/>
+      <c r="G68" s="31" t="n"/>
+      <c r="H68" s="31" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="31" t="n"/>
+      <c r="B69" s="31" t="n"/>
+      <c r="C69" s="31" t="n"/>
+      <c r="D69" s="31" t="n"/>
+      <c r="E69" s="31" t="n"/>
+      <c r="F69" s="31" t="n"/>
+      <c r="G69" s="31" t="n"/>
+      <c r="H69" s="31" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="18" t="inlineStr">
@@ -2622,6 +2845,7 @@
         </is>
       </c>
     </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
         <is>
@@ -3111,6 +3335,7 @@
         <v>4994394</v>
       </c>
     </row>
+    <row r="93"/>
     <row r="94">
       <c r="A94" s="16" t="inlineStr">
         <is>
@@ -3126,19 +3351,35 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>t/month (new plan)</t>
+          <t>BEFORE re-dispatch t/mo</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>December sales share</t>
+          <t>AFTER re-dispatch t/mo</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>Coverage</t>
-        </is>
-      </c>
+          <t>Δ t/mo</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>Change %</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>Dec sales share</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>Coverage after</t>
+        </is>
+      </c>
+      <c r="H95" s="31" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
@@ -3146,15 +3387,25 @@
           <t>SAP</t>
         </is>
       </c>
-      <c r="B96" s="5" t="n">
+      <c r="B96" s="15" t="n">
         <v>2315483</v>
       </c>
-      <c r="C96" s="5" t="n">
+      <c r="C96" s="32" t="n">
+        <v>2315483</v>
+      </c>
+      <c r="D96" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" s="15" t="n">
         <v>2311213</v>
       </c>
-      <c r="D96" s="7" t="n">
+      <c r="G96" s="34" t="n">
         <v>1.001847514703318</v>
       </c>
+      <c r="H96" s="31" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="14" t="inlineStr">
@@ -3162,15 +3413,25 @@
           <t>LIM-TOS</t>
         </is>
       </c>
-      <c r="B97" s="5" t="n">
+      <c r="B97" s="15" t="n">
         <v>1332318</v>
       </c>
-      <c r="C97" s="5" t="n">
+      <c r="C97" s="32" t="n">
+        <v>1332318</v>
+      </c>
+      <c r="D97" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F97" s="15" t="n">
         <v>1326082</v>
       </c>
-      <c r="D97" s="7" t="n">
+      <c r="G97" s="34" t="n">
         <v>1.004702574953887</v>
       </c>
+      <c r="H97" s="31" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
@@ -3178,35 +3439,87 @@
           <t>LIM-LD</t>
         </is>
       </c>
-      <c r="B98" s="5" t="n">
+      <c r="B98" s="15" t="n">
+        <v>1323607</v>
+      </c>
+      <c r="C98" s="32" t="n">
         <v>1163826</v>
       </c>
-      <c r="C98" s="5" t="n">
+      <c r="D98" s="35" t="n">
+        <v>-159781</v>
+      </c>
+      <c r="E98" s="36" t="n">
+        <v>-0.1207163455617868</v>
+      </c>
+      <c r="F98" s="15" t="n">
         <v>992213</v>
       </c>
-      <c r="D98" s="7" t="n">
+      <c r="G98" s="34" t="n">
         <v>1.172959838260535</v>
       </c>
+      <c r="H98" s="31" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="26" t="inlineStr">
+      <c r="A99" s="28" t="inlineStr">
         <is>
           <t>STOCK (kilnable, FeNi KM0)</t>
         </is>
       </c>
-      <c r="B99" s="5" t="n">
+      <c r="B99" s="15" t="n"/>
+      <c r="C99" s="32" t="n">
         <v>182767</v>
       </c>
-      <c r="C99" s="30" t="inlineStr">
+      <c r="D99" s="27" t="n">
+        <v>182767</v>
+      </c>
+      <c r="E99" s="26" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="F99" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D99" s="26" t="inlineStr">
+      <c r="G99" s="37" t="inlineStr">
         <is>
           <t>on top of the met sales lines</t>
         </is>
       </c>
+      <c r="H99" s="31" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="38" t="inlineStr">
+        <is>
+          <t>TOTAL moved</t>
+        </is>
+      </c>
+      <c r="B100" s="32" t="n">
+        <v>4971408</v>
+      </c>
+      <c r="C100" s="32" t="n">
+        <v>4994394</v>
+      </c>
+      <c r="D100" s="27" t="n">
+        <v>22986</v>
+      </c>
+      <c r="E100" s="33" t="n">
+        <v>0.004623639821957884</v>
+      </c>
+      <c r="F100" s="31" t="n"/>
+      <c r="G100" s="31" t="n"/>
+      <c r="H100" s="31" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="31" t="n"/>
+      <c r="B101" s="31" t="n"/>
+      <c r="C101" s="31" t="n"/>
+      <c r="D101" s="31" t="n"/>
+      <c r="E101" s="31" t="n"/>
+      <c r="F101" s="31" t="n"/>
+      <c r="G101" s="31" t="n"/>
+      <c r="H101" s="31" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="18" t="inlineStr">
@@ -3308,6 +3621,7 @@
         </is>
       </c>
     </row>
+    <row r="108"/>
     <row r="109">
       <c r="A109" s="16" t="inlineStr">
         <is>
@@ -3861,6 +4175,7 @@
         <v>5040027</v>
       </c>
     </row>
+    <row r="127"/>
     <row r="128">
       <c r="A128" s="16" t="inlineStr">
         <is>
@@ -3876,19 +4191,35 @@
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>t/month (new plan)</t>
+          <t>BEFORE re-dispatch t/mo</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>December sales share</t>
+          <t>AFTER re-dispatch t/mo</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>Coverage</t>
-        </is>
-      </c>
+          <t>Δ t/mo</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>Change %</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="inlineStr">
+        <is>
+          <t>Dec sales share</t>
+        </is>
+      </c>
+      <c r="G129" s="3" t="inlineStr">
+        <is>
+          <t>Coverage after</t>
+        </is>
+      </c>
+      <c r="H129" s="31" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
@@ -3896,15 +4227,25 @@
           <t>SAP</t>
         </is>
       </c>
-      <c r="B130" s="5" t="n">
+      <c r="B130" s="15" t="n">
         <v>2315483</v>
       </c>
-      <c r="C130" s="5" t="n">
+      <c r="C130" s="32" t="n">
+        <v>2315483</v>
+      </c>
+      <c r="D130" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E130" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F130" s="15" t="n">
         <v>2311213</v>
       </c>
-      <c r="D130" s="7" t="n">
+      <c r="G130" s="34" t="n">
         <v>1.001847514703318</v>
       </c>
+      <c r="H130" s="31" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="14" t="inlineStr">
@@ -3912,15 +4253,25 @@
           <t>LIM-TOS</t>
         </is>
       </c>
-      <c r="B131" s="5" t="n">
+      <c r="B131" s="15" t="n">
         <v>1331853</v>
       </c>
-      <c r="C131" s="5" t="n">
+      <c r="C131" s="32" t="n">
+        <v>1331853</v>
+      </c>
+      <c r="D131" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E131" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F131" s="15" t="n">
         <v>1326082</v>
       </c>
-      <c r="D131" s="7" t="n">
+      <c r="G131" s="34" t="n">
         <v>1.004351917905529</v>
       </c>
+      <c r="H131" s="31" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="14" t="inlineStr">
@@ -3928,35 +4279,87 @@
           <t>LIM-LD</t>
         </is>
       </c>
-      <c r="B132" s="5" t="n">
+      <c r="B132" s="15" t="n">
+        <v>1397883</v>
+      </c>
+      <c r="C132" s="32" t="n">
         <v>1164388</v>
       </c>
-      <c r="C132" s="5" t="n">
+      <c r="D132" s="35" t="n">
+        <v>-233495</v>
+      </c>
+      <c r="E132" s="36" t="n">
+        <v>-0.167034723220756</v>
+      </c>
+      <c r="F132" s="15" t="n">
         <v>992213</v>
       </c>
-      <c r="D132" s="7" t="n">
+      <c r="G132" s="34" t="n">
         <v>1.173526248900186</v>
       </c>
+      <c r="H132" s="31" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="26" t="inlineStr">
+      <c r="A133" s="28" t="inlineStr">
         <is>
           <t>STOCK (kilnable, FeNi KM0)</t>
         </is>
       </c>
-      <c r="B133" s="5" t="n">
+      <c r="B133" s="15" t="n"/>
+      <c r="C133" s="32" t="n">
         <v>228303</v>
       </c>
-      <c r="C133" s="30" t="inlineStr">
+      <c r="D133" s="27" t="n">
+        <v>228303</v>
+      </c>
+      <c r="E133" s="26" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="F133" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D133" s="26" t="inlineStr">
+      <c r="G133" s="37" t="inlineStr">
         <is>
           <t>on top of the met sales lines</t>
         </is>
       </c>
+      <c r="H133" s="31" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="38" t="inlineStr">
+        <is>
+          <t>TOTAL moved</t>
+        </is>
+      </c>
+      <c r="B134" s="32" t="n">
+        <v>5045219</v>
+      </c>
+      <c r="C134" s="32" t="n">
+        <v>5040027</v>
+      </c>
+      <c r="D134" s="35" t="n">
+        <v>-5192</v>
+      </c>
+      <c r="E134" s="36" t="n">
+        <v>-0.001029093087931366</v>
+      </c>
+      <c r="F134" s="31" t="n"/>
+      <c r="G134" s="31" t="n"/>
+      <c r="H134" s="31" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="31" t="n"/>
+      <c r="B135" s="31" t="n"/>
+      <c r="C135" s="31" t="n"/>
+      <c r="D135" s="31" t="n"/>
+      <c r="E135" s="31" t="n"/>
+      <c r="F135" s="31" t="n"/>
+      <c r="G135" s="31" t="n"/>
+      <c r="H135" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
The re-dispatched FeNi KM0 tonnage counts inside the SAP row, not a separate STOCK line
Owner: the kilnable material hauled KR/TF>FENI KM0 IS SAP feed, so the
material table must show old SAP vs new SAP and the percent increase.

Each scenario's table now reads SAP before -> after with the gain inline
(3.0.1: 2,311,732 -> 2,410,852, +4.3%, coverage 104.3%), with a green
sub-row 'of which reallocated to FeNi KM0 stockpile' carrying the split.
Route table rows relabelled 'SAP (stock at FeNi KM0)'. LD unchanged
(-4.4%, still 105.8%), TOS 0%.
</commit_message>
<xml_diff>
--- a/reports/scenario_comparison_dec_options.xlsx
+++ b/reports/scenario_comparison_dec_options.xlsx
@@ -18,11 +18,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="166" formatCode="+0.0%;-0.0%;0%"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -145,6 +146,17 @@
       <color rgb="000F4C81"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="005B6B7F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001B7A41"/>
+      <sz val="8"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -196,7 +208,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -294,6 +306,26 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1101,7 +1133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H135"/>
+  <dimension ref="A1:H136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1644,7 +1676,7 @@
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>STOCK (kilnable, FeNi KM0)</t>
+          <t>SAP (stock at FeNi KM0)</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
@@ -1678,7 +1710,7 @@
       </c>
       <c r="C25" s="20" t="inlineStr">
         <is>
-          <t>STOCK (kilnable, FeNi KM0)</t>
+          <t>SAP (stock at FeNi KM0)</t>
         </is>
       </c>
       <c r="D25" s="20" t="inlineStr">
@@ -1766,7 +1798,7 @@
       <c r="H29" s="31" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="inlineStr">
+      <c r="A30" s="19" t="inlineStr">
         <is>
           <t>SAP</t>
         </is>
@@ -1775,19 +1807,19 @@
         <v>2311732</v>
       </c>
       <c r="C30" s="32" t="n">
-        <v>2311732</v>
+        <v>2410852</v>
       </c>
       <c r="D30" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="33" t="n">
-        <v>0</v>
+        <v>99120</v>
+      </c>
+      <c r="E30" s="39" t="n">
+        <v>0.04287694248295218</v>
       </c>
       <c r="F30" s="15" t="n">
         <v>2311213</v>
       </c>
       <c r="G30" s="34" t="n">
-        <v>1.000224557407734</v>
+        <v>1.043111128225741</v>
       </c>
       <c r="H30" s="31" t="n"/>
     </row>
@@ -1803,10 +1835,10 @@
       <c r="C31" s="32" t="n">
         <v>1001362</v>
       </c>
-      <c r="D31" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="33" t="n">
+      <c r="D31" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="41" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="15" t="n">
@@ -1832,7 +1864,7 @@
       <c r="D32" s="35" t="n">
         <v>-84351</v>
       </c>
-      <c r="E32" s="36" t="n">
+      <c r="E32" s="42" t="n">
         <v>-0.04430946603917992</v>
       </c>
       <c r="F32" s="15" t="n">
@@ -1844,33 +1876,25 @@
       <c r="H32" s="31" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="28" t="inlineStr">
-        <is>
-          <t>STOCK (kilnable, FeNi KM0)</t>
-        </is>
-      </c>
-      <c r="B33" s="15" t="n"/>
-      <c r="C33" s="32" t="n">
+      <c r="A33" s="43" t="inlineStr">
+        <is>
+          <t>of which reallocated to FeNi KM0 stockpile (KR/TF&gt;FENI KM0)</t>
+        </is>
+      </c>
+      <c r="B33" s="44" t="n"/>
+      <c r="C33" s="27" t="n">
         <v>99120</v>
       </c>
       <c r="D33" s="27" t="n">
         <v>99120</v>
       </c>
-      <c r="E33" s="26" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="F33" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G33" s="37" t="inlineStr">
-        <is>
-          <t>on top of the met sales lines</t>
-        </is>
-      </c>
+      <c r="E33" s="45" t="inlineStr">
+        <is>
+          <t>in SAP row</t>
+        </is>
+      </c>
+      <c r="F33" s="30" t="n"/>
+      <c r="G33" s="37" t="n"/>
       <c r="H33" s="31" t="n"/>
     </row>
     <row r="34">
@@ -1888,7 +1912,7 @@
       <c r="D34" s="27" t="n">
         <v>14769</v>
       </c>
-      <c r="E34" s="33" t="n">
+      <c r="E34" s="39" t="n">
         <v>0.002831060504261926</v>
       </c>
       <c r="F34" s="31" t="n"/>
@@ -1906,11 +1930,14 @@
       <c r="H35" s="31" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="inlineStr">
-        <is>
-          <t>Scenario 3.0.2 — December</t>
-        </is>
-      </c>
+      <c r="A36" s="46" t="n"/>
+      <c r="B36" s="31" t="n"/>
+      <c r="C36" s="31" t="n"/>
+      <c r="D36" s="31" t="n"/>
+      <c r="E36" s="31" t="n"/>
+      <c r="F36" s="31" t="n"/>
+      <c r="G36" s="31" t="n"/>
+      <c r="H36" s="31" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr"/>
@@ -2484,7 +2511,7 @@
       </c>
       <c r="C58" s="20" t="inlineStr">
         <is>
-          <t>STOCK (kilnable, FeNi KM0)</t>
+          <t>SAP (stock at FeNi KM0)</t>
         </is>
       </c>
       <c r="D58" s="20" t="inlineStr">
@@ -2518,7 +2545,7 @@
       </c>
       <c r="C59" s="20" t="inlineStr">
         <is>
-          <t>STOCK (kilnable, FeNi KM0)</t>
+          <t>SAP (stock at FeNi KM0)</t>
         </is>
       </c>
       <c r="D59" s="20" t="inlineStr">
@@ -2606,7 +2633,7 @@
       <c r="H63" s="31" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="14" t="inlineStr">
+      <c r="A64" s="19" t="inlineStr">
         <is>
           <t>SAP</t>
         </is>
@@ -2615,19 +2642,19 @@
         <v>2311732</v>
       </c>
       <c r="C64" s="32" t="n">
-        <v>2311732</v>
+        <v>2517274</v>
       </c>
       <c r="D64" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E64" s="33" t="n">
-        <v>0</v>
+        <v>205542</v>
+      </c>
+      <c r="E64" s="39" t="n">
+        <v>0.08891255560765694</v>
       </c>
       <c r="F64" s="15" t="n">
         <v>2311213</v>
       </c>
       <c r="G64" s="34" t="n">
-        <v>1.000224557407734</v>
+        <v>1.089157078988393</v>
       </c>
       <c r="H64" s="31" t="n"/>
     </row>
@@ -2643,10 +2670,10 @@
       <c r="C65" s="32" t="n">
         <v>1000556</v>
       </c>
-      <c r="D65" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E65" s="33" t="n">
+      <c r="D65" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" s="41" t="n">
         <v>0</v>
       </c>
       <c r="F65" s="15" t="n">
@@ -2672,7 +2699,7 @@
       <c r="D66" s="35" t="n">
         <v>-212620</v>
       </c>
-      <c r="E66" s="36" t="n">
+      <c r="E66" s="42" t="n">
         <v>-0.1046603951813492</v>
       </c>
       <c r="F66" s="15" t="n">
@@ -2684,33 +2711,25 @@
       <c r="H66" s="31" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="28" t="inlineStr">
-        <is>
-          <t>STOCK (kilnable, FeNi KM0)</t>
-        </is>
-      </c>
-      <c r="B67" s="15" t="n"/>
-      <c r="C67" s="32" t="n">
+      <c r="A67" s="43" t="inlineStr">
+        <is>
+          <t>of which reallocated to FeNi KM0 stockpile (KR/TF&gt;FENI KM0)</t>
+        </is>
+      </c>
+      <c r="B67" s="44" t="n"/>
+      <c r="C67" s="27" t="n">
         <v>205542</v>
       </c>
       <c r="D67" s="27" t="n">
         <v>205542</v>
       </c>
-      <c r="E67" s="26" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="F67" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G67" s="37" t="inlineStr">
-        <is>
-          <t>on top of the met sales lines</t>
-        </is>
-      </c>
+      <c r="E67" s="45" t="inlineStr">
+        <is>
+          <t>in SAP row</t>
+        </is>
+      </c>
+      <c r="F67" s="30" t="n"/>
+      <c r="G67" s="37" t="n"/>
       <c r="H67" s="31" t="n"/>
     </row>
     <row r="68">
@@ -2728,7 +2747,7 @@
       <c r="D68" s="35" t="n">
         <v>-7078</v>
       </c>
-      <c r="E68" s="36" t="n">
+      <c r="E68" s="42" t="n">
         <v>-0.001324522891995993</v>
       </c>
       <c r="F68" s="31" t="n"/>
@@ -2746,11 +2765,14 @@
       <c r="H69" s="31" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="18" t="inlineStr">
-        <is>
-          <t>Scenario 3.1.1 — December</t>
-        </is>
-      </c>
+      <c r="A70" s="46" t="n"/>
+      <c r="B70" s="31" t="n"/>
+      <c r="C70" s="31" t="n"/>
+      <c r="D70" s="31" t="n"/>
+      <c r="E70" s="31" t="n"/>
+      <c r="F70" s="31" t="n"/>
+      <c r="G70" s="31" t="n"/>
+      <c r="H70" s="31" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr"/>
@@ -3260,7 +3282,7 @@
       </c>
       <c r="C90" s="20" t="inlineStr">
         <is>
-          <t>STOCK (kilnable, FeNi KM0)</t>
+          <t>SAP (stock at FeNi KM0)</t>
         </is>
       </c>
       <c r="D90" s="20" t="inlineStr">
@@ -3294,7 +3316,7 @@
       </c>
       <c r="C91" s="20" t="inlineStr">
         <is>
-          <t>STOCK (kilnable, FeNi KM0)</t>
+          <t>SAP (stock at FeNi KM0)</t>
         </is>
       </c>
       <c r="D91" s="20" t="inlineStr">
@@ -3382,7 +3404,7 @@
       <c r="H95" s="31" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="14" t="inlineStr">
+      <c r="A96" s="19" t="inlineStr">
         <is>
           <t>SAP</t>
         </is>
@@ -3391,19 +3413,19 @@
         <v>2315483</v>
       </c>
       <c r="C96" s="32" t="n">
-        <v>2315483</v>
+        <v>2498250</v>
       </c>
       <c r="D96" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E96" s="33" t="n">
-        <v>0</v>
+        <v>182767</v>
+      </c>
+      <c r="E96" s="39" t="n">
+        <v>0.07893255964306367</v>
       </c>
       <c r="F96" s="15" t="n">
         <v>2311213</v>
       </c>
       <c r="G96" s="34" t="n">
-        <v>1.001847514703318</v>
+        <v>1.080925903410893</v>
       </c>
       <c r="H96" s="31" t="n"/>
     </row>
@@ -3419,10 +3441,10 @@
       <c r="C97" s="32" t="n">
         <v>1332318</v>
       </c>
-      <c r="D97" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E97" s="33" t="n">
+      <c r="D97" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" s="41" t="n">
         <v>0</v>
       </c>
       <c r="F97" s="15" t="n">
@@ -3448,7 +3470,7 @@
       <c r="D98" s="35" t="n">
         <v>-159781</v>
       </c>
-      <c r="E98" s="36" t="n">
+      <c r="E98" s="42" t="n">
         <v>-0.1207163455617868</v>
       </c>
       <c r="F98" s="15" t="n">
@@ -3460,33 +3482,25 @@
       <c r="H98" s="31" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="28" t="inlineStr">
-        <is>
-          <t>STOCK (kilnable, FeNi KM0)</t>
-        </is>
-      </c>
-      <c r="B99" s="15" t="n"/>
-      <c r="C99" s="32" t="n">
+      <c r="A99" s="43" t="inlineStr">
+        <is>
+          <t>of which reallocated to FeNi KM0 stockpile (KR/TF&gt;FENI KM0)</t>
+        </is>
+      </c>
+      <c r="B99" s="44" t="n"/>
+      <c r="C99" s="27" t="n">
         <v>182767</v>
       </c>
       <c r="D99" s="27" t="n">
         <v>182767</v>
       </c>
-      <c r="E99" s="26" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="F99" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G99" s="37" t="inlineStr">
-        <is>
-          <t>on top of the met sales lines</t>
-        </is>
-      </c>
+      <c r="E99" s="45" t="inlineStr">
+        <is>
+          <t>in SAP row</t>
+        </is>
+      </c>
+      <c r="F99" s="30" t="n"/>
+      <c r="G99" s="37" t="n"/>
       <c r="H99" s="31" t="n"/>
     </row>
     <row r="100">
@@ -3504,7 +3518,7 @@
       <c r="D100" s="27" t="n">
         <v>22986</v>
       </c>
-      <c r="E100" s="33" t="n">
+      <c r="E100" s="39" t="n">
         <v>0.004623639821957884</v>
       </c>
       <c r="F100" s="31" t="n"/>
@@ -3522,11 +3536,14 @@
       <c r="H101" s="31" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="18" t="inlineStr">
-        <is>
-          <t>Scenario 3.1.2 — December</t>
-        </is>
-      </c>
+      <c r="A102" s="46" t="n"/>
+      <c r="B102" s="31" t="n"/>
+      <c r="C102" s="31" t="n"/>
+      <c r="D102" s="31" t="n"/>
+      <c r="E102" s="31" t="n"/>
+      <c r="F102" s="31" t="n"/>
+      <c r="G102" s="31" t="n"/>
+      <c r="H102" s="31" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr"/>
@@ -4100,7 +4117,7 @@
       </c>
       <c r="C124" s="20" t="inlineStr">
         <is>
-          <t>STOCK (kilnable, FeNi KM0)</t>
+          <t>SAP (stock at FeNi KM0)</t>
         </is>
       </c>
       <c r="D124" s="20" t="inlineStr">
@@ -4134,7 +4151,7 @@
       </c>
       <c r="C125" s="20" t="inlineStr">
         <is>
-          <t>STOCK (kilnable, FeNi KM0)</t>
+          <t>SAP (stock at FeNi KM0)</t>
         </is>
       </c>
       <c r="D125" s="20" t="inlineStr">
@@ -4222,7 +4239,7 @@
       <c r="H129" s="31" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="14" t="inlineStr">
+      <c r="A130" s="19" t="inlineStr">
         <is>
           <t>SAP</t>
         </is>
@@ -4231,19 +4248,19 @@
         <v>2315483</v>
       </c>
       <c r="C130" s="32" t="n">
-        <v>2315483</v>
+        <v>2543786</v>
       </c>
       <c r="D130" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E130" s="33" t="n">
-        <v>0</v>
+        <v>228303</v>
+      </c>
+      <c r="E130" s="39" t="n">
+        <v>0.09859843497015526</v>
       </c>
       <c r="F130" s="15" t="n">
         <v>2311213</v>
       </c>
       <c r="G130" s="34" t="n">
-        <v>1.001847514703318</v>
+        <v>1.100628111731805</v>
       </c>
       <c r="H130" s="31" t="n"/>
     </row>
@@ -4259,10 +4276,10 @@
       <c r="C131" s="32" t="n">
         <v>1331853</v>
       </c>
-      <c r="D131" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E131" s="33" t="n">
+      <c r="D131" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E131" s="41" t="n">
         <v>0</v>
       </c>
       <c r="F131" s="15" t="n">
@@ -4288,7 +4305,7 @@
       <c r="D132" s="35" t="n">
         <v>-233495</v>
       </c>
-      <c r="E132" s="36" t="n">
+      <c r="E132" s="42" t="n">
         <v>-0.167034723220756</v>
       </c>
       <c r="F132" s="15" t="n">
@@ -4300,33 +4317,25 @@
       <c r="H132" s="31" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="28" t="inlineStr">
-        <is>
-          <t>STOCK (kilnable, FeNi KM0)</t>
-        </is>
-      </c>
-      <c r="B133" s="15" t="n"/>
-      <c r="C133" s="32" t="n">
+      <c r="A133" s="43" t="inlineStr">
+        <is>
+          <t>of which reallocated to FeNi KM0 stockpile (KR/TF&gt;FENI KM0)</t>
+        </is>
+      </c>
+      <c r="B133" s="44" t="n"/>
+      <c r="C133" s="27" t="n">
         <v>228303</v>
       </c>
       <c r="D133" s="27" t="n">
         <v>228303</v>
       </c>
-      <c r="E133" s="26" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="F133" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G133" s="37" t="inlineStr">
-        <is>
-          <t>on top of the met sales lines</t>
-        </is>
-      </c>
+      <c r="E133" s="45" t="inlineStr">
+        <is>
+          <t>in SAP row</t>
+        </is>
+      </c>
+      <c r="F133" s="30" t="n"/>
+      <c r="G133" s="37" t="n"/>
       <c r="H133" s="31" t="n"/>
     </row>
     <row r="134">
@@ -4344,7 +4353,7 @@
       <c r="D134" s="35" t="n">
         <v>-5192</v>
       </c>
-      <c r="E134" s="36" t="n">
+      <c r="E134" s="42" t="n">
         <v>-0.001029093087931366</v>
       </c>
       <c r="F134" s="31" t="n"/>
@@ -4361,13 +4370,27 @@
       <c r="G135" s="31" t="n"/>
       <c r="H135" s="31" t="n"/>
     </row>
+    <row r="136">
+      <c r="A136" s="31" t="n"/>
+      <c r="B136" s="31" t="n"/>
+      <c r="C136" s="31" t="n"/>
+      <c r="D136" s="31" t="n"/>
+      <c r="E136" s="31" t="n"/>
+      <c r="F136" s="31" t="n"/>
+      <c r="G136" s="31" t="n"/>
+      <c r="H136" s="31" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="9">
     <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A33:B33"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A107:H107"/>
+    <mergeCell ref="A99:B99"/>
+    <mergeCell ref="A133:B133"/>
     <mergeCell ref="A41:H41"/>
     <mergeCell ref="A75:H75"/>
+    <mergeCell ref="A67:B67"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Comparison workbook refreshed from the audited, refrozen December saves (exact 50/50 POS 6)
</commit_message>
<xml_diff>
--- a/reports/scenario_comparison_dec_options.xlsx
+++ b/reports/scenario_comparison_dec_options.xlsx
@@ -2015,300 +2015,218 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:H137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="38" t="inlineStr">
         <is>
-          <t>December — the full 1,281-DT pool works (frozen 2026-08-27)</t>
+          <t>December runs over target in every scenario — two ways to spend the surplus</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="39" t="inlineStr">
         <is>
-          <t>Owner's rule: SAP 100%, LIM-TOS 100%, and EVERY remaining truck hauls LIM-LD — the target is a goal, not a ceiling. The previously idle trucks (91 SMA in 3.0.x, 74 RIM + 155 SMA in 3.1.x) now ride the TF&gt;HUAFEI LD rows. This is the frozen plan, not an option.</t>
+          <t>Option 1: park the surplus DT (total month lands at 100.0%). Option 2: cut LIM-LD to exactly its December line and re-dispatch every freed DT to KR&gt;FENI KM0 + TF&gt;FENI KM0 — the hauled material is kilnable SAP feed stocked at the plant.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="40" t="inlineStr">
         <is>
-          <t>Scenario 3.0.1 — December (frozen, 1,281 DT)</t>
+          <t>Scenario 3.0.1 — December</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="41" t="inlineStr">
+      <c r="A5" s="41" t="inlineStr"/>
+      <c r="B5" s="41" t="inlineStr">
+        <is>
+          <t>Target t</t>
+        </is>
+      </c>
+      <c r="C5" s="41" t="inlineStr">
+        <is>
+          <t>Predicted t</t>
+        </is>
+      </c>
+      <c r="D5" s="41" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="E5" s="41" t="inlineStr">
+        <is>
+          <t>Fleet DT</t>
+        </is>
+      </c>
+      <c r="F5" s="41" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="42" t="inlineStr">
+        <is>
+          <t>As frozen</t>
+        </is>
+      </c>
+      <c r="B6" s="43" t="n">
+        <v>5131386</v>
+      </c>
+      <c r="C6" s="43" t="n">
+        <v>5216721</v>
+      </c>
+      <c r="D6" s="44" t="n">
+        <v>1.016630009903757</v>
+      </c>
+      <c r="E6" s="43" t="n">
+        <v>1190</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="42" t="inlineStr">
+        <is>
+          <t>OPTION 1 · park 26 DT (total month → 100.0%)</t>
+        </is>
+      </c>
+      <c r="B7" s="43" t="n">
+        <v>5131386</v>
+      </c>
+      <c r="C7" s="43" t="n">
+        <v>5132370</v>
+      </c>
+      <c r="D7" s="45" t="n">
+        <v>1.00019176105637</v>
+      </c>
+      <c r="E7" s="43" t="n">
+        <v>1164</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="42" t="inlineStr">
+        <is>
+          <t>OPTION 2 · re-dispatch 56 DT (LIM-LD → 100.0%)</t>
+        </is>
+      </c>
+      <c r="B8" s="43" t="n">
+        <v>5131386</v>
+      </c>
+      <c r="C8" s="43" t="n">
+        <v>5248586</v>
+      </c>
+      <c r="D8" s="46" t="n">
+        <v>1.0228398331367</v>
+      </c>
+      <c r="E8" s="43" t="n">
+        <v>1190</v>
+      </c>
+      <c r="F8" s="48" t="inlineStr">
+        <is>
+          <t>+ 213,461 t SAP stocked at FeNi KM0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="49" t="inlineStr">
+        <is>
+          <t>Option 2 cut (sized so LIM-LD lands exactly on its line): TF&gt;HUAFEI (RIM, LD): −56 DT @ 104.7 t/day/DT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="50" t="inlineStr">
+        <is>
+          <t>OPTION 2 — full December plan (re-dispatched)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="41" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="B5" s="41" t="inlineStr">
+      <c r="B12" s="41" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="C5" s="41" t="inlineStr">
+      <c r="C12" s="41" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="D5" s="41" t="inlineStr">
-        <is>
-          <t>DT</t>
-        </is>
-      </c>
-      <c r="E5" s="41" t="inlineStr">
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>DT before</t>
+        </is>
+      </c>
+      <c r="E12" s="41" t="inlineStr">
+        <is>
+          <t>DT after</t>
+        </is>
+      </c>
+      <c r="F12" s="41" t="inlineStr">
+        <is>
+          <t>Δ DT</t>
+        </is>
+      </c>
+      <c r="G12" s="41" t="inlineStr">
         <is>
           <t>t/day</t>
         </is>
       </c>
-      <c r="F5" s="41" t="inlineStr">
+      <c r="H12" s="41" t="inlineStr">
         <is>
           <t>t/month</t>
         </is>
       </c>
-      <c r="G5" s="41" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="67" t="inlineStr">
-        <is>
-          <t>TF&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B6" s="67" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C6" s="67" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="D6" s="68" t="n">
-        <v>436</v>
-      </c>
-      <c r="E6" s="43" t="n">
-        <v>45474</v>
-      </c>
-      <c r="F6" s="43" t="n">
-        <v>1409694</v>
-      </c>
-      <c r="G6" s="69" t="inlineStr">
-        <is>
-          <t>includes activated idle DT</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="67" t="inlineStr">
-        <is>
-          <t>TF&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B7" s="67" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C7" s="67" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="D7" s="68" t="n">
-        <v>240</v>
-      </c>
-      <c r="E7" s="43" t="n">
-        <v>24987</v>
-      </c>
-      <c r="F7" s="43" t="n">
-        <v>774597</v>
-      </c>
-      <c r="G7" s="69" t="inlineStr">
-        <is>
-          <t>includes activated idle DT</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="51" t="inlineStr">
-        <is>
-          <t>BLB&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B8" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C8" s="51" t="inlineStr">
-        <is>
-          <t>LIM-TOS</t>
-        </is>
-      </c>
-      <c r="D8" s="43" t="n">
-        <v>95</v>
-      </c>
-      <c r="E8" s="43" t="n">
-        <v>23244</v>
-      </c>
-      <c r="F8" s="43" t="n">
-        <v>720564</v>
-      </c>
-      <c r="G8" s="66" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B9" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C9" s="51" t="inlineStr">
-        <is>
-          <t>LIM-TOS</t>
-        </is>
-      </c>
-      <c r="D9" s="43" t="n">
-        <v>62</v>
-      </c>
-      <c r="E9" s="43" t="n">
-        <v>6467</v>
-      </c>
-      <c r="F9" s="43" t="n">
-        <v>200477</v>
-      </c>
-      <c r="G9" s="66" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="51" t="inlineStr">
-        <is>
-          <t>KR&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B10" s="51" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C10" s="51" t="inlineStr">
-        <is>
-          <t>LIM-TOS</t>
-        </is>
-      </c>
-      <c r="D10" s="43" t="n">
-        <v>19</v>
-      </c>
-      <c r="E10" s="43" t="n">
-        <v>2540</v>
-      </c>
-      <c r="F10" s="43" t="n">
-        <v>78740</v>
-      </c>
-      <c r="G10" s="66" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="51" t="inlineStr">
-        <is>
-          <t>BLB&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="B11" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C11" s="51" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="D11" s="43" t="n">
-        <v>202</v>
-      </c>
-      <c r="E11" s="43" t="n">
-        <v>45774</v>
-      </c>
-      <c r="F11" s="43" t="n">
-        <v>1418994</v>
-      </c>
-      <c r="G11" s="66" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="B12" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C12" s="51" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="D12" s="43" t="n">
-        <v>141</v>
-      </c>
-      <c r="E12" s="43" t="n">
-        <v>14776</v>
-      </c>
-      <c r="F12" s="43" t="n">
-        <v>458056</v>
-      </c>
-      <c r="G12" s="66" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="51" t="inlineStr">
         <is>
-          <t>KR&gt;FENI KM15</t>
+          <t>TF&gt;HUAFEI</t>
         </is>
       </c>
       <c r="B13" s="51" t="inlineStr">
         <is>
-          <t>SMA</t>
+          <t>RIM</t>
         </is>
       </c>
       <c r="C13" s="51" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>LIM-LD</t>
         </is>
       </c>
       <c r="D13" s="43" t="n">
-        <v>50</v>
-      </c>
-      <c r="E13" s="43" t="n">
-        <v>7885</v>
-      </c>
-      <c r="F13" s="43" t="n">
-        <v>244435</v>
-      </c>
-      <c r="G13" s="66" t="n"/>
+        <v>437</v>
+      </c>
+      <c r="E13" s="47" t="n">
+        <v>381</v>
+      </c>
+      <c r="F13" s="52" t="n">
+        <v>-56</v>
+      </c>
+      <c r="G13" s="43" t="n">
+        <v>39874</v>
+      </c>
+      <c r="H13" s="43" t="n">
+        <v>1236106</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="51" t="inlineStr">
         <is>
-          <t>KR&gt;POS 12</t>
+          <t>TF&gt;HUAFEI</t>
         </is>
       </c>
       <c r="B14" s="51" t="inlineStr">
@@ -2318,24 +2236,29 @@
       </c>
       <c r="C14" s="51" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>LIM-LD</t>
         </is>
       </c>
       <c r="D14" s="43" t="n">
-        <v>11</v>
+        <v>150</v>
       </c>
       <c r="E14" s="43" t="n">
-        <v>2187</v>
-      </c>
-      <c r="F14" s="43" t="n">
-        <v>67797</v>
-      </c>
-      <c r="G14" s="66" t="n"/>
+        <v>150</v>
+      </c>
+      <c r="F14" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="43" t="n">
+        <v>15675</v>
+      </c>
+      <c r="H14" s="43" t="n">
+        <v>485925</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="51" t="inlineStr">
         <is>
-          <t>BLB&gt;POS 14</t>
+          <t>BLB&gt;HUAFEI</t>
         </is>
       </c>
       <c r="B15" s="51" t="inlineStr">
@@ -2345,24 +2268,29 @@
       </c>
       <c r="C15" s="51" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>LIM-TOS</t>
         </is>
       </c>
       <c r="D15" s="43" t="n">
-        <v>7</v>
+        <v>95</v>
       </c>
       <c r="E15" s="43" t="n">
-        <v>2043</v>
-      </c>
-      <c r="F15" s="43" t="n">
-        <v>63333</v>
-      </c>
-      <c r="G15" s="66" t="n"/>
+        <v>95</v>
+      </c>
+      <c r="F15" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="43" t="n">
+        <v>23250</v>
+      </c>
+      <c r="H15" s="43" t="n">
+        <v>720750</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="51" t="inlineStr">
         <is>
-          <t>TF&gt;POS 12</t>
+          <t>TF&gt;HUAFEI</t>
         </is>
       </c>
       <c r="B16" s="51" t="inlineStr">
@@ -2372,712 +2300,840 @@
       </c>
       <c r="C16" s="51" t="inlineStr">
         <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="D16" s="43" t="n">
+        <v>62</v>
+      </c>
+      <c r="E16" s="43" t="n">
+        <v>62</v>
+      </c>
+      <c r="F16" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="43" t="n">
+        <v>6489</v>
+      </c>
+      <c r="H16" s="43" t="n">
+        <v>201159</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="51" t="inlineStr">
+        <is>
+          <t>KR&gt;HUAFEI</t>
+        </is>
+      </c>
+      <c r="B17" s="51" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="C17" s="51" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="D17" s="43" t="n">
+        <v>19</v>
+      </c>
+      <c r="E17" s="43" t="n">
+        <v>19</v>
+      </c>
+      <c r="F17" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="43" t="n">
+        <v>2563</v>
+      </c>
+      <c r="H17" s="43" t="n">
+        <v>79453</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="51" t="inlineStr">
+        <is>
+          <t>BLB&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="B18" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C18" s="51" t="inlineStr">
+        <is>
           <t>SAP</t>
         </is>
       </c>
-      <c r="D16" s="43" t="n">
-        <v>18</v>
-      </c>
-      <c r="E16" s="43" t="n">
-        <v>2036</v>
-      </c>
-      <c r="F16" s="43" t="n">
-        <v>63116</v>
-      </c>
-      <c r="G16" s="66" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="60" t="inlineStr">
-        <is>
-          <t>TOTAL (full matrix pool)</t>
-        </is>
-      </c>
-      <c r="D17" s="47" t="n">
-        <v>1281</v>
-      </c>
-      <c r="F17" s="47" t="n">
-        <v>5499803</v>
+      <c r="D18" s="43" t="n">
+        <v>202</v>
+      </c>
+      <c r="E18" s="43" t="n">
+        <v>202</v>
+      </c>
+      <c r="F18" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="43" t="n">
+        <v>45786</v>
+      </c>
+      <c r="H18" s="43" t="n">
+        <v>1419366</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="41" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B19" s="41" t="inlineStr">
-        <is>
-          <t>t/month (frozen)</t>
-        </is>
-      </c>
-      <c r="C19" s="41" t="inlineStr">
-        <is>
-          <t>December TARGET t</t>
-        </is>
-      </c>
-      <c r="D19" s="41" t="inlineStr">
-        <is>
-          <t>Coverage</t>
-        </is>
-      </c>
-      <c r="E19" s="41" t="inlineStr"/>
-      <c r="F19" s="41" t="inlineStr"/>
-      <c r="G19" s="41" t="inlineStr"/>
+      <c r="A19" s="51" t="inlineStr">
+        <is>
+          <t>TF&gt;FENI KM15</t>
+        </is>
+      </c>
+      <c r="B19" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C19" s="51" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D19" s="43" t="n">
+        <v>140</v>
+      </c>
+      <c r="E19" s="43" t="n">
+        <v>140</v>
+      </c>
+      <c r="F19" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="43" t="n">
+        <v>14736</v>
+      </c>
+      <c r="H19" s="43" t="n">
+        <v>456816</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="51" t="inlineStr">
         <is>
+          <t>KR&gt;FENI KM15</t>
+        </is>
+      </c>
+      <c r="B20" s="51" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="C20" s="51" t="inlineStr">
+        <is>
           <t>SAP</t>
         </is>
       </c>
-      <c r="B20" s="47" t="n">
-        <v>2315731</v>
-      </c>
-      <c r="C20" s="43" t="n">
-        <v>2311213</v>
-      </c>
-      <c r="D20" s="45" t="n">
-        <v>1.00195481766501</v>
+      <c r="D20" s="43" t="n">
+        <v>50</v>
+      </c>
+      <c r="E20" s="43" t="n">
+        <v>50</v>
+      </c>
+      <c r="F20" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="43" t="n">
+        <v>7958</v>
+      </c>
+      <c r="H20" s="43" t="n">
+        <v>246698</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="51" t="inlineStr">
         <is>
-          <t>LIM-TOS</t>
-        </is>
-      </c>
-      <c r="B21" s="47" t="n">
-        <v>999781</v>
-      </c>
-      <c r="C21" s="43" t="n">
-        <v>996084</v>
-      </c>
-      <c r="D21" s="45" t="n">
-        <v>1.003711534368587</v>
+          <t>BLB&gt;POS 14</t>
+        </is>
+      </c>
+      <c r="B21" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C21" s="51" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D21" s="43" t="n">
+        <v>7</v>
+      </c>
+      <c r="E21" s="43" t="n">
+        <v>7</v>
+      </c>
+      <c r="F21" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="43" t="n">
+        <v>2044</v>
+      </c>
+      <c r="H21" s="43" t="n">
+        <v>63364</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="51" t="inlineStr">
         <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="B22" s="47" t="n">
-        <v>2184291</v>
-      </c>
-      <c r="C22" s="43" t="n">
-        <v>1719964</v>
-      </c>
-      <c r="D22" s="45" t="n">
-        <v>1.269963208532272</v>
-      </c>
-      <c r="E22" s="70" t="inlineStr">
-        <is>
-          <t>above target by design — surplus fleet hauls LD</t>
-        </is>
+          <t>TF&gt;POS 12</t>
+        </is>
+      </c>
+      <c r="B22" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C22" s="51" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D22" s="43" t="n">
+        <v>18</v>
+      </c>
+      <c r="E22" s="43" t="n">
+        <v>18</v>
+      </c>
+      <c r="F22" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="43" t="n">
+        <v>2039</v>
+      </c>
+      <c r="H22" s="43" t="n">
+        <v>63209</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="51" t="inlineStr">
+        <is>
+          <t>KR&gt;POS 12</t>
+        </is>
+      </c>
+      <c r="B23" s="51" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="C23" s="51" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D23" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="E23" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="F23" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="43" t="n">
+        <v>2009</v>
+      </c>
+      <c r="H23" s="43" t="n">
+        <v>62279</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="54" t="inlineStr">
+        <is>
+          <t>KR&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="B24" s="54" t="inlineStr">
+        <is>
+          <t>reallocated</t>
+        </is>
+      </c>
+      <c r="C24" s="54" t="inlineStr">
+        <is>
+          <t>SAP (stock at FeNi KM0)</t>
+        </is>
+      </c>
+      <c r="D24" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="56" t="n">
+        <v>28</v>
+      </c>
+      <c r="F24" s="56" t="n">
+        <v>28</v>
+      </c>
+      <c r="G24" s="56" t="n">
+        <v>3802</v>
+      </c>
+      <c r="H24" s="56" t="n">
+        <v>117848</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="40" t="inlineStr">
-        <is>
-          <t>Scenario 3.0.2 — December (frozen, 1,281 DT)</t>
-        </is>
+      <c r="A25" s="54" t="inlineStr">
+        <is>
+          <t>TF&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="B25" s="54" t="inlineStr">
+        <is>
+          <t>reallocated</t>
+        </is>
+      </c>
+      <c r="C25" s="54" t="inlineStr">
+        <is>
+          <t>SAP (stock at FeNi KM0)</t>
+        </is>
+      </c>
+      <c r="D25" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="56" t="n">
+        <v>28</v>
+      </c>
+      <c r="F25" s="56" t="n">
+        <v>28</v>
+      </c>
+      <c r="G25" s="56" t="n">
+        <v>3084</v>
+      </c>
+      <c r="H25" s="56" t="n">
+        <v>95614</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="41" t="inlineStr">
-        <is>
-          <t>Route</t>
-        </is>
-      </c>
-      <c r="B26" s="41" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="C26" s="41" t="inlineStr">
+      <c r="A26" s="60" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D26" s="47" t="n">
+        <v>1190</v>
+      </c>
+      <c r="E26" s="47" t="n">
+        <v>1190</v>
+      </c>
+      <c r="H26" s="47" t="n">
+        <v>5248587</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="50" t="inlineStr">
+        <is>
+          <t>OPTION 2 — tonnage by material (December)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="41" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="D26" s="41" t="inlineStr">
-        <is>
-          <t>DT</t>
-        </is>
-      </c>
-      <c r="E26" s="41" t="inlineStr">
-        <is>
-          <t>t/day</t>
-        </is>
-      </c>
-      <c r="F26" s="41" t="inlineStr">
-        <is>
-          <t>t/month</t>
-        </is>
-      </c>
-      <c r="G26" s="41" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="67" t="inlineStr">
-        <is>
-          <t>TF&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B27" s="67" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C27" s="67" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="D27" s="68" t="n">
-        <v>285</v>
-      </c>
-      <c r="E27" s="43" t="n">
-        <v>29654</v>
-      </c>
-      <c r="F27" s="43" t="n">
-        <v>919274</v>
-      </c>
-      <c r="G27" s="69" t="inlineStr">
-        <is>
-          <t>includes activated idle DT</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;POS 6</t>
-        </is>
-      </c>
-      <c r="B28" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C28" s="51" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="D28" s="43" t="n">
-        <v>150</v>
-      </c>
-      <c r="E28" s="43" t="n">
-        <v>18989</v>
-      </c>
-      <c r="F28" s="43" t="n">
-        <v>588659</v>
-      </c>
-      <c r="G28" s="66" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;POS 6</t>
-        </is>
-      </c>
-      <c r="B29" s="51" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C29" s="51" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="D29" s="43" t="n">
-        <v>120</v>
-      </c>
-      <c r="E29" s="43" t="n">
-        <v>13876</v>
-      </c>
-      <c r="F29" s="43" t="n">
-        <v>430156</v>
-      </c>
-      <c r="G29" s="66" t="n"/>
+      <c r="B29" s="41" t="inlineStr">
+        <is>
+          <t>BEFORE re-dispatch t/mo</t>
+        </is>
+      </c>
+      <c r="C29" s="41" t="inlineStr">
+        <is>
+          <t>AFTER re-dispatch t/mo</t>
+        </is>
+      </c>
+      <c r="D29" s="41" t="inlineStr">
+        <is>
+          <t>Δ t/mo</t>
+        </is>
+      </c>
+      <c r="E29" s="41" t="inlineStr">
+        <is>
+          <t>Change %</t>
+        </is>
+      </c>
+      <c r="F29" s="41" t="inlineStr">
+        <is>
+          <t>December TARGET t</t>
+        </is>
+      </c>
+      <c r="G29" s="41" t="inlineStr">
+        <is>
+          <t>Coverage after</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="67" t="inlineStr">
-        <is>
-          <t>TF&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B30" s="67" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C30" s="67" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="D30" s="68" t="n">
-        <v>120</v>
-      </c>
-      <c r="E30" s="43" t="n">
-        <v>12461</v>
+      <c r="A30" s="42" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="B30" s="43" t="n">
+        <v>2311732</v>
+      </c>
+      <c r="C30" s="47" t="n">
+        <v>2525193</v>
+      </c>
+      <c r="D30" s="61" t="n">
+        <v>213461</v>
+      </c>
+      <c r="E30" s="62" t="n">
+        <v>0.09233812569969184</v>
       </c>
       <c r="F30" s="43" t="n">
-        <v>386291</v>
-      </c>
-      <c r="G30" s="69" t="inlineStr">
-        <is>
-          <t>includes activated idle DT</t>
-        </is>
+        <v>2311213</v>
+      </c>
+      <c r="G30" s="45" t="n">
+        <v>1.092583418317567</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="51" t="inlineStr">
         <is>
-          <t>BLB&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B31" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C31" s="51" t="inlineStr">
-        <is>
           <t>LIM-TOS</t>
         </is>
       </c>
-      <c r="D31" s="43" t="n">
-        <v>95</v>
-      </c>
-      <c r="E31" s="43" t="n">
-        <v>23244</v>
+      <c r="B31" s="43" t="n">
+        <v>1001362</v>
+      </c>
+      <c r="C31" s="47" t="n">
+        <v>1001362</v>
+      </c>
+      <c r="D31" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="63" t="n">
+        <v>0</v>
       </c>
       <c r="F31" s="43" t="n">
-        <v>720564</v>
-      </c>
-      <c r="G31" s="66" t="n"/>
+        <v>996084</v>
+      </c>
+      <c r="G31" s="45" t="n">
+        <v>1.005298749904626</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="51" t="inlineStr">
         <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="B32" s="43" t="n">
+        <v>1903716</v>
+      </c>
+      <c r="C32" s="47" t="n">
+        <v>1722031</v>
+      </c>
+      <c r="D32" s="52" t="n">
+        <v>-181685</v>
+      </c>
+      <c r="E32" s="64" t="n">
+        <v>-0.09543702947288356</v>
+      </c>
+      <c r="F32" s="43" t="n">
+        <v>1719964</v>
+      </c>
+      <c r="G32" s="45" t="n">
+        <v>1.001201769339358</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="65" t="inlineStr">
+        <is>
+          <t>of which SAP stocked at FeNi KM0 (KR 28 DT + TF 28 DT reallocated)</t>
+        </is>
+      </c>
+      <c r="B33" s="66" t="n"/>
+      <c r="C33" s="61" t="n">
+        <v>213461</v>
+      </c>
+      <c r="D33" s="61" t="n">
+        <v>213461</v>
+      </c>
+      <c r="E33" s="70" t="inlineStr">
+        <is>
+          <t>inside the SAP row</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="60" t="inlineStr">
+        <is>
+          <t>TOTAL moved</t>
+        </is>
+      </c>
+      <c r="B34" s="47" t="n">
+        <v>5216810</v>
+      </c>
+      <c r="C34" s="47" t="n">
+        <v>5248586</v>
+      </c>
+      <c r="D34" s="61" t="n">
+        <v>31776</v>
+      </c>
+      <c r="E34" s="62" t="n">
+        <v>0.006091078647679329</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="40" t="inlineStr">
+        <is>
+          <t>Scenario 3.0.2 — December</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="41" t="inlineStr"/>
+      <c r="B38" s="41" t="inlineStr">
+        <is>
+          <t>Target t</t>
+        </is>
+      </c>
+      <c r="C38" s="41" t="inlineStr">
+        <is>
+          <t>Predicted t</t>
+        </is>
+      </c>
+      <c r="D38" s="41" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="E38" s="41" t="inlineStr">
+        <is>
+          <t>Fleet DT</t>
+        </is>
+      </c>
+      <c r="F38" s="41" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="42" t="inlineStr">
+        <is>
+          <t>As frozen</t>
+        </is>
+      </c>
+      <c r="B39" s="43" t="n">
+        <v>5131386</v>
+      </c>
+      <c r="C39" s="43" t="n">
+        <v>5343787</v>
+      </c>
+      <c r="D39" s="44" t="n">
+        <v>1.041392520461333</v>
+      </c>
+      <c r="E39" s="43" t="n">
+        <v>1190</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="42" t="inlineStr">
+        <is>
+          <t>OPTION 1 · park 54 DT (total month → 100.0%)</t>
+        </is>
+      </c>
+      <c r="B40" s="43" t="n">
+        <v>5131386</v>
+      </c>
+      <c r="C40" s="43" t="n">
+        <v>5131167</v>
+      </c>
+      <c r="D40" s="45" t="n">
+        <v>0.9999573214722104</v>
+      </c>
+      <c r="E40" s="43" t="n">
+        <v>1136</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="42" t="inlineStr">
+        <is>
+          <t>OPTION 2 · re-dispatch 79 DT (LIM-LD → 100.0%)</t>
+        </is>
+      </c>
+      <c r="B41" s="43" t="n">
+        <v>5131386</v>
+      </c>
+      <c r="C41" s="43" t="n">
+        <v>5333821</v>
+      </c>
+      <c r="D41" s="46" t="n">
+        <v>1.039450355128225</v>
+      </c>
+      <c r="E41" s="43" t="n">
+        <v>1190</v>
+      </c>
+      <c r="F41" s="48" t="inlineStr">
+        <is>
+          <t>+ 301,080 t SAP stocked at FeNi KM0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="49" t="inlineStr">
+        <is>
+          <t>Option 2 cut (sized so LIM-LD lands exactly on its line): TF&gt;POS 6 (RIM, LD): −79 DT @ 127.0 t/day/DT</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="50" t="inlineStr">
+        <is>
+          <t>OPTION 2 — full December plan (re-dispatched)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="41" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B45" s="41" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="C45" s="41" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="D45" s="41" t="inlineStr">
+        <is>
+          <t>DT before</t>
+        </is>
+      </c>
+      <c r="E45" s="41" t="inlineStr">
+        <is>
+          <t>DT after</t>
+        </is>
+      </c>
+      <c r="F45" s="41" t="inlineStr">
+        <is>
+          <t>Δ DT</t>
+        </is>
+      </c>
+      <c r="G45" s="41" t="inlineStr">
+        <is>
+          <t>t/day</t>
+        </is>
+      </c>
+      <c r="H45" s="41" t="inlineStr">
+        <is>
+          <t>t/month</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="51" t="inlineStr">
+        <is>
           <t>TF&gt;HUAFEI</t>
         </is>
       </c>
-      <c r="B32" s="51" t="inlineStr">
+      <c r="B46" s="51" t="inlineStr">
         <is>
           <t>RIM</t>
         </is>
       </c>
-      <c r="C32" s="51" t="inlineStr">
+      <c r="C46" s="51" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="D46" s="43" t="n">
+        <v>288</v>
+      </c>
+      <c r="E46" s="43" t="n">
+        <v>288</v>
+      </c>
+      <c r="F46" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="43" t="n">
+        <v>30085</v>
+      </c>
+      <c r="H46" s="43" t="n">
+        <v>932635</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="51" t="inlineStr">
+        <is>
+          <t>TF&gt;POS 6</t>
+        </is>
+      </c>
+      <c r="B47" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C47" s="51" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="D47" s="43" t="n">
+        <v>149</v>
+      </c>
+      <c r="E47" s="47" t="n">
+        <v>70</v>
+      </c>
+      <c r="F47" s="52" t="n">
+        <v>-79</v>
+      </c>
+      <c r="G47" s="43" t="n">
+        <v>8890</v>
+      </c>
+      <c r="H47" s="43" t="n">
+        <v>275605</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="51" t="inlineStr">
+        <is>
+          <t>TF&gt;POS 6</t>
+        </is>
+      </c>
+      <c r="B48" s="51" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="C48" s="51" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="D48" s="43" t="n">
+        <v>75</v>
+      </c>
+      <c r="E48" s="43" t="n">
+        <v>75</v>
+      </c>
+      <c r="F48" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="43" t="n">
+        <v>8701</v>
+      </c>
+      <c r="H48" s="43" t="n">
+        <v>269731</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="51" t="inlineStr">
+        <is>
+          <t>TF&gt;HUAFEI</t>
+        </is>
+      </c>
+      <c r="B49" s="51" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="C49" s="51" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="D49" s="43" t="n">
+        <v>75</v>
+      </c>
+      <c r="E49" s="43" t="n">
+        <v>75</v>
+      </c>
+      <c r="F49" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="43" t="n">
+        <v>7822</v>
+      </c>
+      <c r="H49" s="43" t="n">
+        <v>242482</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="51" t="inlineStr">
+        <is>
+          <t>BLB&gt;HUAFEI</t>
+        </is>
+      </c>
+      <c r="B50" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C50" s="51" t="inlineStr">
         <is>
           <t>LIM-TOS</t>
         </is>
       </c>
-      <c r="D32" s="43" t="n">
-        <v>63</v>
-      </c>
-      <c r="E32" s="43" t="n">
-        <v>6555</v>
-      </c>
-      <c r="F32" s="43" t="n">
-        <v>203205</v>
-      </c>
-      <c r="G32" s="66" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="51" t="inlineStr">
-        <is>
-          <t>KR&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B33" s="51" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C33" s="51" t="inlineStr">
+      <c r="D50" s="43" t="n">
+        <v>95</v>
+      </c>
+      <c r="E50" s="43" t="n">
+        <v>95</v>
+      </c>
+      <c r="F50" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="43" t="n">
+        <v>23250</v>
+      </c>
+      <c r="H50" s="43" t="n">
+        <v>720750</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="51" t="inlineStr">
+        <is>
+          <t>TF&gt;HUAFEI</t>
+        </is>
+      </c>
+      <c r="B51" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C51" s="51" t="inlineStr">
         <is>
           <t>LIM-TOS</t>
         </is>
       </c>
-      <c r="D33" s="43" t="n">
-        <v>19</v>
-      </c>
-      <c r="E33" s="43" t="n">
-        <v>2522</v>
-      </c>
-      <c r="F33" s="43" t="n">
-        <v>78182</v>
-      </c>
-      <c r="G33" s="66" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="51" t="inlineStr">
-        <is>
-          <t>BLB&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="B34" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C34" s="51" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="D34" s="43" t="n">
-        <v>202</v>
-      </c>
-      <c r="E34" s="43" t="n">
-        <v>45774</v>
-      </c>
-      <c r="F34" s="43" t="n">
-        <v>1418994</v>
-      </c>
-      <c r="G34" s="66" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="B35" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C35" s="51" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="D35" s="43" t="n">
-        <v>141</v>
-      </c>
-      <c r="E35" s="43" t="n">
-        <v>14776</v>
-      </c>
-      <c r="F35" s="43" t="n">
-        <v>458056</v>
-      </c>
-      <c r="G35" s="66" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="51" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="B36" s="51" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C36" s="51" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="D36" s="43" t="n">
-        <v>50</v>
-      </c>
-      <c r="E36" s="43" t="n">
-        <v>7885</v>
-      </c>
-      <c r="F36" s="43" t="n">
-        <v>244435</v>
-      </c>
-      <c r="G36" s="66" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="51" t="inlineStr">
-        <is>
-          <t>KR&gt;POS 12</t>
-        </is>
-      </c>
-      <c r="B37" s="51" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C37" s="51" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="D37" s="43" t="n">
-        <v>11</v>
-      </c>
-      <c r="E37" s="43" t="n">
-        <v>2187</v>
-      </c>
-      <c r="F37" s="43" t="n">
-        <v>67797</v>
-      </c>
-      <c r="G37" s="66" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="51" t="inlineStr">
-        <is>
-          <t>BLB&gt;POS 14</t>
-        </is>
-      </c>
-      <c r="B38" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C38" s="51" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="D38" s="43" t="n">
-        <v>7</v>
-      </c>
-      <c r="E38" s="43" t="n">
-        <v>2043</v>
-      </c>
-      <c r="F38" s="43" t="n">
-        <v>63333</v>
-      </c>
-      <c r="G38" s="66" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;POS 12</t>
-        </is>
-      </c>
-      <c r="B39" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C39" s="51" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="D39" s="43" t="n">
-        <v>18</v>
-      </c>
-      <c r="E39" s="43" t="n">
-        <v>2036</v>
-      </c>
-      <c r="F39" s="43" t="n">
-        <v>63116</v>
-      </c>
-      <c r="G39" s="66" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="60" t="inlineStr">
-        <is>
-          <t>TOTAL (full matrix pool)</t>
-        </is>
-      </c>
-      <c r="D40" s="47" t="n">
-        <v>1281</v>
-      </c>
-      <c r="F40" s="47" t="n">
-        <v>5642062</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="41" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B42" s="41" t="inlineStr">
-        <is>
-          <t>t/month (frozen)</t>
-        </is>
-      </c>
-      <c r="C42" s="41" t="inlineStr">
-        <is>
-          <t>December TARGET t</t>
-        </is>
-      </c>
-      <c r="D42" s="41" t="inlineStr">
-        <is>
-          <t>Coverage</t>
-        </is>
-      </c>
-      <c r="E42" s="41" t="inlineStr"/>
-      <c r="F42" s="41" t="inlineStr"/>
-      <c r="G42" s="41" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="51" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="B43" s="47" t="n">
-        <v>2315731</v>
-      </c>
-      <c r="C43" s="43" t="n">
-        <v>2311213</v>
-      </c>
-      <c r="D43" s="45" t="n">
-        <v>1.00195481766501</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="51" t="inlineStr">
-        <is>
-          <t>LIM-TOS</t>
-        </is>
-      </c>
-      <c r="B44" s="47" t="n">
-        <v>1001951</v>
-      </c>
-      <c r="C44" s="43" t="n">
-        <v>996084</v>
-      </c>
-      <c r="D44" s="45" t="n">
-        <v>1.005890065496484</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="51" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="B45" s="47" t="n">
-        <v>2324380</v>
-      </c>
-      <c r="C45" s="43" t="n">
-        <v>1719964</v>
-      </c>
-      <c r="D45" s="45" t="n">
-        <v>1.351412006297806</v>
-      </c>
-      <c r="E45" s="70" t="inlineStr">
-        <is>
-          <t>above target by design — surplus fleet hauls LD</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="40" t="inlineStr">
-        <is>
-          <t>Scenario 3.1.1 — December (frozen, 1,281 DT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="41" t="inlineStr">
-        <is>
-          <t>Route</t>
-        </is>
-      </c>
-      <c r="B49" s="41" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="C49" s="41" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="D49" s="41" t="inlineStr">
-        <is>
-          <t>DT</t>
-        </is>
-      </c>
-      <c r="E49" s="41" t="inlineStr">
-        <is>
-          <t>t/day</t>
-        </is>
-      </c>
-      <c r="F49" s="41" t="inlineStr">
-        <is>
-          <t>t/month</t>
-        </is>
-      </c>
-      <c r="G49" s="41" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="67" t="inlineStr">
-        <is>
-          <t>TF&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B50" s="67" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C50" s="67" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="D50" s="68" t="n">
-        <v>393</v>
-      </c>
-      <c r="E50" s="43" t="n">
-        <v>41017</v>
-      </c>
-      <c r="F50" s="43" t="n">
-        <v>1271527</v>
-      </c>
-      <c r="G50" s="69" t="inlineStr">
-        <is>
-          <t>includes activated idle DT</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="67" t="inlineStr">
-        <is>
-          <t>TF&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B51" s="67" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C51" s="67" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="D51" s="68" t="n">
-        <v>241</v>
+      <c r="D51" s="43" t="n">
+        <v>62</v>
       </c>
       <c r="E51" s="43" t="n">
-        <v>25110</v>
-      </c>
-      <c r="F51" s="43" t="n">
-        <v>778410</v>
-      </c>
-      <c r="G51" s="69" t="inlineStr">
-        <is>
-          <t>includes activated idle DT</t>
-        </is>
+        <v>62</v>
+      </c>
+      <c r="F51" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="43" t="n">
+        <v>6477</v>
+      </c>
+      <c r="H51" s="43" t="n">
+        <v>200787</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="51" t="inlineStr">
         <is>
-          <t>BLB&gt;HUAFEI</t>
+          <t>KR&gt;HUAFEI</t>
         </is>
       </c>
       <c r="B52" s="51" t="inlineStr">
         <is>
-          <t>RIM</t>
+          <t>SMA</t>
         </is>
       </c>
       <c r="C52" s="51" t="inlineStr">
@@ -3086,20 +3142,25 @@
         </is>
       </c>
       <c r="D52" s="43" t="n">
-        <v>139</v>
+        <v>19</v>
       </c>
       <c r="E52" s="43" t="n">
-        <v>33851</v>
-      </c>
-      <c r="F52" s="43" t="n">
-        <v>1049381</v>
-      </c>
-      <c r="G52" s="66" t="n"/>
+        <v>19</v>
+      </c>
+      <c r="F52" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="43" t="n">
+        <v>2549</v>
+      </c>
+      <c r="H52" s="43" t="n">
+        <v>79019</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="51" t="inlineStr">
         <is>
-          <t>TF&gt;HUAFEI</t>
+          <t>BLB&gt;FENI KM0</t>
         </is>
       </c>
       <c r="B53" s="51" t="inlineStr">
@@ -3109,56 +3170,66 @@
       </c>
       <c r="C53" s="51" t="inlineStr">
         <is>
-          <t>LIM-TOS</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="D53" s="43" t="n">
-        <v>62</v>
+        <v>202</v>
       </c>
       <c r="E53" s="43" t="n">
-        <v>6471</v>
-      </c>
-      <c r="F53" s="43" t="n">
-        <v>200601</v>
-      </c>
-      <c r="G53" s="66" t="n"/>
+        <v>202</v>
+      </c>
+      <c r="F53" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="43" t="n">
+        <v>45786</v>
+      </c>
+      <c r="H53" s="43" t="n">
+        <v>1419366</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="51" t="inlineStr">
         <is>
-          <t>KR&gt;HUAFEI</t>
+          <t>TF&gt;FENI KM15</t>
         </is>
       </c>
       <c r="B54" s="51" t="inlineStr">
         <is>
-          <t>SMA</t>
+          <t>RIM</t>
         </is>
       </c>
       <c r="C54" s="51" t="inlineStr">
         <is>
-          <t>LIM-TOS</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="D54" s="43" t="n">
-        <v>19</v>
+        <v>140</v>
       </c>
       <c r="E54" s="43" t="n">
-        <v>2545</v>
-      </c>
-      <c r="F54" s="43" t="n">
-        <v>78895</v>
-      </c>
-      <c r="G54" s="66" t="n"/>
+        <v>140</v>
+      </c>
+      <c r="F54" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="43" t="n">
+        <v>14736</v>
+      </c>
+      <c r="H54" s="43" t="n">
+        <v>456816</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="51" t="inlineStr">
         <is>
-          <t>BLB&gt;FENI KM0</t>
+          <t>KR&gt;FENI KM15</t>
         </is>
       </c>
       <c r="B55" s="51" t="inlineStr">
         <is>
-          <t>RIM</t>
+          <t>SMA</t>
         </is>
       </c>
       <c r="C55" s="51" t="inlineStr">
@@ -3167,20 +3238,25 @@
         </is>
       </c>
       <c r="D55" s="43" t="n">
-        <v>202</v>
+        <v>50</v>
       </c>
       <c r="E55" s="43" t="n">
-        <v>45774</v>
-      </c>
-      <c r="F55" s="43" t="n">
-        <v>1418994</v>
-      </c>
-      <c r="G55" s="66" t="n"/>
+        <v>50</v>
+      </c>
+      <c r="F55" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="43" t="n">
+        <v>7958</v>
+      </c>
+      <c r="H55" s="43" t="n">
+        <v>246698</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="51" t="inlineStr">
         <is>
-          <t>TF&gt;FENI KM15</t>
+          <t>BLB&gt;POS 14</t>
         </is>
       </c>
       <c r="B56" s="51" t="inlineStr">
@@ -3194,25 +3270,30 @@
         </is>
       </c>
       <c r="D56" s="43" t="n">
-        <v>140</v>
+        <v>7</v>
       </c>
       <c r="E56" s="43" t="n">
-        <v>14702</v>
-      </c>
-      <c r="F56" s="43" t="n">
-        <v>455762</v>
-      </c>
-      <c r="G56" s="66" t="n"/>
+        <v>7</v>
+      </c>
+      <c r="F56" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="43" t="n">
+        <v>2044</v>
+      </c>
+      <c r="H56" s="43" t="n">
+        <v>63364</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="51" t="inlineStr">
         <is>
-          <t>KR&gt;FENI KM15</t>
+          <t>TF&gt;POS 12</t>
         </is>
       </c>
       <c r="B57" s="51" t="inlineStr">
         <is>
-          <t>SMA</t>
+          <t>RIM</t>
         </is>
       </c>
       <c r="C57" s="51" t="inlineStr">
@@ -3221,25 +3302,30 @@
         </is>
       </c>
       <c r="D57" s="43" t="n">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="E57" s="43" t="n">
-        <v>7919</v>
-      </c>
-      <c r="F57" s="43" t="n">
-        <v>245489</v>
-      </c>
-      <c r="G57" s="66" t="n"/>
+        <v>18</v>
+      </c>
+      <c r="F57" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="43" t="n">
+        <v>2039</v>
+      </c>
+      <c r="H57" s="43" t="n">
+        <v>63209</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="51" t="inlineStr">
         <is>
-          <t>BLB&gt;POS 14</t>
+          <t>KR&gt;POS 12</t>
         </is>
       </c>
       <c r="B58" s="51" t="inlineStr">
         <is>
-          <t>RIM</t>
+          <t>SMA</t>
         </is>
       </c>
       <c r="C58" s="51" t="inlineStr">
@@ -3248,483 +3334,415 @@
         </is>
       </c>
       <c r="D58" s="43" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E58" s="43" t="n">
-        <v>2043</v>
-      </c>
-      <c r="F58" s="43" t="n">
-        <v>63333</v>
-      </c>
-      <c r="G58" s="66" t="n"/>
+        <v>10</v>
+      </c>
+      <c r="F58" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="43" t="n">
+        <v>2009</v>
+      </c>
+      <c r="H58" s="43" t="n">
+        <v>62279</v>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;POS 12</t>
-        </is>
-      </c>
-      <c r="B59" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C59" s="51" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="D59" s="43" t="n">
-        <v>18</v>
-      </c>
-      <c r="E59" s="43" t="n">
-        <v>2037</v>
-      </c>
-      <c r="F59" s="43" t="n">
-        <v>63147</v>
-      </c>
-      <c r="G59" s="66" t="n"/>
+      <c r="A59" s="54" t="inlineStr">
+        <is>
+          <t>KR&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="B59" s="54" t="inlineStr">
+        <is>
+          <t>reallocated</t>
+        </is>
+      </c>
+      <c r="C59" s="54" t="inlineStr">
+        <is>
+          <t>SAP (stock at FeNi KM0)</t>
+        </is>
+      </c>
+      <c r="D59" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E59" s="56" t="n">
+        <v>40</v>
+      </c>
+      <c r="F59" s="56" t="n">
+        <v>40</v>
+      </c>
+      <c r="G59" s="56" t="n">
+        <v>5424</v>
+      </c>
+      <c r="H59" s="56" t="n">
+        <v>168135</v>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="51" t="inlineStr">
-        <is>
-          <t>KR&gt;POS 12</t>
-        </is>
-      </c>
-      <c r="B60" s="51" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C60" s="51" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="D60" s="43" t="n">
-        <v>10</v>
-      </c>
-      <c r="E60" s="43" t="n">
-        <v>1999</v>
-      </c>
-      <c r="F60" s="43" t="n">
-        <v>61969</v>
-      </c>
-      <c r="G60" s="66" t="n"/>
+      <c r="A60" s="54" t="inlineStr">
+        <is>
+          <t>TF&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="B60" s="54" t="inlineStr">
+        <is>
+          <t>reallocated</t>
+        </is>
+      </c>
+      <c r="C60" s="54" t="inlineStr">
+        <is>
+          <t>SAP (stock at FeNi KM0)</t>
+        </is>
+      </c>
+      <c r="D60" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E60" s="56" t="n">
+        <v>39</v>
+      </c>
+      <c r="F60" s="56" t="n">
+        <v>39</v>
+      </c>
+      <c r="G60" s="56" t="n">
+        <v>4289</v>
+      </c>
+      <c r="H60" s="56" t="n">
+        <v>132945</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="60" t="inlineStr">
         <is>
-          <t>TOTAL (full matrix pool)</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D61" s="47" t="n">
-        <v>1281</v>
-      </c>
-      <c r="F61" s="47" t="n">
-        <v>5687508</v>
+        <v>1190</v>
+      </c>
+      <c r="E61" s="47" t="n">
+        <v>1190</v>
+      </c>
+      <c r="H61" s="47" t="n">
+        <v>5333821</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="41" t="inlineStr">
+      <c r="A63" s="50" t="inlineStr">
+        <is>
+          <t>OPTION 2 — tonnage by material (December)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="41" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="B63" s="41" t="inlineStr">
-        <is>
-          <t>t/month (frozen)</t>
-        </is>
-      </c>
-      <c r="C63" s="41" t="inlineStr">
+      <c r="B64" s="41" t="inlineStr">
+        <is>
+          <t>BEFORE re-dispatch t/mo</t>
+        </is>
+      </c>
+      <c r="C64" s="41" t="inlineStr">
+        <is>
+          <t>AFTER re-dispatch t/mo</t>
+        </is>
+      </c>
+      <c r="D64" s="41" t="inlineStr">
+        <is>
+          <t>Δ t/mo</t>
+        </is>
+      </c>
+      <c r="E64" s="41" t="inlineStr">
+        <is>
+          <t>Change %</t>
+        </is>
+      </c>
+      <c r="F64" s="41" t="inlineStr">
         <is>
           <t>December TARGET t</t>
         </is>
       </c>
-      <c r="D63" s="41" t="inlineStr">
-        <is>
-          <t>Coverage</t>
-        </is>
-      </c>
-      <c r="E63" s="41" t="inlineStr"/>
-      <c r="F63" s="41" t="inlineStr"/>
-      <c r="G63" s="41" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="51" t="inlineStr">
+      <c r="G64" s="41" t="inlineStr">
+        <is>
+          <t>Coverage after</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="42" t="inlineStr">
         <is>
           <t>SAP</t>
         </is>
       </c>
-      <c r="B64" s="47" t="n">
-        <v>2308694</v>
-      </c>
-      <c r="C64" s="43" t="n">
+      <c r="B65" s="43" t="n">
+        <v>2311732</v>
+      </c>
+      <c r="C65" s="47" t="n">
+        <v>2612812</v>
+      </c>
+      <c r="D65" s="61" t="n">
+        <v>301080</v>
+      </c>
+      <c r="E65" s="62" t="n">
+        <v>0.1302400105202506</v>
+      </c>
+      <c r="F65" s="43" t="n">
         <v>2311213</v>
       </c>
-      <c r="D64" s="71" t="n">
-        <v>0.9989100961270121</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="51" t="inlineStr">
-        <is>
-          <t>LIM-TOS</t>
-        </is>
-      </c>
-      <c r="B65" s="47" t="n">
-        <v>1328877</v>
-      </c>
-      <c r="C65" s="43" t="n">
-        <v>1326082</v>
-      </c>
-      <c r="D65" s="45" t="n">
-        <v>1.002107712796041</v>
+      <c r="G65" s="45" t="n">
+        <v>1.13049381428713</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="51" t="inlineStr">
         <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="B66" s="43" t="n">
+        <v>1000556</v>
+      </c>
+      <c r="C66" s="47" t="n">
+        <v>1000556</v>
+      </c>
+      <c r="D66" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" s="43" t="n">
+        <v>996084</v>
+      </c>
+      <c r="G66" s="45" t="n">
+        <v>1.004489581199979</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="51" t="inlineStr">
+        <is>
           <t>LIM-LD</t>
         </is>
       </c>
-      <c r="B66" s="47" t="n">
-        <v>2049937</v>
-      </c>
-      <c r="C66" s="43" t="n">
-        <v>992213</v>
-      </c>
-      <c r="D66" s="45" t="n">
-        <v>2.066025137747641</v>
-      </c>
-      <c r="E66" s="70" t="inlineStr">
-        <is>
-          <t>above target by design — surplus fleet hauls LD</t>
+      <c r="B67" s="43" t="n">
+        <v>2031492</v>
+      </c>
+      <c r="C67" s="47" t="n">
+        <v>1720453</v>
+      </c>
+      <c r="D67" s="52" t="n">
+        <v>-311039</v>
+      </c>
+      <c r="E67" s="64" t="n">
+        <v>-0.1531086511785427</v>
+      </c>
+      <c r="F67" s="43" t="n">
+        <v>1719964</v>
+      </c>
+      <c r="G67" s="45" t="n">
+        <v>1.00028430827622</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="65" t="inlineStr">
+        <is>
+          <t>of which SAP stocked at FeNi KM0 (KR 40 DT + TF 39 DT reallocated)</t>
+        </is>
+      </c>
+      <c r="B68" s="66" t="n"/>
+      <c r="C68" s="61" t="n">
+        <v>301080</v>
+      </c>
+      <c r="D68" s="61" t="n">
+        <v>301080</v>
+      </c>
+      <c r="E68" s="70" t="inlineStr">
+        <is>
+          <t>inside the SAP row</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="40" t="inlineStr">
-        <is>
-          <t>Scenario 3.1.2 — December (frozen, 1,281 DT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="41" t="inlineStr">
+      <c r="A69" s="60" t="inlineStr">
+        <is>
+          <t>TOTAL moved</t>
+        </is>
+      </c>
+      <c r="B69" s="47" t="n">
+        <v>5343780</v>
+      </c>
+      <c r="C69" s="47" t="n">
+        <v>5333821</v>
+      </c>
+      <c r="D69" s="52" t="n">
+        <v>-9959</v>
+      </c>
+      <c r="E69" s="64" t="n">
+        <v>-0.001863662051955732</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="40" t="inlineStr">
+        <is>
+          <t>Scenario 3.1.1 — December</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="41" t="inlineStr"/>
+      <c r="B73" s="41" t="inlineStr">
+        <is>
+          <t>Target t</t>
+        </is>
+      </c>
+      <c r="C73" s="41" t="inlineStr">
+        <is>
+          <t>Predicted t</t>
+        </is>
+      </c>
+      <c r="D73" s="41" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="E73" s="41" t="inlineStr">
+        <is>
+          <t>Fleet DT</t>
+        </is>
+      </c>
+      <c r="F73" s="41" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="42" t="inlineStr">
+        <is>
+          <t>As frozen</t>
+        </is>
+      </c>
+      <c r="B74" s="43" t="n">
+        <v>4810381</v>
+      </c>
+      <c r="C74" s="43" t="n">
+        <v>4971401</v>
+      </c>
+      <c r="D74" s="44" t="n">
+        <v>1.033473440045601</v>
+      </c>
+      <c r="E74" s="43" t="n">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="42" t="inlineStr">
+        <is>
+          <t>OPTION 1 · park 49 DT (total month → 100.0%)</t>
+        </is>
+      </c>
+      <c r="B75" s="43" t="n">
+        <v>4810381</v>
+      </c>
+      <c r="C75" s="43" t="n">
+        <v>4811620</v>
+      </c>
+      <c r="D75" s="45" t="n">
+        <v>1.000257567955636</v>
+      </c>
+      <c r="E75" s="43" t="n">
+        <v>1003</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="42" t="inlineStr">
+        <is>
+          <t>OPTION 2 · re-dispatch 101 DT (LIM-LD → 100.0%)</t>
+        </is>
+      </c>
+      <c r="B76" s="43" t="n">
+        <v>4810381</v>
+      </c>
+      <c r="C76" s="43" t="n">
+        <v>5027004</v>
+      </c>
+      <c r="D76" s="46" t="n">
+        <v>1.045032399720521</v>
+      </c>
+      <c r="E76" s="43" t="n">
+        <v>1052</v>
+      </c>
+      <c r="F76" s="48" t="inlineStr">
+        <is>
+          <t>+ 384,923 t SAP stocked at FeNi KM0</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="49" t="inlineStr">
+        <is>
+          <t>Option 2 cut (sized so LIM-LD lands exactly on its line): TF&gt;HUAFEI (RIM, LD): −101 DT @ 105.2 t/day/DT</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="50" t="inlineStr">
+        <is>
+          <t>OPTION 2 — full December plan (re-dispatched)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="41" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="B70" s="41" t="inlineStr">
+      <c r="B80" s="41" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="C70" s="41" t="inlineStr">
+      <c r="C80" s="41" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="D70" s="41" t="inlineStr">
-        <is>
-          <t>DT</t>
-        </is>
-      </c>
-      <c r="E70" s="41" t="inlineStr">
+      <c r="D80" s="41" t="inlineStr">
+        <is>
+          <t>DT before</t>
+        </is>
+      </c>
+      <c r="E80" s="41" t="inlineStr">
+        <is>
+          <t>DT after</t>
+        </is>
+      </c>
+      <c r="F80" s="41" t="inlineStr">
+        <is>
+          <t>Δ DT</t>
+        </is>
+      </c>
+      <c r="G80" s="41" t="inlineStr">
         <is>
           <t>t/day</t>
         </is>
       </c>
-      <c r="F70" s="41" t="inlineStr">
+      <c r="H80" s="41" t="inlineStr">
         <is>
           <t>t/month</t>
         </is>
       </c>
-      <c r="G70" s="41" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="67" t="inlineStr">
-        <is>
-          <t>TF&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B71" s="67" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C71" s="67" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="D71" s="68" t="n">
-        <v>266</v>
-      </c>
-      <c r="E71" s="43" t="n">
-        <v>27708</v>
-      </c>
-      <c r="F71" s="43" t="n">
-        <v>858948</v>
-      </c>
-      <c r="G71" s="69" t="inlineStr">
-        <is>
-          <t>includes activated idle DT</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;POS 6</t>
-        </is>
-      </c>
-      <c r="B72" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C72" s="51" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="D72" s="43" t="n">
-        <v>126</v>
-      </c>
-      <c r="E72" s="43" t="n">
-        <v>15972</v>
-      </c>
-      <c r="F72" s="43" t="n">
-        <v>495132</v>
-      </c>
-      <c r="G72" s="66" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;POS 6</t>
-        </is>
-      </c>
-      <c r="B73" s="51" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C73" s="51" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="D73" s="43" t="n">
-        <v>120</v>
-      </c>
-      <c r="E73" s="43" t="n">
-        <v>13894</v>
-      </c>
-      <c r="F73" s="43" t="n">
-        <v>430714</v>
-      </c>
-      <c r="G73" s="66" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="67" t="inlineStr">
-        <is>
-          <t>TF&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B74" s="67" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C74" s="67" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="D74" s="68" t="n">
-        <v>121</v>
-      </c>
-      <c r="E74" s="43" t="n">
-        <v>12580</v>
-      </c>
-      <c r="F74" s="43" t="n">
-        <v>389980</v>
-      </c>
-      <c r="G74" s="69" t="inlineStr">
-        <is>
-          <t>includes activated idle DT</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="51" t="inlineStr">
-        <is>
-          <t>BLB&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B75" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C75" s="51" t="inlineStr">
-        <is>
-          <t>LIM-TOS</t>
-        </is>
-      </c>
-      <c r="D75" s="43" t="n">
-        <v>139</v>
-      </c>
-      <c r="E75" s="43" t="n">
-        <v>33851</v>
-      </c>
-      <c r="F75" s="43" t="n">
-        <v>1049381</v>
-      </c>
-      <c r="G75" s="66" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B76" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C76" s="51" t="inlineStr">
-        <is>
-          <t>LIM-TOS</t>
-        </is>
-      </c>
-      <c r="D76" s="43" t="n">
-        <v>63</v>
-      </c>
-      <c r="E76" s="43" t="n">
-        <v>6562</v>
-      </c>
-      <c r="F76" s="43" t="n">
-        <v>203422</v>
-      </c>
-      <c r="G76" s="66" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="51" t="inlineStr">
-        <is>
-          <t>KR&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B77" s="51" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C77" s="51" t="inlineStr">
-        <is>
-          <t>LIM-TOS</t>
-        </is>
-      </c>
-      <c r="D77" s="43" t="n">
-        <v>19</v>
-      </c>
-      <c r="E77" s="43" t="n">
-        <v>2528</v>
-      </c>
-      <c r="F77" s="43" t="n">
-        <v>78368</v>
-      </c>
-      <c r="G77" s="66" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="51" t="inlineStr">
-        <is>
-          <t>BLB&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="B78" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C78" s="51" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="D78" s="43" t="n">
-        <v>202</v>
-      </c>
-      <c r="E78" s="43" t="n">
-        <v>45774</v>
-      </c>
-      <c r="F78" s="43" t="n">
-        <v>1418994</v>
-      </c>
-      <c r="G78" s="66" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="B79" s="51" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C79" s="51" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="D79" s="43" t="n">
-        <v>140</v>
-      </c>
-      <c r="E79" s="43" t="n">
-        <v>14702</v>
-      </c>
-      <c r="F79" s="43" t="n">
-        <v>455762</v>
-      </c>
-      <c r="G79" s="66" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="51" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="B80" s="51" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C80" s="51" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="D80" s="43" t="n">
-        <v>50</v>
-      </c>
-      <c r="E80" s="43" t="n">
-        <v>7919</v>
-      </c>
-      <c r="F80" s="43" t="n">
-        <v>245489</v>
-      </c>
-      <c r="G80" s="66" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="51" t="inlineStr">
         <is>
-          <t>BLB&gt;POS 14</t>
+          <t>TF&gt;HUAFEI</t>
         </is>
       </c>
       <c r="B81" s="51" t="inlineStr">
@@ -3734,166 +3752,1399 @@
       </c>
       <c r="C81" s="51" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>LIM-LD</t>
         </is>
       </c>
       <c r="D81" s="43" t="n">
-        <v>7</v>
-      </c>
-      <c r="E81" s="43" t="n">
-        <v>2043</v>
-      </c>
-      <c r="F81" s="43" t="n">
-        <v>63333</v>
-      </c>
-      <c r="G81" s="66" t="n"/>
+        <v>319</v>
+      </c>
+      <c r="E81" s="47" t="n">
+        <v>218</v>
+      </c>
+      <c r="F81" s="52" t="n">
+        <v>-101</v>
+      </c>
+      <c r="G81" s="43" t="n">
+        <v>22932</v>
+      </c>
+      <c r="H81" s="43" t="n">
+        <v>710878</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="51" t="inlineStr">
         <is>
-          <t>TF&gt;POS 12</t>
+          <t>TF&gt;HUAFEI</t>
         </is>
       </c>
       <c r="B82" s="51" t="inlineStr">
         <is>
-          <t>RIM</t>
+          <t>SMA</t>
         </is>
       </c>
       <c r="C82" s="51" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>LIM-LD</t>
         </is>
       </c>
       <c r="D82" s="43" t="n">
-        <v>18</v>
+        <v>87</v>
       </c>
       <c r="E82" s="43" t="n">
-        <v>2037</v>
-      </c>
-      <c r="F82" s="43" t="n">
-        <v>63147</v>
-      </c>
-      <c r="G82" s="66" t="n"/>
+        <v>87</v>
+      </c>
+      <c r="F82" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" s="43" t="n">
+        <v>9142</v>
+      </c>
+      <c r="H82" s="43" t="n">
+        <v>283402</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="51" t="inlineStr">
         <is>
-          <t>KR&gt;POS 12</t>
+          <t>BLB&gt;HUAFEI</t>
         </is>
       </c>
       <c r="B83" s="51" t="inlineStr">
         <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C83" s="51" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="D83" s="43" t="n">
+        <v>139</v>
+      </c>
+      <c r="E83" s="43" t="n">
+        <v>139</v>
+      </c>
+      <c r="F83" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" s="43" t="n">
+        <v>33859</v>
+      </c>
+      <c r="H83" s="43" t="n">
+        <v>1049629</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="51" t="inlineStr">
+        <is>
+          <t>TF&gt;HUAFEI</t>
+        </is>
+      </c>
+      <c r="B84" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C84" s="51" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="D84" s="43" t="n">
+        <v>62</v>
+      </c>
+      <c r="E84" s="43" t="n">
+        <v>62</v>
+      </c>
+      <c r="F84" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="43" t="n">
+        <v>6522</v>
+      </c>
+      <c r="H84" s="43" t="n">
+        <v>202182</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="51" t="inlineStr">
+        <is>
+          <t>KR&gt;HUAFEI</t>
+        </is>
+      </c>
+      <c r="B85" s="51" t="inlineStr">
+        <is>
           <t>SMA</t>
         </is>
       </c>
-      <c r="C83" s="51" t="inlineStr">
+      <c r="C85" s="51" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="D85" s="43" t="n">
+        <v>19</v>
+      </c>
+      <c r="E85" s="43" t="n">
+        <v>19</v>
+      </c>
+      <c r="F85" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" s="43" t="n">
+        <v>2597</v>
+      </c>
+      <c r="H85" s="43" t="n">
+        <v>80507</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="51" t="inlineStr">
+        <is>
+          <t>BLB&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="B86" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C86" s="51" t="inlineStr">
         <is>
           <t>SAP</t>
         </is>
       </c>
-      <c r="D83" s="43" t="n">
-        <v>10</v>
-      </c>
-      <c r="E83" s="43" t="n">
-        <v>1999</v>
-      </c>
-      <c r="F83" s="43" t="n">
-        <v>61969</v>
-      </c>
-      <c r="G83" s="66" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="60" t="inlineStr">
-        <is>
-          <t>TOTAL (full matrix pool)</t>
-        </is>
-      </c>
-      <c r="D84" s="47" t="n">
-        <v>1281</v>
-      </c>
-      <c r="F84" s="47" t="n">
-        <v>5814639</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="41" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B86" s="41" t="inlineStr">
-        <is>
-          <t>t/month (frozen)</t>
-        </is>
-      </c>
-      <c r="C86" s="41" t="inlineStr">
-        <is>
-          <t>December TARGET t</t>
-        </is>
-      </c>
-      <c r="D86" s="41" t="inlineStr">
-        <is>
-          <t>Coverage</t>
-        </is>
-      </c>
-      <c r="E86" s="41" t="inlineStr"/>
-      <c r="F86" s="41" t="inlineStr"/>
-      <c r="G86" s="41" t="inlineStr"/>
+      <c r="D86" s="43" t="n">
+        <v>202</v>
+      </c>
+      <c r="E86" s="43" t="n">
+        <v>202</v>
+      </c>
+      <c r="F86" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="43" t="n">
+        <v>45786</v>
+      </c>
+      <c r="H86" s="43" t="n">
+        <v>1419366</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="51" t="inlineStr">
         <is>
+          <t>TF&gt;FENI KM15</t>
+        </is>
+      </c>
+      <c r="B87" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C87" s="51" t="inlineStr">
+        <is>
           <t>SAP</t>
         </is>
       </c>
-      <c r="B87" s="47" t="n">
-        <v>2308694</v>
-      </c>
-      <c r="C87" s="43" t="n">
-        <v>2311213</v>
-      </c>
-      <c r="D87" s="71" t="n">
-        <v>0.9989100961270121</v>
+      <c r="D87" s="43" t="n">
+        <v>140</v>
+      </c>
+      <c r="E87" s="43" t="n">
+        <v>140</v>
+      </c>
+      <c r="F87" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="43" t="n">
+        <v>14847</v>
+      </c>
+      <c r="H87" s="43" t="n">
+        <v>460257</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="51" t="inlineStr">
         <is>
-          <t>LIM-TOS</t>
-        </is>
-      </c>
-      <c r="B88" s="47" t="n">
-        <v>1331171</v>
-      </c>
-      <c r="C88" s="43" t="n">
-        <v>1326082</v>
-      </c>
-      <c r="D88" s="45" t="n">
-        <v>1.003837620901272</v>
+          <t>KR&gt;FENI KM15</t>
+        </is>
+      </c>
+      <c r="B88" s="51" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="C88" s="51" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D88" s="43" t="n">
+        <v>49</v>
+      </c>
+      <c r="E88" s="43" t="n">
+        <v>49</v>
+      </c>
+      <c r="F88" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="43" t="n">
+        <v>7929</v>
+      </c>
+      <c r="H88" s="43" t="n">
+        <v>245799</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="51" t="inlineStr">
         <is>
+          <t>TF&gt;POS 12</t>
+        </is>
+      </c>
+      <c r="B89" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C89" s="51" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D89" s="43" t="n">
+        <v>18</v>
+      </c>
+      <c r="E89" s="43" t="n">
+        <v>18</v>
+      </c>
+      <c r="F89" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="43" t="n">
+        <v>2045</v>
+      </c>
+      <c r="H89" s="43" t="n">
+        <v>63395</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="51" t="inlineStr">
+        <is>
+          <t>BLB&gt;POS 14</t>
+        </is>
+      </c>
+      <c r="B90" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C90" s="51" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D90" s="43" t="n">
+        <v>7</v>
+      </c>
+      <c r="E90" s="43" t="n">
+        <v>7</v>
+      </c>
+      <c r="F90" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" s="43" t="n">
+        <v>2044</v>
+      </c>
+      <c r="H90" s="43" t="n">
+        <v>63364</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="51" t="inlineStr">
+        <is>
+          <t>KR&gt;POS 12</t>
+        </is>
+      </c>
+      <c r="B91" s="51" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="C91" s="51" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D91" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="E91" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="F91" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" s="43" t="n">
+        <v>2042</v>
+      </c>
+      <c r="H91" s="43" t="n">
+        <v>63302</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="54" t="inlineStr">
+        <is>
+          <t>KR&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="B92" s="54" t="inlineStr">
+        <is>
+          <t>reallocated</t>
+        </is>
+      </c>
+      <c r="C92" s="54" t="inlineStr">
+        <is>
+          <t>SAP (stock at FeNi KM0)</t>
+        </is>
+      </c>
+      <c r="D92" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E92" s="56" t="n">
+        <v>51</v>
+      </c>
+      <c r="F92" s="56" t="n">
+        <v>51</v>
+      </c>
+      <c r="G92" s="56" t="n">
+        <v>6917</v>
+      </c>
+      <c r="H92" s="56" t="n">
+        <v>214423</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="54" t="inlineStr">
+        <is>
+          <t>TF&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="B93" s="54" t="inlineStr">
+        <is>
+          <t>reallocated</t>
+        </is>
+      </c>
+      <c r="C93" s="54" t="inlineStr">
+        <is>
+          <t>SAP (stock at FeNi KM0)</t>
+        </is>
+      </c>
+      <c r="D93" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E93" s="56" t="n">
+        <v>50</v>
+      </c>
+      <c r="F93" s="56" t="n">
+        <v>50</v>
+      </c>
+      <c r="G93" s="56" t="n">
+        <v>5500</v>
+      </c>
+      <c r="H93" s="56" t="n">
+        <v>170500</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="60" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D94" s="47" t="n">
+        <v>1052</v>
+      </c>
+      <c r="E94" s="47" t="n">
+        <v>1052</v>
+      </c>
+      <c r="H94" s="47" t="n">
+        <v>5027004</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="50" t="inlineStr">
+        <is>
+          <t>OPTION 2 — tonnage by material (December)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="41" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="B97" s="41" t="inlineStr">
+        <is>
+          <t>BEFORE re-dispatch t/mo</t>
+        </is>
+      </c>
+      <c r="C97" s="41" t="inlineStr">
+        <is>
+          <t>AFTER re-dispatch t/mo</t>
+        </is>
+      </c>
+      <c r="D97" s="41" t="inlineStr">
+        <is>
+          <t>Δ t/mo</t>
+        </is>
+      </c>
+      <c r="E97" s="41" t="inlineStr">
+        <is>
+          <t>Change %</t>
+        </is>
+      </c>
+      <c r="F97" s="41" t="inlineStr">
+        <is>
+          <t>December TARGET t</t>
+        </is>
+      </c>
+      <c r="G97" s="41" t="inlineStr">
+        <is>
+          <t>Coverage after</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="42" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="B98" s="43" t="n">
+        <v>2315483</v>
+      </c>
+      <c r="C98" s="47" t="n">
+        <v>2700406</v>
+      </c>
+      <c r="D98" s="61" t="n">
+        <v>384923</v>
+      </c>
+      <c r="E98" s="62" t="n">
+        <v>0.1662387501873259</v>
+      </c>
+      <c r="F98" s="43" t="n">
+        <v>2311213</v>
+      </c>
+      <c r="G98" s="45" t="n">
+        <v>1.168393393425876</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="51" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="B99" s="43" t="n">
+        <v>1332318</v>
+      </c>
+      <c r="C99" s="47" t="n">
+        <v>1332318</v>
+      </c>
+      <c r="D99" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" s="43" t="n">
+        <v>1326082</v>
+      </c>
+      <c r="G99" s="45" t="n">
+        <v>1.004702574953887</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="51" t="inlineStr">
+        <is>
           <t>LIM-LD</t>
         </is>
       </c>
-      <c r="B89" s="47" t="n">
-        <v>2174774</v>
-      </c>
-      <c r="C89" s="43" t="n">
+      <c r="B100" s="43" t="n">
+        <v>1323632</v>
+      </c>
+      <c r="C100" s="47" t="n">
+        <v>994280</v>
+      </c>
+      <c r="D100" s="52" t="n">
+        <v>-329352</v>
+      </c>
+      <c r="E100" s="64" t="n">
+        <v>-0.248824446674</v>
+      </c>
+      <c r="F100" s="43" t="n">
         <v>992213</v>
       </c>
-      <c r="D89" s="45" t="n">
-        <v>2.191841872662422</v>
-      </c>
-      <c r="E89" s="70" t="inlineStr">
-        <is>
-          <t>above target by design — surplus fleet hauls LD</t>
-        </is>
+      <c r="G100" s="45" t="n">
+        <v>1.002083222050104</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="65" t="inlineStr">
+        <is>
+          <t>of which SAP stocked at FeNi KM0 (KR 51 DT + TF 50 DT reallocated)</t>
+        </is>
+      </c>
+      <c r="B101" s="66" t="n"/>
+      <c r="C101" s="61" t="n">
+        <v>384923</v>
+      </c>
+      <c r="D101" s="61" t="n">
+        <v>384923</v>
+      </c>
+      <c r="E101" s="70" t="inlineStr">
+        <is>
+          <t>inside the SAP row</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="60" t="inlineStr">
+        <is>
+          <t>TOTAL moved</t>
+        </is>
+      </c>
+      <c r="B102" s="47" t="n">
+        <v>4971433</v>
+      </c>
+      <c r="C102" s="47" t="n">
+        <v>5027004</v>
+      </c>
+      <c r="D102" s="61" t="n">
+        <v>55571</v>
+      </c>
+      <c r="E102" s="62" t="n">
+        <v>0.0111780647551722</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="40" t="inlineStr">
+        <is>
+          <t>Scenario 3.1.2 — December</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="41" t="inlineStr"/>
+      <c r="B106" s="41" t="inlineStr">
+        <is>
+          <t>Target t</t>
+        </is>
+      </c>
+      <c r="C106" s="41" t="inlineStr">
+        <is>
+          <t>Predicted t</t>
+        </is>
+      </c>
+      <c r="D106" s="41" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="E106" s="41" t="inlineStr">
+        <is>
+          <t>Fleet DT</t>
+        </is>
+      </c>
+      <c r="F106" s="41" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="42" t="inlineStr">
+        <is>
+          <t>As frozen</t>
+        </is>
+      </c>
+      <c r="B107" s="43" t="n">
+        <v>4810381</v>
+      </c>
+      <c r="C107" s="43" t="n">
+        <v>5045234</v>
+      </c>
+      <c r="D107" s="44" t="n">
+        <v>1.048822120326852</v>
+      </c>
+      <c r="E107" s="43" t="n">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="42" t="inlineStr">
+        <is>
+          <t>OPTION 1 · park 59 DT (total month → 100.0%)</t>
+        </is>
+      </c>
+      <c r="B108" s="43" t="n">
+        <v>4810381</v>
+      </c>
+      <c r="C108" s="43" t="n">
+        <v>4811739</v>
+      </c>
+      <c r="D108" s="45" t="n">
+        <v>1.000282306120867</v>
+      </c>
+      <c r="E108" s="43" t="n">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="42" t="inlineStr">
+        <is>
+          <t>OPTION 2 · re-dispatch 104 DT (LIM-LD → 100.0%)</t>
+        </is>
+      </c>
+      <c r="B109" s="43" t="n">
+        <v>4810381</v>
+      </c>
+      <c r="C109" s="43" t="n">
+        <v>5035551</v>
+      </c>
+      <c r="D109" s="46" t="n">
+        <v>1.046809182058552</v>
+      </c>
+      <c r="E109" s="43" t="n">
+        <v>1052</v>
+      </c>
+      <c r="F109" s="48" t="inlineStr">
+        <is>
+          <t>+ 395,746 t SAP stocked at FeNi KM0</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="49" t="inlineStr">
+        <is>
+          <t>Option 2 cut (sized so LIM-LD lands exactly on its line): TF&gt;POS 6 (RIM, LD): −86 DT @ 127.7 t/day/DT · TF&gt;POS 6 (SMA, LD): −18 DT @ 116.6 t/day/DT</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="50" t="inlineStr">
+        <is>
+          <t>OPTION 2 — full December plan (re-dispatched)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="41" t="inlineStr">
+        <is>
+          <t>Route</t>
+        </is>
+      </c>
+      <c r="B113" s="41" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="C113" s="41" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="D113" s="41" t="inlineStr">
+        <is>
+          <t>DT before</t>
+        </is>
+      </c>
+      <c r="E113" s="41" t="inlineStr">
+        <is>
+          <t>DT after</t>
+        </is>
+      </c>
+      <c r="F113" s="41" t="inlineStr">
+        <is>
+          <t>Δ DT</t>
+        </is>
+      </c>
+      <c r="G113" s="41" t="inlineStr">
+        <is>
+          <t>t/day</t>
+        </is>
+      </c>
+      <c r="H113" s="41" t="inlineStr">
+        <is>
+          <t>t/month</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="51" t="inlineStr">
+        <is>
+          <t>TF&gt;HUAFEI</t>
+        </is>
+      </c>
+      <c r="B114" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C114" s="51" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="D114" s="43" t="n">
+        <v>233</v>
+      </c>
+      <c r="E114" s="43" t="n">
+        <v>233</v>
+      </c>
+      <c r="F114" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G114" s="43" t="n">
+        <v>24482</v>
+      </c>
+      <c r="H114" s="43" t="n">
+        <v>758942</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="51" t="inlineStr">
+        <is>
+          <t>TF&gt;POS 6</t>
+        </is>
+      </c>
+      <c r="B115" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C115" s="51" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="D115" s="43" t="n">
+        <v>86</v>
+      </c>
+      <c r="E115" s="47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F115" s="52" t="n">
+        <v>-86</v>
+      </c>
+      <c r="G115" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" s="43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="51" t="inlineStr">
+        <is>
+          <t>TF&gt;POS 6</t>
+        </is>
+      </c>
+      <c r="B116" s="51" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="C116" s="51" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="D116" s="43" t="n">
+        <v>43</v>
+      </c>
+      <c r="E116" s="47" t="n">
+        <v>25</v>
+      </c>
+      <c r="F116" s="52" t="n">
+        <v>-18</v>
+      </c>
+      <c r="G116" s="43" t="n">
+        <v>2915</v>
+      </c>
+      <c r="H116" s="43" t="n">
+        <v>90369</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="51" t="inlineStr">
+        <is>
+          <t>TF&gt;HUAFEI</t>
+        </is>
+      </c>
+      <c r="B117" s="51" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="C117" s="51" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="D117" s="43" t="n">
+        <v>44</v>
+      </c>
+      <c r="E117" s="43" t="n">
+        <v>44</v>
+      </c>
+      <c r="F117" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G117" s="43" t="n">
+        <v>4618</v>
+      </c>
+      <c r="H117" s="43" t="n">
+        <v>143158</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="51" t="inlineStr">
+        <is>
+          <t>BLB&gt;HUAFEI</t>
+        </is>
+      </c>
+      <c r="B118" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C118" s="51" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="D118" s="43" t="n">
+        <v>139</v>
+      </c>
+      <c r="E118" s="43" t="n">
+        <v>139</v>
+      </c>
+      <c r="F118" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G118" s="43" t="n">
+        <v>33859</v>
+      </c>
+      <c r="H118" s="43" t="n">
+        <v>1049629</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="51" t="inlineStr">
+        <is>
+          <t>TF&gt;HUAFEI</t>
+        </is>
+      </c>
+      <c r="B119" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C119" s="51" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="D119" s="43" t="n">
+        <v>62</v>
+      </c>
+      <c r="E119" s="43" t="n">
+        <v>62</v>
+      </c>
+      <c r="F119" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G119" s="43" t="n">
+        <v>6514</v>
+      </c>
+      <c r="H119" s="43" t="n">
+        <v>201934</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="51" t="inlineStr">
+        <is>
+          <t>KR&gt;HUAFEI</t>
+        </is>
+      </c>
+      <c r="B120" s="51" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="C120" s="51" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="D120" s="43" t="n">
+        <v>19</v>
+      </c>
+      <c r="E120" s="43" t="n">
+        <v>19</v>
+      </c>
+      <c r="F120" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G120" s="43" t="n">
+        <v>2590</v>
+      </c>
+      <c r="H120" s="43" t="n">
+        <v>80290</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="51" t="inlineStr">
+        <is>
+          <t>BLB&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="B121" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C121" s="51" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D121" s="43" t="n">
+        <v>202</v>
+      </c>
+      <c r="E121" s="43" t="n">
+        <v>202</v>
+      </c>
+      <c r="F121" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G121" s="43" t="n">
+        <v>45786</v>
+      </c>
+      <c r="H121" s="43" t="n">
+        <v>1419366</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="51" t="inlineStr">
+        <is>
+          <t>TF&gt;FENI KM15</t>
+        </is>
+      </c>
+      <c r="B122" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C122" s="51" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D122" s="43" t="n">
+        <v>140</v>
+      </c>
+      <c r="E122" s="43" t="n">
+        <v>140</v>
+      </c>
+      <c r="F122" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G122" s="43" t="n">
+        <v>14847</v>
+      </c>
+      <c r="H122" s="43" t="n">
+        <v>460257</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="51" t="inlineStr">
+        <is>
+          <t>KR&gt;FENI KM15</t>
+        </is>
+      </c>
+      <c r="B123" s="51" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="C123" s="51" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D123" s="43" t="n">
+        <v>49</v>
+      </c>
+      <c r="E123" s="43" t="n">
+        <v>49</v>
+      </c>
+      <c r="F123" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G123" s="43" t="n">
+        <v>7929</v>
+      </c>
+      <c r="H123" s="43" t="n">
+        <v>245799</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="51" t="inlineStr">
+        <is>
+          <t>TF&gt;POS 12</t>
+        </is>
+      </c>
+      <c r="B124" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C124" s="51" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D124" s="43" t="n">
+        <v>18</v>
+      </c>
+      <c r="E124" s="43" t="n">
+        <v>18</v>
+      </c>
+      <c r="F124" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G124" s="43" t="n">
+        <v>2045</v>
+      </c>
+      <c r="H124" s="43" t="n">
+        <v>63395</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="51" t="inlineStr">
+        <is>
+          <t>BLB&gt;POS 14</t>
+        </is>
+      </c>
+      <c r="B125" s="51" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C125" s="51" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D125" s="43" t="n">
+        <v>7</v>
+      </c>
+      <c r="E125" s="43" t="n">
+        <v>7</v>
+      </c>
+      <c r="F125" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G125" s="43" t="n">
+        <v>2044</v>
+      </c>
+      <c r="H125" s="43" t="n">
+        <v>63364</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="51" t="inlineStr">
+        <is>
+          <t>KR&gt;POS 12</t>
+        </is>
+      </c>
+      <c r="B126" s="51" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="C126" s="51" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="D126" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="E126" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="F126" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G126" s="43" t="n">
+        <v>2042</v>
+      </c>
+      <c r="H126" s="43" t="n">
+        <v>63302</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="54" t="inlineStr">
+        <is>
+          <t>KR&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="B127" s="54" t="inlineStr">
+        <is>
+          <t>reallocated</t>
+        </is>
+      </c>
+      <c r="C127" s="54" t="inlineStr">
+        <is>
+          <t>SAP (stock at FeNi KM0)</t>
+        </is>
+      </c>
+      <c r="D127" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E127" s="56" t="n">
+        <v>52</v>
+      </c>
+      <c r="F127" s="56" t="n">
+        <v>52</v>
+      </c>
+      <c r="G127" s="56" t="n">
+        <v>7049</v>
+      </c>
+      <c r="H127" s="56" t="n">
+        <v>218533</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="54" t="inlineStr">
+        <is>
+          <t>TF&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="B128" s="54" t="inlineStr">
+        <is>
+          <t>reallocated</t>
+        </is>
+      </c>
+      <c r="C128" s="54" t="inlineStr">
+        <is>
+          <t>SAP (stock at FeNi KM0)</t>
+        </is>
+      </c>
+      <c r="D128" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E128" s="56" t="n">
+        <v>52</v>
+      </c>
+      <c r="F128" s="56" t="n">
+        <v>52</v>
+      </c>
+      <c r="G128" s="56" t="n">
+        <v>5717</v>
+      </c>
+      <c r="H128" s="56" t="n">
+        <v>177213</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="60" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D129" s="47" t="n">
+        <v>1052</v>
+      </c>
+      <c r="E129" s="47" t="n">
+        <v>1052</v>
+      </c>
+      <c r="H129" s="47" t="n">
+        <v>5035551</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="50" t="inlineStr">
+        <is>
+          <t>OPTION 2 — tonnage by material (December)</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="41" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="B132" s="41" t="inlineStr">
+        <is>
+          <t>BEFORE re-dispatch t/mo</t>
+        </is>
+      </c>
+      <c r="C132" s="41" t="inlineStr">
+        <is>
+          <t>AFTER re-dispatch t/mo</t>
+        </is>
+      </c>
+      <c r="D132" s="41" t="inlineStr">
+        <is>
+          <t>Δ t/mo</t>
+        </is>
+      </c>
+      <c r="E132" s="41" t="inlineStr">
+        <is>
+          <t>Change %</t>
+        </is>
+      </c>
+      <c r="F132" s="41" t="inlineStr">
+        <is>
+          <t>December TARGET t</t>
+        </is>
+      </c>
+      <c r="G132" s="41" t="inlineStr">
+        <is>
+          <t>Coverage after</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="42" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="B133" s="43" t="n">
+        <v>2315483</v>
+      </c>
+      <c r="C133" s="47" t="n">
+        <v>2711229</v>
+      </c>
+      <c r="D133" s="61" t="n">
+        <v>395746</v>
+      </c>
+      <c r="E133" s="62" t="n">
+        <v>0.1709129369552702</v>
+      </c>
+      <c r="F133" s="43" t="n">
+        <v>2311213</v>
+      </c>
+      <c r="G133" s="45" t="n">
+        <v>1.1730762158226</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="51" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="B134" s="43" t="n">
+        <v>1331853</v>
+      </c>
+      <c r="C134" s="47" t="n">
+        <v>1331853</v>
+      </c>
+      <c r="D134" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E134" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F134" s="43" t="n">
+        <v>1326082</v>
+      </c>
+      <c r="G134" s="45" t="n">
+        <v>1.004351917905529</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="51" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="B135" s="43" t="n">
+        <v>1397954</v>
+      </c>
+      <c r="C135" s="47" t="n">
+        <v>992469</v>
+      </c>
+      <c r="D135" s="52" t="n">
+        <v>-405485</v>
+      </c>
+      <c r="E135" s="64" t="n">
+        <v>-0.2900560390399112</v>
+      </c>
+      <c r="F135" s="43" t="n">
+        <v>992213</v>
+      </c>
+      <c r="G135" s="45" t="n">
+        <v>1.000258009116994</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="65" t="inlineStr">
+        <is>
+          <t>of which SAP stocked at FeNi KM0 (KR 52 DT + TF 52 DT reallocated)</t>
+        </is>
+      </c>
+      <c r="B136" s="66" t="n"/>
+      <c r="C136" s="61" t="n">
+        <v>395746</v>
+      </c>
+      <c r="D136" s="61" t="n">
+        <v>395746</v>
+      </c>
+      <c r="E136" s="70" t="inlineStr">
+        <is>
+          <t>inside the SAP row</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="60" t="inlineStr">
+        <is>
+          <t>TOTAL moved</t>
+        </is>
+      </c>
+      <c r="B137" s="47" t="n">
+        <v>5045290</v>
+      </c>
+      <c r="C137" s="47" t="n">
+        <v>5035551</v>
+      </c>
+      <c r="D137" s="52" t="n">
+        <v>-9739</v>
+      </c>
+      <c r="E137" s="64" t="n">
+        <v>-0.001930315204874249</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="A101:B101"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A136:B136"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Comparison workbook rebuilt on the refrozen plans — same template, new numbers
Owner: redo the comparison with the same options and template, numbers
per the new updates. All three sheets now read the post-refreeze world
(1,281 DT December, exact 50/50 POS 6, surplus on LD by rule):

Compare — year coverage 98.4 / 101.7 / 101.7 / 104.6% (was 96.8 / 99.6 /
97.5 / 99.8%), Dec DT 1,281 in all four (was 1,190 / 1,190 / 1,052 /
1,052), plus a new year-by-material block against the sales lines.
December options — the frozen plan per scenario, LD rows flagged as the
carriers of the surplus fleet. Insights — six findings refreshed,
including the road actually carrying 1,948-2,650 DT once the 1,340-DT
tenant register is counted.
</commit_message>
<xml_diff>
--- a/reports/scenario_comparison_dec_options.xlsx
+++ b/reports/scenario_comparison_dec_options.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="167" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="168" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="53">
+  <fonts count="55">
     <font>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -380,6 +380,17 @@
       <name val="Arial"/>
       <color rgb="008A6100"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000F4C81"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001A2332"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="40">
@@ -974,7 +985,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1165,6 +1176,10 @@
     </xf>
     <xf numFmtId="0" fontId="52" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1578,436 +1593,561 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
+  <dimension ref="A1:H33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="23.2" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Four scenarios · Sep–Dec 2026 · one clock (sales targets)</t>
+    <row r="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>Four scenarios · Sep–Dec 2026 · refrozen at the full 1,281-DT December pool</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t>3.0 = base mining plan · 3.1 = +330 kt/month BLB LIM Oct–Dec (the sales table already contains it). .1 = all leftover LD trucks to HUAFEI/BSE · .2 = half to POS 6 from October. All targets are the sales lines distributed over months in the plan shape.</t>
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>3.0 = base mining plan · 3.1 = +330 kt/mo BLB LIM Oct–Dec · .1 = all leftover LD to HUAFEI/BSE · .2 = half the TF LD trucks to POS 6 from October (exact 50/50). Every truck in the matrix pool works: SAP 100%, LIM-TOS 100%, all remaining DT haul LIM-LD past its target.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="41" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="41" t="inlineStr">
         <is>
           <t>Year sales target</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="41" t="inlineStr">
         <is>
           <t>Predicted plan</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="41" t="inlineStr">
         <is>
           <t>Coverage</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="41" t="inlineStr">
         <is>
           <t>SAP %</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="41" t="inlineStr">
         <is>
           <t>LIM-TOS %</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="41" t="inlineStr">
         <is>
           <t>LIM-LD %</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="41" t="inlineStr">
         <is>
           <t>Dec DT</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="42" t="inlineStr">
         <is>
           <t>3.0.1</t>
         </is>
       </c>
-      <c r="B5" s="31" t="n">
+      <c r="B5" s="43" t="n">
         <v>17003193</v>
       </c>
-      <c r="C5" s="31" t="n">
-        <v>16453539</v>
-      </c>
-      <c r="D5" s="36" t="n">
-        <v>0.968</v>
-      </c>
-      <c r="E5" s="37" t="n">
-        <v>1.00547485908476</v>
-      </c>
-      <c r="F5" s="37" t="n">
-        <v>1.00502547667923</v>
-      </c>
-      <c r="G5" s="36" t="n">
-        <v>0.921500002750741</v>
-      </c>
-      <c r="H5" s="31" t="n">
-        <v>1190</v>
-      </c>
-    </row>
-    <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="C5" s="43" t="n">
+        <v>16738008</v>
+      </c>
+      <c r="D5" s="71" t="n">
+        <v>0.9840000000000001</v>
+      </c>
+      <c r="E5" s="45" t="n">
+        <v>1.006</v>
+      </c>
+      <c r="F5" s="45" t="n">
+        <v>1.005</v>
+      </c>
+      <c r="G5" s="71" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="H5" s="47" t="n">
+        <v>1281</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="42" t="inlineStr">
         <is>
           <t>3.0.2</t>
         </is>
       </c>
-      <c r="B6" s="31" t="n">
+      <c r="B6" s="43" t="n">
         <v>17003193</v>
       </c>
-      <c r="C6" s="31" t="n">
-        <v>16941732</v>
-      </c>
-      <c r="D6" s="36" t="n">
-        <v>0.996</v>
-      </c>
-      <c r="E6" s="37" t="n">
-        <v>1.00547485908476</v>
-      </c>
-      <c r="F6" s="37" t="n">
-        <v>1.00587063561705</v>
-      </c>
-      <c r="G6" s="36" t="n">
-        <v>0.985040159511552</v>
-      </c>
-      <c r="H6" s="31" t="n">
-        <v>1190</v>
-      </c>
-    </row>
-    <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="30" t="inlineStr">
+      <c r="C6" s="43" t="n">
+        <v>17286699</v>
+      </c>
+      <c r="D6" s="45" t="n">
+        <v>1.017</v>
+      </c>
+      <c r="E6" s="45" t="n">
+        <v>1.006</v>
+      </c>
+      <c r="F6" s="45" t="n">
+        <v>1.006</v>
+      </c>
+      <c r="G6" s="45" t="n">
+        <v>1.029</v>
+      </c>
+      <c r="H6" s="47" t="n">
+        <v>1281</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="42" t="inlineStr">
         <is>
           <t>3.1.1</t>
         </is>
       </c>
-      <c r="B7" s="31" t="n">
+      <c r="B7" s="43" t="n">
         <v>17003193</v>
       </c>
-      <c r="C7" s="31" t="n">
-        <v>16580201</v>
-      </c>
-      <c r="D7" s="36" t="n">
-        <v>0.975</v>
-      </c>
-      <c r="E7" s="37" t="n">
-        <v>1.00506182714001</v>
-      </c>
-      <c r="F7" s="37" t="n">
-        <v>1.00347592701264</v>
-      </c>
-      <c r="G7" s="36" t="n">
-        <v>0.92954674272979</v>
-      </c>
-      <c r="H7" s="31" t="n">
-        <v>1052</v>
-      </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="C7" s="43" t="n">
+        <v>17296329</v>
+      </c>
+      <c r="D7" s="45" t="n">
+        <v>1.017</v>
+      </c>
+      <c r="E7" s="45" t="n">
+        <v>1.004</v>
+      </c>
+      <c r="F7" s="45" t="n">
+        <v>1.003</v>
+      </c>
+      <c r="G7" s="45" t="n">
+        <v>1.039</v>
+      </c>
+      <c r="H7" s="47" t="n">
+        <v>1281</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="42" t="inlineStr">
         <is>
           <t>3.1.2</t>
         </is>
       </c>
-      <c r="B8" s="31" t="n">
+      <c r="B8" s="43" t="n">
         <v>17003193</v>
       </c>
-      <c r="C8" s="31" t="n">
-        <v>16974809</v>
-      </c>
-      <c r="D8" s="36" t="n">
-        <v>0.998</v>
-      </c>
-      <c r="E8" s="37" t="n">
-        <v>1.00506182714001</v>
-      </c>
-      <c r="F8" s="37" t="n">
-        <v>1.00347161685453</v>
-      </c>
-      <c r="G8" s="36" t="n">
-        <v>0.9889440672961179</v>
-      </c>
-      <c r="H8" s="31" t="n">
-        <v>1052</v>
-      </c>
-    </row>
-    <row r="11" ht="19.2" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Month by month — Predicted % of the distributed sales target</t>
+      <c r="C8" s="43" t="n">
+        <v>17791858</v>
+      </c>
+      <c r="D8" s="45" t="n">
+        <v>1.046</v>
+      </c>
+      <c r="E8" s="45" t="n">
+        <v>1.004</v>
+      </c>
+      <c r="F8" s="45" t="n">
+        <v>1.003</v>
+      </c>
+      <c r="G8" s="45" t="n">
+        <v>1.113</v>
+      </c>
+      <c r="H8" s="47" t="n">
+        <v>1281</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="50" t="inlineStr">
+        <is>
+          <t>Month by month — Predicted ÷ target</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="41" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="41" t="inlineStr">
         <is>
           <t>3.0.1</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="41" t="inlineStr">
         <is>
           <t>3.0.2</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="41" t="inlineStr">
         <is>
           <t>3.1.1</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="41" t="inlineStr">
         <is>
           <t>3.1.2</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="34" t="inlineStr">
+      <c r="A13" s="42" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="B13" s="36" t="n">
-        <v>0.962</v>
-      </c>
-      <c r="C13" s="36" t="n">
-        <v>0.962</v>
-      </c>
-      <c r="D13" s="36" t="n">
-        <v>0.962</v>
-      </c>
-      <c r="E13" s="36" t="n">
-        <v>0.962</v>
+      <c r="B13" s="45" t="n">
+        <v>1.045482521411984</v>
+      </c>
+      <c r="C13" s="45" t="n">
+        <v>1.045482521411984</v>
+      </c>
+      <c r="D13" s="45" t="n">
+        <v>1.045482521411984</v>
+      </c>
+      <c r="E13" s="45" t="n">
+        <v>1.045482521411984</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="34" t="inlineStr">
+      <c r="A14" s="42" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="B14" s="36" t="n">
-        <v>0.9320000000000001</v>
-      </c>
-      <c r="C14" s="36" t="n">
-        <v>0.971</v>
-      </c>
-      <c r="D14" s="36" t="n">
-        <v>0.9350000000000001</v>
-      </c>
-      <c r="E14" s="36" t="n">
-        <v>0.968</v>
+      <c r="B14" s="45" t="n">
+        <v>1.012856749072166</v>
+      </c>
+      <c r="C14" s="45" t="n">
+        <v>1.055805550922092</v>
+      </c>
+      <c r="D14" s="45" t="n">
+        <v>1.016155521828965</v>
+      </c>
+      <c r="E14" s="45" t="n">
+        <v>1.051434176532733</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="34" t="inlineStr">
+      <c r="A15" s="42" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="B15" s="36" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="C15" s="36" t="n">
-        <v>0.988</v>
-      </c>
-      <c r="D15" s="36" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="E15" s="36" t="n">
-        <v>0.994</v>
+      <c r="B15" s="45" t="n">
+        <v>1.033122002370932</v>
+      </c>
+      <c r="C15" s="45" t="n">
+        <v>1.074038091902804</v>
+      </c>
+      <c r="D15" s="45" t="n">
+        <v>1.043424413593518</v>
+      </c>
+      <c r="E15" s="45" t="n">
+        <v>1.079733218673122</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="34" t="inlineStr">
+      <c r="A16" s="42" t="inlineStr">
         <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="B16" s="37" t="n">
-        <v>1.017</v>
-      </c>
-      <c r="C16" s="37" t="n">
-        <v>1.041</v>
-      </c>
-      <c r="D16" s="37" t="n">
-        <v>1.033</v>
-      </c>
-      <c r="E16" s="37" t="n">
-        <v>1.049</v>
+      <c r="B16" s="45" t="n">
+        <v>1.099858328904862</v>
+      </c>
+      <c r="C16" s="45" t="n">
+        <v>1.137358183954899</v>
+      </c>
+      <c r="D16" s="45" t="n">
+        <v>1.09793766371253</v>
+      </c>
+      <c r="E16" s="45" t="n">
+        <v>1.131672700225648</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>Reading: every month judges its share of the sales target. December is the only month above 100% in all four scenarios — the December sheet gives the two options to land it at exactly 100%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="19.2" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Month by month — Predicted tonnes</t>
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>Reading: every month is now run with its whole fleet, so coverage is at or above 100% from October on. September is short because the matrix only fields 581 DT that month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="50" t="inlineStr">
+        <is>
+          <t>Month by month — Predicted plan t</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="41" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="41" t="inlineStr">
         <is>
           <t>3.0.1</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="41" t="inlineStr">
         <is>
           <t>3.0.2</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="41" t="inlineStr">
         <is>
           <t>3.1.1</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="41" t="inlineStr">
         <is>
           <t>3.1.2</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="34" t="inlineStr">
+      <c r="A22" s="42" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="B22" s="31" t="n">
+      <c r="B22" s="43" t="n">
         <v>2381536</v>
       </c>
-      <c r="C22" s="31" t="n">
+      <c r="C22" s="43" t="n">
         <v>2381536</v>
       </c>
-      <c r="D22" s="31" t="n">
+      <c r="D22" s="43" t="n">
         <v>2381536</v>
       </c>
-      <c r="E22" s="31" t="n">
+      <c r="E22" s="43" t="n">
         <v>2381536</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="34" t="inlineStr">
+      <c r="A23" s="42" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="B23" s="31" t="n">
+      <c r="B23" s="43" t="n">
         <v>3722205</v>
       </c>
-      <c r="C23" s="31" t="n">
+      <c r="C23" s="43" t="n">
         <v>3880040</v>
       </c>
-      <c r="D23" s="31" t="n">
+      <c r="D23" s="43" t="n">
         <v>3912780</v>
       </c>
-      <c r="E23" s="31" t="n">
+      <c r="E23" s="43" t="n">
         <v>4048623</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="34" t="inlineStr">
+      <c r="A24" s="42" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="B24" s="31" t="n">
+      <c r="B24" s="43" t="n">
         <v>5133077</v>
       </c>
-      <c r="C24" s="31" t="n">
+      <c r="C24" s="43" t="n">
         <v>5336369</v>
       </c>
-      <c r="D24" s="31" t="n">
+      <c r="D24" s="43" t="n">
         <v>5314484</v>
       </c>
-      <c r="E24" s="31" t="n">
+      <c r="E24" s="43" t="n">
         <v>5499416</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="34" t="inlineStr">
+      <c r="A25" s="42" t="inlineStr">
         <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="B25" s="31" t="n">
-        <v>5216721</v>
-      </c>
-      <c r="C25" s="31" t="n">
-        <v>5343787</v>
-      </c>
-      <c r="D25" s="31" t="n">
-        <v>4971401</v>
-      </c>
-      <c r="E25" s="31" t="n">
-        <v>5045234</v>
+      <c r="B25" s="43" t="n">
+        <v>5501190</v>
+      </c>
+      <c r="C25" s="43" t="n">
+        <v>5688754</v>
+      </c>
+      <c r="D25" s="43" t="n">
+        <v>5687529</v>
+      </c>
+      <c r="E25" s="43" t="n">
+        <v>5862283</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="34" t="inlineStr">
+      <c r="A26" s="60" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B26" s="35" t="n">
-        <v>16453539</v>
-      </c>
-      <c r="C26" s="35" t="n">
-        <v>16941732</v>
-      </c>
-      <c r="D26" s="35" t="n">
-        <v>16580201</v>
-      </c>
-      <c r="E26" s="35" t="n">
-        <v>16974809</v>
+      <c r="B26" s="47" t="n">
+        <v>16738008</v>
+      </c>
+      <c r="C26" s="47" t="n">
+        <v>17286699</v>
+      </c>
+      <c r="D26" s="47" t="n">
+        <v>17296329</v>
+      </c>
+      <c r="E26" s="47" t="n">
+        <v>17791858</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="50" t="inlineStr">
+        <is>
+          <t>Year tonnage by material (t) — predicted vs sales line</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="41" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="B29" s="41" t="inlineStr">
+        <is>
+          <t>Sales line</t>
+        </is>
+      </c>
+      <c r="C29" s="41" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="D29" s="41" t="inlineStr">
+        <is>
+          <t>3.0.2</t>
+        </is>
+      </c>
+      <c r="E29" s="41" t="inlineStr">
+        <is>
+          <t>3.1.1</t>
+        </is>
+      </c>
+      <c r="F29" s="41" t="inlineStr">
+        <is>
+          <t>3.1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="42" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="B30" s="43" t="n">
+        <v>5718686</v>
+      </c>
+      <c r="C30" s="43" t="n">
+        <v>5754583</v>
+      </c>
+      <c r="D30" s="43" t="n">
+        <v>5754366</v>
+      </c>
+      <c r="E30" s="43" t="n">
+        <v>5740906</v>
+      </c>
+      <c r="F30" s="43" t="n">
+        <v>5740906</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="42" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="B31" s="43" t="n">
+        <v>3650201</v>
+      </c>
+      <c r="C31" s="43" t="n">
+        <v>3667243</v>
+      </c>
+      <c r="D31" s="43" t="n">
+        <v>3672901</v>
+      </c>
+      <c r="E31" s="43" t="n">
+        <v>4652858</v>
+      </c>
+      <c r="F31" s="43" t="n">
+        <v>4655256</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="42" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="B32" s="43" t="n">
+        <v>7634306</v>
+      </c>
+      <c r="C32" s="43" t="n">
+        <v>7316183</v>
+      </c>
+      <c r="D32" s="43" t="n">
+        <v>7859393</v>
+      </c>
+      <c r="E32" s="43" t="n">
+        <v>6902523</v>
+      </c>
+      <c r="F32" s="43" t="n">
+        <v>7395695</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="60" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B33" s="47" t="n">
+        <v>17003193</v>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>16738008</v>
+      </c>
+      <c r="D33" s="47" t="n">
+        <v>17286699</v>
+      </c>
+      <c r="E33" s="47" t="n">
+        <v>17296329</v>
+      </c>
+      <c r="F33" s="47" t="n">
+        <v>17791858</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A18:I18"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3923,112 +4063,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
+  <dimension ref="A1:A19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="140" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="23.2" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="73" t="inlineStr">
         <is>
           <t>Insights</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>1 · The scenarios are separated by LD, nothing else.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>SAP and LIM-TOS clear their sales lines in all four scenarios (100.3–100.5%). The whole difference between plans is how much LIM-LD the leftover fleet can move: 92.2–93.0% of its line. TF&gt;HUAFEI is the binding corridor.</t>
+      <c r="A3" s="50" t="inlineStr">
+        <is>
+          <t>1 · Every truck now works, so the year clears its line in three of four scenarios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="74" t="inlineStr">
+        <is>
+          <t>With the full December pool fielded (1,281 DT: RIM 961 + SMA 320) the year predicts 16,738,008 / 17,286,699 / 17,296,329 / 17,791,858 t — 98.4%, 101.7%, 101.7% and 104.6% of the 17,003,193 t sales line. Only 3.0.1 stays just under.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>2 · The .2 split scenarios move more total tonnes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>3.0.2 predicts ~488 kt more than 3.0.1 (97.7% vs 96.8% of 17.0 Mt); 3.1.2 ~395 kt more than 3.1.1. Splitting leftover LD trucks to POS 6 relieves the saturated HUAFEI corridor - the split is worth roughly half a million tonnes over the quarter.</t>
+      <c r="A6" s="50" t="inlineStr">
+        <is>
+          <t>2 · The scenarios still differ only in LIM-LD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="74" t="inlineStr">
+        <is>
+          <t>SAP and LIM-TOS clear their lines in all four (99.9-100.6%). The whole spread between plans is how much LIM-LD the leftover fleet moves — and since the surplus now rides LD by rule, LD is where the extra tonnage lands.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>3 · December is the only month with slack.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Sep-Nov run 93-97% of their distributed sales share in every scenario; December runs 101.7-104.9%. The fleet grows to 1,190-1,280 DT while the remaining target shrinks - December has spare trucks.</t>
+      <c r="A9" s="50" t="inlineStr">
+        <is>
+          <t>3 · The .2 split is worth roughly half a megatonne a year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="74" t="inlineStr">
+        <is>
+          <t>3.0.2 predicts 548,691 t more than 3.0.1 and 3.1.2 predicts 495,529 t more than 3.1.1. Splitting the leftover TF LD trucks to POS 6 (exact 50/50 per contractor since the 2026-08-27 fix) relieves the saturated HUAFEI corridor.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>4 · Option 1 (park) reaches 100% but wastes capacity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Parking 26-59 DT lands the total month at exactly 100.0%. Simple, but those trucks produce nothing and the plants build no buffer.</t>
+      <c r="A12" s="50" t="inlineStr">
+        <is>
+          <t>4 · The 3.1 uplift pays for itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="74" t="inlineStr">
+        <is>
+          <t>3.1 adds 330 kt/mo of BLB LIM TOS in Oct-Dec. It lifts LIM-TOS from 3.65 Mt to 4.64 Mt and still leaves enough fleet for LD, because the total haulage line is constant at 17.0 Mt — 3.0 simply carries the difference in LD.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>5 · Option 2 (re-dispatch to stock) is strictly better if KM0 can take stock.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="42" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Sized to the real goal — LIM-LD at exactly 100% — the cut is 56-104 DT, and re-dispatching them to KR&gt;FENI KM0 + TF&gt;FENI KM0 builds 213-396 kt of kilnable SAP stock at the plant in December while every sales line still clears (SAP rises to 109-117%). Requires KM0 to accept stock.</t>
+      <c r="A15" s="50" t="inlineStr">
+        <is>
+          <t>5 · December is the month with real slack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="74" t="inlineStr">
+        <is>
+          <t>Sep-Nov are fleet-limited (581 / 931 / 1,280 DT from the matrix). December fields 1,281 and lands above every line: SAP ~100%, TOS ~100%, LD 127-224% depending on scenario. The surplus is deliberate — the target is a goal, not a ceiling.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>6 · Where the cuts come from.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>In .1 scenarios the donor is TF&gt;HUAFEI RIM (the biggest untensioned LD row); in .2 scenarios the donor is the TF&gt;POS 6 split flow (untargeted by design). No targeted route drops below its own line in any option.</t>
+      <c r="A18" s="50" t="inlineStr">
+        <is>
+          <t>6 · The road carries far more than our fleet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="74" t="inlineStr">
+        <is>
+          <t>Road crowding is priced on 1,948 / 2,299 / 2,650 / 2,650 DT for Sep-Dec: our plan plus IWIP transit plus the 1,340-DT tenant register (POSITION 500, HUAFEI&gt;RSF 500, PMA 150, MHM 100, HSM 50, KR&gt;RSF 40). POS 12-KM15 runs RED on that basis in every month. Those trucks are not ours to schedule but they take the lane.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A19:H19"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reclaiming WMT shown in the comparison workbook (Compare block + per-scenario line)
</commit_message>
<xml_diff>
--- a/reports/scenario_comparison_dec_options.xlsx
+++ b/reports/scenario_comparison_dec_options.xlsx
@@ -419,7 +419,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="41">
     <fill>
       <patternFill/>
     </fill>
@@ -650,6 +650,11 @@
         <fgColor rgb="00FFF4DC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF3FA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="18">
     <border>
@@ -1011,7 +1016,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1234,6 +1239,22 @@
     </xf>
     <xf numFmtId="164" fontId="47" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="43" fillId="40" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="40" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="49" fillId="40" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="40" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1647,7 +1668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2292,6 +2313,256 @@
         <v>17791858</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="50" t="inlineStr">
+        <is>
+          <t>RECLAIMING — WMT moved out of the POS stockpiles (IWIP own fleet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="28" customHeight="1">
+      <c r="A44" s="49" t="inlineStr">
+        <is>
+          <t>Material we dump INTO a POS has to come back out to the plant. IWIP runs that leg with its own trucks (not in our 1,281 DT and not in the sales tonnage above), and input must equal output — so the reclaim WMT below equals what the plan tips into POS 12 / POS 14 / POS 6 that month. The .2 scenarios reclaim far more because the POS 6 split sends half the TF LD trucks there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="41" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B45" s="41" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="C45" s="41" t="inlineStr">
+        <is>
+          <t>3.0.2</t>
+        </is>
+      </c>
+      <c r="D45" s="41" t="inlineStr">
+        <is>
+          <t>3.1.1</t>
+        </is>
+      </c>
+      <c r="E45" s="41" t="inlineStr">
+        <is>
+          <t>3.1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="42" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="B46" s="85" t="n">
+        <v>184890</v>
+      </c>
+      <c r="C46" s="85" t="n">
+        <v>184890</v>
+      </c>
+      <c r="D46" s="85" t="n">
+        <v>184890</v>
+      </c>
+      <c r="E46" s="85" t="n">
+        <v>184890</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="42" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="B47" s="85" t="n">
+        <v>189472</v>
+      </c>
+      <c r="C47" s="85" t="n">
+        <v>1294622</v>
+      </c>
+      <c r="D47" s="85" t="n">
+        <v>189751</v>
+      </c>
+      <c r="E47" s="85" t="n">
+        <v>1129826</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="42" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="B48" s="85" t="n">
+        <v>187650</v>
+      </c>
+      <c r="C48" s="85" t="n">
+        <v>1594740</v>
+      </c>
+      <c r="D48" s="85" t="n">
+        <v>182130</v>
+      </c>
+      <c r="E48" s="85" t="n">
+        <v>1465470</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="42" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="B49" s="85" t="n">
+        <v>194308</v>
+      </c>
+      <c r="C49" s="85" t="n">
+        <v>1476499</v>
+      </c>
+      <c r="D49" s="85" t="n">
+        <v>188449</v>
+      </c>
+      <c r="E49" s="85" t="n">
+        <v>1389141</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="60" t="inlineStr">
+        <is>
+          <t>TOTAL Sep–Dec</t>
+        </is>
+      </c>
+      <c r="B50" s="61" t="n">
+        <v>756320</v>
+      </c>
+      <c r="C50" s="61" t="n">
+        <v>4550751</v>
+      </c>
+      <c r="D50" s="61" t="n">
+        <v>745220</v>
+      </c>
+      <c r="E50" s="61" t="n">
+        <v>4169327</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="42" t="inlineStr">
+        <is>
+          <t>IWIP DT (Dec)</t>
+        </is>
+      </c>
+      <c r="B51" s="43" t="n">
+        <v>29</v>
+      </c>
+      <c r="C51" s="43" t="n">
+        <v>178</v>
+      </c>
+      <c r="D51" s="43" t="n">
+        <v>28</v>
+      </c>
+      <c r="E51" s="43" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="81" t="inlineStr">
+        <is>
+          <t>December reclaim by stockpile (t/month)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="41" t="inlineStr">
+        <is>
+          <t>Stockpile</t>
+        </is>
+      </c>
+      <c r="B54" s="41" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="C54" s="41" t="inlineStr">
+        <is>
+          <t>3.0.2</t>
+        </is>
+      </c>
+      <c r="D54" s="41" t="inlineStr">
+        <is>
+          <t>3.1.1</t>
+        </is>
+      </c>
+      <c r="E54" s="41" t="inlineStr">
+        <is>
+          <t>3.1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="42" t="inlineStr">
+        <is>
+          <t>POS 12</t>
+        </is>
+      </c>
+      <c r="B55" s="85" t="n">
+        <v>130944</v>
+      </c>
+      <c r="C55" s="85" t="n">
+        <v>130944</v>
+      </c>
+      <c r="D55" s="85" t="n">
+        <v>125116</v>
+      </c>
+      <c r="E55" s="85" t="n">
+        <v>125116</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="42" t="inlineStr">
+        <is>
+          <t>POS 14</t>
+        </is>
+      </c>
+      <c r="B56" s="85" t="n">
+        <v>63364</v>
+      </c>
+      <c r="C56" s="85" t="n">
+        <v>63364</v>
+      </c>
+      <c r="D56" s="85" t="n">
+        <v>63333</v>
+      </c>
+      <c r="E56" s="85" t="n">
+        <v>63333</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="42" t="inlineStr">
+        <is>
+          <t>POS 6</t>
+        </is>
+      </c>
+      <c r="B57" s="86" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C57" s="85" t="n">
+        <v>1282191</v>
+      </c>
+      <c r="D57" s="86" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E57" s="85" t="n">
+        <v>1200692</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2303,7 +2574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2350,6 +2621,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="40" t="inlineStr">
         <is>
@@ -2471,278 +2743,276 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="41" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="87" t="inlineStr">
+        <is>
+          <t>RECLAIMING (IWIP own fleet)</t>
+        </is>
+      </c>
+      <c r="B12" s="88" t="n">
+        <v>29</v>
+      </c>
+      <c r="C12" s="89" t="n"/>
+      <c r="D12" s="89" t="n"/>
+      <c r="E12" s="89" t="n"/>
+      <c r="F12" s="88" t="n">
+        <v>194308</v>
+      </c>
+      <c r="G12" s="90" t="inlineStr">
+        <is>
+          <t>WMT hauled back out of the stockpiles: POS 12 130,944 t · POS 14 63,364 t. Same in all three options — it follows what the plan tips IN, not which option we pick.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="41" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="B13" s="41" t="inlineStr">
+      <c r="B14" s="41" t="inlineStr">
         <is>
           <t>December TARGET t</t>
         </is>
       </c>
-      <c r="C13" s="41" t="inlineStr">
+      <c r="C14" s="41" t="inlineStr">
         <is>
           <t>As frozen</t>
         </is>
       </c>
-      <c r="D13" s="41" t="inlineStr">
+      <c r="D14" s="41" t="inlineStr">
         <is>
           <t>Option 1 (park)</t>
         </is>
       </c>
-      <c r="E13" s="41" t="inlineStr">
+      <c r="E14" s="41" t="inlineStr">
         <is>
           <t>Option 2 (re-dispatch)</t>
         </is>
       </c>
-      <c r="F13" s="41" t="inlineStr"/>
-      <c r="G13" s="41" t="inlineStr">
+      <c r="F14" s="41" t="inlineStr"/>
+      <c r="G14" s="41" t="inlineStr">
         <is>
           <t> </t>
         </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="42" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="B14" s="43" t="n">
-        <v>2311213</v>
-      </c>
-      <c r="C14" s="45" t="n">
-        <v>1.002223075069238</v>
-      </c>
-      <c r="D14" s="45" t="n">
-        <v>1.002223075069238</v>
-      </c>
-      <c r="E14" s="45" t="n">
-        <v>1.109456289835684</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="42" t="inlineStr">
         <is>
-          <t>LIM-TOS</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B15" s="43" t="n">
-        <v>996084</v>
+        <v>2311213</v>
       </c>
       <c r="C15" s="45" t="n">
-        <v>1.003960509354633</v>
+        <v>1.002223075069238</v>
       </c>
       <c r="D15" s="45" t="n">
-        <v>1.003960509354633</v>
+        <v>1.002223075069238</v>
       </c>
       <c r="E15" s="45" t="n">
-        <v>1.003960509354633</v>
+        <v>1.109456289835684</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="42" t="inlineStr">
         <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="B16" s="43" t="n">
+        <v>996084</v>
+      </c>
+      <c r="C16" s="45" t="n">
+        <v>1.003960509354633</v>
+      </c>
+      <c r="D16" s="45" t="n">
+        <v>1.003960509354633</v>
+      </c>
+      <c r="E16" s="45" t="n">
+        <v>1.003960509354633</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="42" t="inlineStr">
+        <is>
           <t>LIM-LD</t>
         </is>
       </c>
-      <c r="B16" s="43" t="n">
+      <c r="B17" s="43" t="n">
         <v>1973655</v>
       </c>
-      <c r="C16" s="45" t="n">
+      <c r="C17" s="45" t="n">
         <v>1.106990836797718</v>
       </c>
-      <c r="D16" s="45" t="n">
+      <c r="D17" s="45" t="n">
         <v>1.000482029580521</v>
       </c>
-      <c r="E16" s="45" t="n">
+      <c r="E17" s="45" t="n">
         <v>1.000482029580521</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="60" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="60" t="inlineStr">
         <is>
           <t>TOTAL t/month</t>
         </is>
       </c>
-      <c r="B17" s="43" t="n">
+      <c r="B18" s="43" t="n">
         <v>5280952</v>
       </c>
-      <c r="C17" s="43" t="n">
+      <c r="C18" s="43" t="n">
         <v>5501198</v>
       </c>
-      <c r="D17" s="79" t="n">
+      <c r="D18" s="79" t="n">
         <v>5290986</v>
       </c>
-      <c r="E17" s="80" t="n">
+      <c r="E18" s="80" t="n">
         <v>5538825</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="81" t="inlineStr">
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="81" t="inlineStr">
         <is>
           <t>Which trucks move (same 65 DT in both options)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="41" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="41" t="inlineStr">
         <is>
           <t>Taken off (LIM-LD)</t>
         </is>
       </c>
-      <c r="B20" s="41" t="inlineStr">
+      <c r="B21" s="41" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="C20" s="41" t="inlineStr">
+      <c r="C21" s="41" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="D20" s="41" t="inlineStr"/>
-      <c r="E20" s="41" t="inlineStr">
+      <c r="D21" s="41" t="inlineStr"/>
+      <c r="E21" s="41" t="inlineStr">
         <is>
           <t>Option 2 sends them to</t>
         </is>
       </c>
-      <c r="F20" s="41" t="inlineStr">
+      <c r="F21" s="41" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="G20" s="41" t="inlineStr">
+      <c r="G21" s="41" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="82" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="82" t="inlineStr">
         <is>
           <t>TF&gt;HUAFEI</t>
         </is>
       </c>
-      <c r="B21" s="82" t="inlineStr">
+      <c r="B22" s="82" t="inlineStr">
         <is>
           <t>RIM</t>
         </is>
       </c>
-      <c r="C21" s="68" t="n">
+      <c r="C22" s="68" t="n">
         <v>65</v>
       </c>
-      <c r="D21" s="66" t="n"/>
-      <c r="E21" s="54" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="F21" s="83" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="G21" s="61" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="66" t="n"/>
-      <c r="B22" s="66" t="n"/>
-      <c r="C22" s="66" t="n"/>
       <c r="D22" s="66" t="n"/>
       <c r="E22" s="54" t="inlineStr">
         <is>
+          <t>KR&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="F22" s="83" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="G22" s="61" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="66" t="n"/>
+      <c r="B23" s="66" t="n"/>
+      <c r="C23" s="66" t="n"/>
+      <c r="D23" s="66" t="n"/>
+      <c r="E23" s="54" t="inlineStr">
+        <is>
           <t>TF&gt;FENI KM0</t>
         </is>
       </c>
-      <c r="F22" s="83" t="inlineStr">
+      <c r="F23" s="83" t="inlineStr">
         <is>
           <t>RIM</t>
         </is>
       </c>
-      <c r="G22" s="61" t="n">
+      <c r="G23" s="61" t="n">
         <v>32</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="40" t="inlineStr">
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="40" t="inlineStr">
         <is>
           <t>Scenario 3.0.2 — December</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="41" t="inlineStr"/>
-      <c r="B26" s="41" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="41" t="inlineStr"/>
+      <c r="B27" s="41" t="inlineStr">
         <is>
           <t>Fleet DT</t>
         </is>
       </c>
-      <c r="C26" s="41" t="inlineStr">
+      <c r="C27" s="41" t="inlineStr">
         <is>
           <t>SAP t/mo</t>
         </is>
       </c>
-      <c r="D26" s="41" t="inlineStr">
+      <c r="D27" s="41" t="inlineStr">
         <is>
           <t>LIM-TOS t/mo</t>
         </is>
       </c>
-      <c r="E26" s="41" t="inlineStr">
+      <c r="E27" s="41" t="inlineStr">
         <is>
           <t>LIM-LD t/mo</t>
         </is>
       </c>
-      <c r="F26" s="41" t="inlineStr">
+      <c r="F27" s="41" t="inlineStr">
         <is>
           <t>TOTAL t/mo</t>
         </is>
       </c>
-      <c r="G26" s="41" t="inlineStr">
+      <c r="G27" s="41" t="inlineStr">
         <is>
           <t>What happens</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="42" t="inlineStr">
-        <is>
-          <t>AS FROZEN</t>
-        </is>
-      </c>
-      <c r="B27" s="47" t="n">
-        <v>1281</v>
-      </c>
-      <c r="C27" s="43" t="n">
-        <v>2316134</v>
-      </c>
-      <c r="D27" s="43" t="n">
-        <v>1001827</v>
-      </c>
-      <c r="E27" s="68" t="n">
-        <v>2370849</v>
-      </c>
-      <c r="F27" s="47" t="n">
-        <v>5688810</v>
-      </c>
-      <c r="G27" s="76" t="inlineStr">
-        <is>
-          <t>LD runs 120% of its 1,973,655 t line — surplus fleet piles onto LD</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="42" t="inlineStr">
         <is>
-          <t>OPTION 1 · park 101 DT</t>
-        </is>
-      </c>
-      <c r="B28" s="52" t="n">
-        <v>1180</v>
+          <t>AS FROZEN</t>
+        </is>
+      </c>
+      <c r="B28" s="47" t="n">
+        <v>1281</v>
       </c>
       <c r="C28" s="43" t="n">
         <v>2316134</v>
@@ -2750,29 +3020,29 @@
       <c r="D28" s="43" t="n">
         <v>1001827</v>
       </c>
-      <c r="E28" s="47" t="n">
-        <v>1974352</v>
-      </c>
-      <c r="F28" s="52" t="n">
-        <v>5292313</v>
-      </c>
-      <c r="G28" s="77" t="inlineStr">
-        <is>
-          <t>LD → 100.0% · 396,497 t NOT hauled · 101 trucks idle</t>
+      <c r="E28" s="68" t="n">
+        <v>2370849</v>
+      </c>
+      <c r="F28" s="47" t="n">
+        <v>5688810</v>
+      </c>
+      <c r="G28" s="76" t="inlineStr">
+        <is>
+          <t>LD runs 120% of its 1,973,655 t line — surplus fleet piles onto LD</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="42" t="inlineStr">
         <is>
-          <t>OPTION 2 · re-dispatch 101 DT</t>
-        </is>
-      </c>
-      <c r="B29" s="61" t="n">
-        <v>1281</v>
-      </c>
-      <c r="C29" s="61" t="n">
-        <v>2701018</v>
+          <t>OPTION 1 · park 101 DT</t>
+        </is>
+      </c>
+      <c r="B29" s="52" t="n">
+        <v>1180</v>
+      </c>
+      <c r="C29" s="43" t="n">
+        <v>2316134</v>
       </c>
       <c r="D29" s="43" t="n">
         <v>1001827</v>
@@ -2780,874 +3050,974 @@
       <c r="E29" s="47" t="n">
         <v>1974352</v>
       </c>
-      <c r="F29" s="61" t="n">
+      <c r="F29" s="52" t="n">
+        <v>5292313</v>
+      </c>
+      <c r="G29" s="77" t="inlineStr">
+        <is>
+          <t>LD → 100.0% · 396,497 t NOT hauled · 101 trucks idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="42" t="inlineStr">
+        <is>
+          <t>OPTION 2 · re-dispatch 101 DT</t>
+        </is>
+      </c>
+      <c r="B30" s="61" t="n">
+        <v>1281</v>
+      </c>
+      <c r="C30" s="61" t="n">
+        <v>2701018</v>
+      </c>
+      <c r="D30" s="43" t="n">
+        <v>1001827</v>
+      </c>
+      <c r="E30" s="47" t="n">
+        <v>1974352</v>
+      </c>
+      <c r="F30" s="61" t="n">
         <v>5677196</v>
       </c>
-      <c r="G29" s="78" t="inlineStr">
+      <c r="G30" s="78" t="inlineStr">
         <is>
           <t>LD → 100.0% · +384,884 t SAP stock at FeNi KM0 · no truck idle</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="41" t="inlineStr">
+      <c r="A31" s="87" t="inlineStr">
+        <is>
+          <t>RECLAIMING (IWIP own fleet)</t>
+        </is>
+      </c>
+      <c r="B31" s="88" t="n">
+        <v>178</v>
+      </c>
+      <c r="C31" s="89" t="n"/>
+      <c r="D31" s="89" t="n"/>
+      <c r="E31" s="89" t="n"/>
+      <c r="F31" s="88" t="n">
+        <v>1476499</v>
+      </c>
+      <c r="G31" s="90" t="inlineStr">
+        <is>
+          <t>WMT hauled back out of the stockpiles: POS 12 130,944 t · POS 14 63,364 t · POS 6 1,282,191 t. Same in all three options — it follows what the plan tips IN, not which option we pick.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="41" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="B31" s="41" t="inlineStr">
+      <c r="B33" s="41" t="inlineStr">
         <is>
           <t>December TARGET t</t>
         </is>
       </c>
-      <c r="C31" s="41" t="inlineStr">
+      <c r="C33" s="41" t="inlineStr">
         <is>
           <t>As frozen</t>
         </is>
       </c>
-      <c r="D31" s="41" t="inlineStr">
+      <c r="D33" s="41" t="inlineStr">
         <is>
           <t>Option 1 (park)</t>
         </is>
       </c>
-      <c r="E31" s="41" t="inlineStr">
+      <c r="E33" s="41" t="inlineStr">
         <is>
           <t>Option 2 (re-dispatch)</t>
         </is>
       </c>
-      <c r="F31" s="41" t="inlineStr"/>
-      <c r="G31" s="41" t="inlineStr">
+      <c r="F33" s="41" t="inlineStr"/>
+      <c r="G33" s="41" t="inlineStr">
         <is>
           <t> </t>
         </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="42" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="B32" s="43" t="n">
-        <v>2311213</v>
-      </c>
-      <c r="C32" s="45" t="n">
-        <v>1.002129184977758</v>
-      </c>
-      <c r="D32" s="45" t="n">
-        <v>1.002129184977758</v>
-      </c>
-      <c r="E32" s="45" t="n">
-        <v>1.168658016374951</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="42" t="inlineStr">
-        <is>
-          <t>LIM-TOS</t>
-        </is>
-      </c>
-      <c r="B33" s="43" t="n">
-        <v>996084</v>
-      </c>
-      <c r="C33" s="45" t="n">
-        <v>1.005765578003462</v>
-      </c>
-      <c r="D33" s="45" t="n">
-        <v>1.005765578003462</v>
-      </c>
-      <c r="E33" s="45" t="n">
-        <v>1.005765578003462</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="42" t="inlineStr">
         <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="B34" s="43" t="n">
+        <v>2311213</v>
+      </c>
+      <c r="C34" s="45" t="n">
+        <v>1.002129184977758</v>
+      </c>
+      <c r="D34" s="45" t="n">
+        <v>1.002129184977758</v>
+      </c>
+      <c r="E34" s="45" t="n">
+        <v>1.168658016374951</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="42" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="B35" s="43" t="n">
+        <v>996084</v>
+      </c>
+      <c r="C35" s="45" t="n">
+        <v>1.005765578003462</v>
+      </c>
+      <c r="D35" s="45" t="n">
+        <v>1.005765578003462</v>
+      </c>
+      <c r="E35" s="45" t="n">
+        <v>1.005765578003462</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="42" t="inlineStr">
+        <is>
           <t>LIM-LD</t>
         </is>
       </c>
-      <c r="B34" s="43" t="n">
+      <c r="B36" s="43" t="n">
         <v>1973655</v>
       </c>
-      <c r="C34" s="45" t="n">
+      <c r="C36" s="45" t="n">
         <v>1.201247938469489</v>
       </c>
-      <c r="D34" s="45" t="n">
+      <c r="D36" s="45" t="n">
         <v>1.000353079511291</v>
       </c>
-      <c r="E34" s="45" t="n">
+      <c r="E36" s="45" t="n">
         <v>1.000353079511291</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="60" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="60" t="inlineStr">
         <is>
           <t>TOTAL t/month</t>
         </is>
       </c>
-      <c r="B35" s="43" t="n">
+      <c r="B37" s="43" t="n">
         <v>5280952</v>
       </c>
-      <c r="C35" s="43" t="n">
+      <c r="C37" s="43" t="n">
         <v>5688810</v>
       </c>
-      <c r="D35" s="79" t="n">
+      <c r="D37" s="79" t="n">
         <v>5292313</v>
       </c>
-      <c r="E35" s="80" t="n">
+      <c r="E37" s="80" t="n">
         <v>5677196</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="81" t="inlineStr">
+    <row r="38"/>
+    <row r="39">
+      <c r="A39" s="81" t="inlineStr">
         <is>
           <t>Which trucks move (same 101 DT in both options)</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="41" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="41" t="inlineStr">
         <is>
           <t>Taken off (LIM-LD)</t>
         </is>
       </c>
-      <c r="B38" s="41" t="inlineStr">
+      <c r="B40" s="41" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="C38" s="41" t="inlineStr">
+      <c r="C40" s="41" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="D38" s="41" t="inlineStr"/>
-      <c r="E38" s="41" t="inlineStr">
+      <c r="D40" s="41" t="inlineStr"/>
+      <c r="E40" s="41" t="inlineStr">
         <is>
           <t>Option 2 sends them to</t>
         </is>
       </c>
-      <c r="F38" s="41" t="inlineStr">
+      <c r="F40" s="41" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="G38" s="41" t="inlineStr">
+      <c r="G40" s="41" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="82" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="82" t="inlineStr">
         <is>
           <t>TF&gt;POS 6</t>
         </is>
       </c>
-      <c r="B39" s="82" t="inlineStr">
+      <c r="B41" s="82" t="inlineStr">
         <is>
           <t>RIM</t>
         </is>
       </c>
-      <c r="C39" s="68" t="n">
+      <c r="C41" s="68" t="n">
         <v>101</v>
       </c>
-      <c r="D39" s="66" t="n"/>
-      <c r="E39" s="54" t="inlineStr">
+      <c r="D41" s="66" t="n"/>
+      <c r="E41" s="54" t="inlineStr">
         <is>
           <t>KR&gt;FENI KM0</t>
         </is>
       </c>
-      <c r="F39" s="83" t="inlineStr">
+      <c r="F41" s="83" t="inlineStr">
         <is>
           <t>RIM</t>
         </is>
       </c>
-      <c r="G39" s="61" t="n">
+      <c r="G41" s="61" t="n">
         <v>51</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="66" t="n"/>
-      <c r="B40" s="66" t="n"/>
-      <c r="C40" s="66" t="n"/>
-      <c r="D40" s="66" t="n"/>
-      <c r="E40" s="54" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="66" t="n"/>
+      <c r="B42" s="66" t="n"/>
+      <c r="C42" s="66" t="n"/>
+      <c r="D42" s="66" t="n"/>
+      <c r="E42" s="54" t="inlineStr">
         <is>
           <t>TF&gt;FENI KM0</t>
         </is>
       </c>
-      <c r="F40" s="83" t="inlineStr">
+      <c r="F42" s="83" t="inlineStr">
         <is>
           <t>RIM</t>
         </is>
       </c>
-      <c r="G40" s="61" t="n">
+      <c r="G42" s="61" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="40" t="inlineStr">
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" s="40" t="inlineStr">
         <is>
           <t>Scenario 3.1.1 — December</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="41" t="inlineStr"/>
-      <c r="B44" s="41" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="41" t="inlineStr"/>
+      <c r="B46" s="41" t="inlineStr">
         <is>
           <t>Fleet DT</t>
         </is>
       </c>
-      <c r="C44" s="41" t="inlineStr">
+      <c r="C46" s="41" t="inlineStr">
         <is>
           <t>SAP t/mo</t>
         </is>
       </c>
-      <c r="D44" s="41" t="inlineStr">
+      <c r="D46" s="41" t="inlineStr">
         <is>
           <t>LIM-TOS t/mo</t>
         </is>
       </c>
-      <c r="E44" s="41" t="inlineStr">
+      <c r="E46" s="41" t="inlineStr">
         <is>
           <t>LIM-LD t/mo</t>
         </is>
       </c>
-      <c r="F44" s="41" t="inlineStr">
+      <c r="F46" s="41" t="inlineStr">
         <is>
           <t>TOTAL t/mo</t>
         </is>
       </c>
-      <c r="G44" s="41" t="inlineStr">
+      <c r="G46" s="41" t="inlineStr">
         <is>
           <t>What happens</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="42" t="inlineStr">
-        <is>
-          <t>AS FROZEN</t>
-        </is>
-      </c>
-      <c r="B45" s="47" t="n">
-        <v>1281</v>
-      </c>
-      <c r="C45" s="43" t="n">
-        <v>2308694</v>
-      </c>
-      <c r="D45" s="43" t="n">
-        <v>1328877</v>
-      </c>
-      <c r="E45" s="68" t="n">
-        <v>2049937</v>
-      </c>
-      <c r="F45" s="47" t="n">
-        <v>5687508</v>
-      </c>
-      <c r="G45" s="76" t="inlineStr">
-        <is>
-          <t>LD runs 121% of its 1,696,393 t line — surplus fleet piles onto LD</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="42" t="inlineStr">
-        <is>
-          <t>OPTION 1 · park 109 DT</t>
-        </is>
-      </c>
-      <c r="B46" s="52" t="n">
-        <v>1172</v>
-      </c>
-      <c r="C46" s="43" t="n">
-        <v>2308694</v>
-      </c>
-      <c r="D46" s="43" t="n">
-        <v>1328877</v>
-      </c>
-      <c r="E46" s="47" t="n">
-        <v>1697274</v>
-      </c>
-      <c r="F46" s="52" t="n">
-        <v>5334845</v>
-      </c>
-      <c r="G46" s="77" t="inlineStr">
-        <is>
-          <t>LD → 100.0% · 352,663 t NOT hauled · 109 trucks idle</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="42" t="inlineStr">
         <is>
-          <t>OPTION 2 · re-dispatch 109 DT</t>
-        </is>
-      </c>
-      <c r="B47" s="61" t="n">
+          <t>AS FROZEN</t>
+        </is>
+      </c>
+      <c r="B47" s="47" t="n">
         <v>1281</v>
       </c>
-      <c r="C47" s="61" t="n">
-        <v>2724032</v>
+      <c r="C47" s="43" t="n">
+        <v>2308694</v>
       </c>
       <c r="D47" s="43" t="n">
         <v>1328877</v>
       </c>
-      <c r="E47" s="47" t="n">
+      <c r="E47" s="68" t="n">
+        <v>2049937</v>
+      </c>
+      <c r="F47" s="47" t="n">
+        <v>5687508</v>
+      </c>
+      <c r="G47" s="76" t="inlineStr">
+        <is>
+          <t>LD runs 121% of its 1,696,393 t line — surplus fleet piles onto LD</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="42" t="inlineStr">
+        <is>
+          <t>OPTION 1 · park 109 DT</t>
+        </is>
+      </c>
+      <c r="B48" s="52" t="n">
+        <v>1172</v>
+      </c>
+      <c r="C48" s="43" t="n">
+        <v>2308694</v>
+      </c>
+      <c r="D48" s="43" t="n">
+        <v>1328877</v>
+      </c>
+      <c r="E48" s="47" t="n">
         <v>1697274</v>
       </c>
-      <c r="F47" s="61" t="n">
+      <c r="F48" s="52" t="n">
+        <v>5334845</v>
+      </c>
+      <c r="G48" s="77" t="inlineStr">
+        <is>
+          <t>LD → 100.0% · 352,663 t NOT hauled · 109 trucks idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="42" t="inlineStr">
+        <is>
+          <t>OPTION 2 · re-dispatch 109 DT</t>
+        </is>
+      </c>
+      <c r="B49" s="61" t="n">
+        <v>1281</v>
+      </c>
+      <c r="C49" s="61" t="n">
+        <v>2724032</v>
+      </c>
+      <c r="D49" s="43" t="n">
+        <v>1328877</v>
+      </c>
+      <c r="E49" s="47" t="n">
+        <v>1697274</v>
+      </c>
+      <c r="F49" s="61" t="n">
         <v>5750183</v>
       </c>
-      <c r="G47" s="78" t="inlineStr">
+      <c r="G49" s="78" t="inlineStr">
         <is>
           <t>LD → 100.0% · +415,338 t SAP stock at FeNi KM0 · no truck idle</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="41" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="87" t="inlineStr">
+        <is>
+          <t>RECLAIMING (IWIP own fleet)</t>
+        </is>
+      </c>
+      <c r="B50" s="88" t="n">
+        <v>28</v>
+      </c>
+      <c r="C50" s="89" t="n"/>
+      <c r="D50" s="89" t="n"/>
+      <c r="E50" s="89" t="n"/>
+      <c r="F50" s="88" t="n">
+        <v>188449</v>
+      </c>
+      <c r="G50" s="90" t="inlineStr">
+        <is>
+          <t>WMT hauled back out of the stockpiles: POS 12 125,116 t · POS 14 63,333 t. Same in all three options — it follows what the plan tips IN, not which option we pick.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51"/>
+    <row r="52">
+      <c r="A52" s="41" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="B49" s="41" t="inlineStr">
+      <c r="B52" s="41" t="inlineStr">
         <is>
           <t>December TARGET t</t>
         </is>
       </c>
-      <c r="C49" s="41" t="inlineStr">
+      <c r="C52" s="41" t="inlineStr">
         <is>
           <t>As frozen</t>
         </is>
       </c>
-      <c r="D49" s="41" t="inlineStr">
+      <c r="D52" s="41" t="inlineStr">
         <is>
           <t>Option 1 (park)</t>
         </is>
       </c>
-      <c r="E49" s="41" t="inlineStr">
+      <c r="E52" s="41" t="inlineStr">
         <is>
           <t>Option 2 (re-dispatch)</t>
         </is>
       </c>
-      <c r="F49" s="41" t="inlineStr"/>
-      <c r="G49" s="41" t="inlineStr">
+      <c r="F52" s="41" t="inlineStr"/>
+      <c r="G52" s="41" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="42" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="42" t="inlineStr">
         <is>
           <t>SAP</t>
         </is>
       </c>
-      <c r="B50" s="43" t="n">
+      <c r="B53" s="43" t="n">
         <v>2311213</v>
       </c>
-      <c r="C50" s="84" t="n">
+      <c r="C53" s="84" t="n">
         <v>0.9989100961270121</v>
       </c>
-      <c r="D50" s="84" t="n">
+      <c r="D53" s="84" t="n">
         <v>0.9989100961270121</v>
       </c>
-      <c r="E50" s="45" t="n">
+      <c r="E53" s="45" t="n">
         <v>1.178615731219927</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="42" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="42" t="inlineStr">
         <is>
           <t>LIM-TOS</t>
         </is>
       </c>
-      <c r="B51" s="43" t="n">
+      <c r="B54" s="43" t="n">
         <v>1326082</v>
       </c>
-      <c r="C51" s="45" t="n">
+      <c r="C54" s="45" t="n">
         <v>1.002107712796041</v>
       </c>
-      <c r="D51" s="45" t="n">
+      <c r="D54" s="45" t="n">
         <v>1.002107712796041</v>
       </c>
-      <c r="E51" s="45" t="n">
+      <c r="E54" s="45" t="n">
         <v>1.002107712796041</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="42" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="42" t="inlineStr">
         <is>
           <t>LIM-LD</t>
         </is>
       </c>
-      <c r="B52" s="43" t="n">
+      <c r="B55" s="43" t="n">
         <v>1696393</v>
       </c>
-      <c r="C52" s="45" t="n">
+      <c r="C55" s="45" t="n">
         <v>1.20840925422352</v>
       </c>
-      <c r="D52" s="45" t="n">
+      <c r="D55" s="45" t="n">
         <v>1.000519511201352</v>
       </c>
-      <c r="E52" s="45" t="n">
+      <c r="E55" s="45" t="n">
         <v>1.000519511201352</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="60" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="60" t="inlineStr">
         <is>
           <t>TOTAL t/month</t>
         </is>
       </c>
-      <c r="B53" s="43" t="n">
+      <c r="B56" s="43" t="n">
         <v>5333688</v>
       </c>
-      <c r="C53" s="43" t="n">
+      <c r="C56" s="43" t="n">
         <v>5687508</v>
       </c>
-      <c r="D53" s="79" t="n">
+      <c r="D56" s="79" t="n">
         <v>5334845</v>
       </c>
-      <c r="E53" s="80" t="n">
+      <c r="E56" s="80" t="n">
         <v>5750183</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="81" t="inlineStr">
+    <row r="57"/>
+    <row r="58">
+      <c r="A58" s="81" t="inlineStr">
         <is>
           <t>Which trucks move (same 109 DT in both options)</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="41" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="41" t="inlineStr">
         <is>
           <t>Taken off (LIM-LD)</t>
         </is>
       </c>
-      <c r="B56" s="41" t="inlineStr">
+      <c r="B59" s="41" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="C56" s="41" t="inlineStr">
+      <c r="C59" s="41" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="D56" s="41" t="inlineStr"/>
-      <c r="E56" s="41" t="inlineStr">
+      <c r="D59" s="41" t="inlineStr"/>
+      <c r="E59" s="41" t="inlineStr">
         <is>
           <t>Option 2 sends them to</t>
         </is>
       </c>
-      <c r="F56" s="41" t="inlineStr">
+      <c r="F59" s="41" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="G56" s="41" t="inlineStr">
+      <c r="G59" s="41" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="82" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="82" t="inlineStr">
         <is>
           <t>TF&gt;HUAFEI</t>
         </is>
       </c>
-      <c r="B57" s="82" t="inlineStr">
+      <c r="B60" s="82" t="inlineStr">
         <is>
           <t>RIM</t>
         </is>
       </c>
-      <c r="C57" s="68" t="n">
+      <c r="C60" s="68" t="n">
         <v>109</v>
       </c>
-      <c r="D57" s="66" t="n"/>
-      <c r="E57" s="54" t="inlineStr">
+      <c r="D60" s="66" t="n"/>
+      <c r="E60" s="54" t="inlineStr">
         <is>
           <t>KR&gt;FENI KM0</t>
         </is>
       </c>
-      <c r="F57" s="83" t="inlineStr">
+      <c r="F60" s="83" t="inlineStr">
         <is>
           <t>RIM</t>
         </is>
       </c>
-      <c r="G57" s="61" t="n">
+      <c r="G60" s="61" t="n">
         <v>55</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="66" t="n"/>
-      <c r="B58" s="66" t="n"/>
-      <c r="C58" s="66" t="n"/>
-      <c r="D58" s="66" t="n"/>
-      <c r="E58" s="54" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="66" t="n"/>
+      <c r="B61" s="66" t="n"/>
+      <c r="C61" s="66" t="n"/>
+      <c r="D61" s="66" t="n"/>
+      <c r="E61" s="54" t="inlineStr">
         <is>
           <t>TF&gt;FENI KM0</t>
         </is>
       </c>
-      <c r="F58" s="83" t="inlineStr">
+      <c r="F61" s="83" t="inlineStr">
         <is>
           <t>RIM</t>
         </is>
       </c>
-      <c r="G58" s="61" t="n">
+      <c r="G61" s="61" t="n">
         <v>54</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="40" t="inlineStr">
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64">
+      <c r="A64" s="40" t="inlineStr">
         <is>
           <t>Scenario 3.1.2 — December</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="41" t="inlineStr"/>
-      <c r="B62" s="41" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="41" t="inlineStr"/>
+      <c r="B65" s="41" t="inlineStr">
         <is>
           <t>Fleet DT</t>
         </is>
       </c>
-      <c r="C62" s="41" t="inlineStr">
+      <c r="C65" s="41" t="inlineStr">
         <is>
           <t>SAP t/mo</t>
         </is>
       </c>
-      <c r="D62" s="41" t="inlineStr">
+      <c r="D65" s="41" t="inlineStr">
         <is>
           <t>LIM-TOS t/mo</t>
         </is>
       </c>
-      <c r="E62" s="41" t="inlineStr">
+      <c r="E65" s="41" t="inlineStr">
         <is>
           <t>LIM-LD t/mo</t>
         </is>
       </c>
-      <c r="F62" s="41" t="inlineStr">
+      <c r="F65" s="41" t="inlineStr">
         <is>
           <t>TOTAL t/mo</t>
         </is>
       </c>
-      <c r="G62" s="41" t="inlineStr">
+      <c r="G65" s="41" t="inlineStr">
         <is>
           <t>What happens</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="42" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="42" t="inlineStr">
         <is>
           <t>AS FROZEN</t>
         </is>
       </c>
-      <c r="B63" s="47" t="n">
+      <c r="B66" s="47" t="n">
         <v>1281</v>
       </c>
-      <c r="C63" s="43" t="n">
+      <c r="C66" s="43" t="n">
         <v>2308694</v>
       </c>
-      <c r="D63" s="43" t="n">
+      <c r="D66" s="43" t="n">
         <v>1330830</v>
       </c>
-      <c r="E63" s="68" t="n">
+      <c r="E66" s="68" t="n">
         <v>2222731</v>
       </c>
-      <c r="F63" s="47" t="n">
+      <c r="F66" s="47" t="n">
         <v>5862255</v>
       </c>
-      <c r="G63" s="76" t="inlineStr">
+      <c r="G66" s="76" t="inlineStr">
         <is>
           <t>LD runs 131% of its 1,696,393 t line — surplus fleet piles onto LD</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="42" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="42" t="inlineStr">
         <is>
           <t>OPTION 1 · park 134 DT</t>
         </is>
       </c>
-      <c r="B64" s="52" t="n">
+      <c r="B67" s="52" t="n">
         <v>1147</v>
       </c>
-      <c r="C64" s="43" t="n">
+      <c r="C67" s="43" t="n">
         <v>2308694</v>
       </c>
-      <c r="D64" s="43" t="n">
+      <c r="D67" s="43" t="n">
         <v>1330830</v>
       </c>
-      <c r="E64" s="47" t="n">
+      <c r="E67" s="47" t="n">
         <v>1696615</v>
       </c>
-      <c r="F64" s="52" t="n">
+      <c r="F67" s="52" t="n">
         <v>5336139</v>
       </c>
-      <c r="G64" s="77" t="inlineStr">
+      <c r="G67" s="77" t="inlineStr">
         <is>
           <t>LD → 100.0% · 526,116 t NOT hauled · 134 trucks idle</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="42" t="inlineStr">
-        <is>
-          <t>OPTION 2 · re-dispatch 134 DT</t>
-        </is>
-      </c>
-      <c r="B65" s="61" t="n">
-        <v>1281</v>
-      </c>
-      <c r="C65" s="61" t="n">
-        <v>2819118</v>
-      </c>
-      <c r="D65" s="43" t="n">
-        <v>1330830</v>
-      </c>
-      <c r="E65" s="47" t="n">
-        <v>1696615</v>
-      </c>
-      <c r="F65" s="61" t="n">
-        <v>5846563</v>
-      </c>
-      <c r="G65" s="78" t="inlineStr">
-        <is>
-          <t>LD → 100.0% · +510,424 t SAP stock at FeNi KM0 · no truck idle</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="41" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B67" s="41" t="inlineStr">
-        <is>
-          <t>December TARGET t</t>
-        </is>
-      </c>
-      <c r="C67" s="41" t="inlineStr">
-        <is>
-          <t>As frozen</t>
-        </is>
-      </c>
-      <c r="D67" s="41" t="inlineStr">
-        <is>
-          <t>Option 1 (park)</t>
-        </is>
-      </c>
-      <c r="E67" s="41" t="inlineStr">
-        <is>
-          <t>Option 2 (re-dispatch)</t>
-        </is>
-      </c>
-      <c r="F67" s="41" t="inlineStr"/>
-      <c r="G67" s="41" t="inlineStr">
-        <is>
-          <t> </t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="42" t="inlineStr">
         <is>
+          <t>OPTION 2 · re-dispatch 134 DT</t>
+        </is>
+      </c>
+      <c r="B68" s="61" t="n">
+        <v>1281</v>
+      </c>
+      <c r="C68" s="61" t="n">
+        <v>2819118</v>
+      </c>
+      <c r="D68" s="43" t="n">
+        <v>1330830</v>
+      </c>
+      <c r="E68" s="47" t="n">
+        <v>1696615</v>
+      </c>
+      <c r="F68" s="61" t="n">
+        <v>5846563</v>
+      </c>
+      <c r="G68" s="78" t="inlineStr">
+        <is>
+          <t>LD → 100.0% · +510,424 t SAP stock at FeNi KM0 · no truck idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="87" t="inlineStr">
+        <is>
+          <t>RECLAIMING (IWIP own fleet)</t>
+        </is>
+      </c>
+      <c r="B69" s="88" t="n">
+        <v>167</v>
+      </c>
+      <c r="C69" s="89" t="n"/>
+      <c r="D69" s="89" t="n"/>
+      <c r="E69" s="89" t="n"/>
+      <c r="F69" s="88" t="n">
+        <v>1389141</v>
+      </c>
+      <c r="G69" s="90" t="inlineStr">
+        <is>
+          <t>WMT hauled back out of the stockpiles: POS 12 125,116 t · POS 14 63,333 t · POS 6 1,200,692 t. Same in all three options — it follows what the plan tips IN, not which option we pick.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70"/>
+    <row r="71">
+      <c r="A71" s="41" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="B71" s="41" t="inlineStr">
+        <is>
+          <t>December TARGET t</t>
+        </is>
+      </c>
+      <c r="C71" s="41" t="inlineStr">
+        <is>
+          <t>As frozen</t>
+        </is>
+      </c>
+      <c r="D71" s="41" t="inlineStr">
+        <is>
+          <t>Option 1 (park)</t>
+        </is>
+      </c>
+      <c r="E71" s="41" t="inlineStr">
+        <is>
+          <t>Option 2 (re-dispatch)</t>
+        </is>
+      </c>
+      <c r="F71" s="41" t="inlineStr"/>
+      <c r="G71" s="41" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="42" t="inlineStr">
+        <is>
           <t>SAP</t>
         </is>
       </c>
-      <c r="B68" s="43" t="n">
+      <c r="B72" s="43" t="n">
         <v>2311213</v>
       </c>
-      <c r="C68" s="84" t="n">
+      <c r="C72" s="84" t="n">
         <v>0.9989100961270121</v>
       </c>
-      <c r="D68" s="84" t="n">
+      <c r="D72" s="84" t="n">
         <v>0.9989100961270121</v>
       </c>
-      <c r="E68" s="45" t="n">
+      <c r="E72" s="45" t="n">
         <v>1.219757028019486</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="42" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="42" t="inlineStr">
         <is>
           <t>LIM-TOS</t>
         </is>
       </c>
-      <c r="B69" s="43" t="n">
+      <c r="B73" s="43" t="n">
         <v>1326082</v>
       </c>
-      <c r="C69" s="45" t="n">
+      <c r="C73" s="45" t="n">
         <v>1.003580472399143</v>
       </c>
-      <c r="D69" s="45" t="n">
+      <c r="D73" s="45" t="n">
         <v>1.003580472399143</v>
       </c>
-      <c r="E69" s="45" t="n">
+      <c r="E73" s="45" t="n">
         <v>1.003580472399143</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="42" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="42" t="inlineStr">
         <is>
           <t>LIM-LD</t>
         </is>
       </c>
-      <c r="B70" s="43" t="n">
+      <c r="B74" s="43" t="n">
         <v>1696393</v>
       </c>
-      <c r="C70" s="45" t="n">
+      <c r="C74" s="45" t="n">
         <v>1.310268905849057</v>
       </c>
-      <c r="D70" s="45" t="n">
+      <c r="D74" s="45" t="n">
         <v>1.000130919236398</v>
       </c>
-      <c r="E70" s="45" t="n">
+      <c r="E74" s="45" t="n">
         <v>1.000130919236398</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="60" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="60" t="inlineStr">
         <is>
           <t>TOTAL t/month</t>
         </is>
       </c>
-      <c r="B71" s="43" t="n">
+      <c r="B75" s="43" t="n">
         <v>5333688</v>
       </c>
-      <c r="C71" s="43" t="n">
+      <c r="C75" s="43" t="n">
         <v>5862255</v>
       </c>
-      <c r="D71" s="79" t="n">
+      <c r="D75" s="79" t="n">
         <v>5336139</v>
       </c>
-      <c r="E71" s="80" t="n">
+      <c r="E75" s="80" t="n">
         <v>5846563</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="81" t="inlineStr">
+    <row r="76"/>
+    <row r="77">
+      <c r="A77" s="81" t="inlineStr">
         <is>
           <t>Which trucks move (same 134 DT in both options)</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="41" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="41" t="inlineStr">
         <is>
           <t>Taken off (LIM-LD)</t>
         </is>
       </c>
-      <c r="B74" s="41" t="inlineStr">
+      <c r="B78" s="41" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="C74" s="41" t="inlineStr">
+      <c r="C78" s="41" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
-      <c r="D74" s="41" t="inlineStr"/>
-      <c r="E74" s="41" t="inlineStr">
+      <c r="D78" s="41" t="inlineStr"/>
+      <c r="E78" s="41" t="inlineStr">
         <is>
           <t>Option 2 sends them to</t>
         </is>
       </c>
-      <c r="F74" s="41" t="inlineStr">
+      <c r="F78" s="41" t="inlineStr">
         <is>
           <t>Contractor</t>
         </is>
       </c>
-      <c r="G74" s="41" t="inlineStr">
+      <c r="G78" s="41" t="inlineStr">
         <is>
           <t>DT</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="82" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="82" t="inlineStr">
         <is>
           <t>TF&gt;POS 6</t>
         </is>
       </c>
-      <c r="B75" s="82" t="inlineStr">
+      <c r="B79" s="82" t="inlineStr">
         <is>
           <t>RIM</t>
         </is>
       </c>
-      <c r="C75" s="68" t="n">
+      <c r="C79" s="68" t="n">
         <v>133</v>
       </c>
-      <c r="D75" s="66" t="n"/>
-      <c r="E75" s="54" t="inlineStr">
+      <c r="D79" s="66" t="n"/>
+      <c r="E79" s="54" t="inlineStr">
         <is>
           <t>KR&gt;FENI KM0</t>
         </is>
       </c>
-      <c r="F75" s="83" t="inlineStr">
+      <c r="F79" s="83" t="inlineStr">
         <is>
           <t>RIM</t>
         </is>
       </c>
-      <c r="G75" s="61" t="n">
+      <c r="G79" s="61" t="n">
         <v>67</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="82" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="82" t="inlineStr">
         <is>
           <t>TF&gt;POS 6</t>
         </is>
       </c>
-      <c r="B76" s="82" t="inlineStr">
+      <c r="B80" s="82" t="inlineStr">
         <is>
           <t>SMA</t>
         </is>
       </c>
-      <c r="C76" s="68" t="n">
+      <c r="C80" s="68" t="n">
         <v>1</v>
       </c>
-      <c r="D76" s="66" t="n"/>
-      <c r="E76" s="54" t="inlineStr">
+      <c r="D80" s="66" t="n"/>
+      <c r="E80" s="54" t="inlineStr">
         <is>
           <t>TF&gt;FENI KM0</t>
         </is>
       </c>
-      <c r="F76" s="83" t="inlineStr">
+      <c r="F80" s="83" t="inlineStr">
         <is>
           <t>RIM</t>
         </is>
       </c>
-      <c r="G76" s="61" t="n">
+      <c r="G80" s="61" t="n">
         <v>66</v>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="66" t="n"/>
-      <c r="B77" s="66" t="n"/>
-      <c r="C77" s="66" t="n"/>
-      <c r="D77" s="66" t="n"/>
-      <c r="E77" s="54" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="66" t="n"/>
+      <c r="B81" s="66" t="n"/>
+      <c r="C81" s="66" t="n"/>
+      <c r="D81" s="66" t="n"/>
+      <c r="E81" s="54" t="inlineStr">
         <is>
           <t>KR&gt;FENI KM0</t>
         </is>
       </c>
-      <c r="F77" s="83" t="inlineStr">
+      <c r="F81" s="83" t="inlineStr">
         <is>
           <t>SMA</t>
         </is>
       </c>
-      <c r="G77" s="61" t="n">
+      <c r="G81" s="61" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjustments sheet: fixed-fleet route-mix analysis, and the POS 6 reclaim correction flows through
Owner set the frame: the DT count must NOT drop (adjustment A rejected),
SAP is fixed per scenario, so the only lever to reach 17 Mt is trip
LENGTH — same trucks, different destinations.

New 'Adjustments' sheet states both adjustments, then measures the
lever: TF>POS 6 yields 121.4 t/DT/day against TF>HUAFEI's 104.8, so one
truck moved buys +16.6 t/day. Per short month it prints the gap, the
truck-shifts needed, the LD trucks actually available on HUAFEI, and a
YES/NO feasibility verdict. Every short month is closable (3.0.1 Oct
needs 501 of 557 available; Nov 468 of 788) — but for 3.0.1/3.1.1 that
means opening a POS 6 leg they do not have, which makes them .2
scenarios. Conclusion: adjustment B IS the split, applied as policy.

Also refreshed on the POS 6>HUAFEI refreeze: year now 16.74 / 17.29 /
17.30 / 17.81 Mt, and December LD gaps (211/396/354/522 kt) size the
Option 1/2 choice.
</commit_message>
<xml_diff>
--- a/reports/scenario_comparison_dec_options.xlsx
+++ b/reports/scenario_comparison_dec_options.xlsx
@@ -8,7 +8,8 @@
   <sheets>
     <sheet name="Compare" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="December options" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Insights" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Adjustments" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Insights" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="167" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="168" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="60">
+  <fonts count="62">
     <font>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -418,8 +419,18 @@
       <color rgb="000F4C81"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00A52929"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001B7A41"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="41">
+  <fills count="42">
     <fill>
       <patternFill/>
     </fill>
@@ -655,6 +666,11 @@
         <fgColor rgb="00EFF3FA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBE9E9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="18">
     <border>
@@ -1016,7 +1032,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1254,6 +1270,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="40" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="55" fillId="40" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="41" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="44" fillId="37" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="37" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2574,7 +2608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2621,7 +2655,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="40" t="inlineStr">
         <is>
@@ -2743,196 +2776,192 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="87" t="inlineStr">
-        <is>
-          <t>RECLAIMING (IWIP own fleet)</t>
-        </is>
-      </c>
-      <c r="B12" s="88" t="n">
-        <v>29</v>
-      </c>
-      <c r="C12" s="89" t="n"/>
-      <c r="D12" s="89" t="n"/>
-      <c r="E12" s="89" t="n"/>
-      <c r="F12" s="88" t="n">
-        <v>194308</v>
-      </c>
-      <c r="G12" s="90" t="inlineStr">
-        <is>
-          <t>WMT hauled back out of the stockpiles: POS 12 130,944 t · POS 14 63,364 t. Same in all three options — it follows what the plan tips IN, not which option we pick.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
+    <row r="13">
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>December TARGET t</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>As frozen</t>
+        </is>
+      </c>
+      <c r="D13" s="41" t="inlineStr">
+        <is>
+          <t>Option 1 (park)</t>
+        </is>
+      </c>
+      <c r="E13" s="41" t="inlineStr">
+        <is>
+          <t>Option 2 (re-dispatch)</t>
+        </is>
+      </c>
+      <c r="F13" s="41" t="inlineStr"/>
+      <c r="G13" s="41" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
     <row r="14">
-      <c r="A14" s="41" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B14" s="41" t="inlineStr">
-        <is>
-          <t>December TARGET t</t>
-        </is>
-      </c>
-      <c r="C14" s="41" t="inlineStr">
-        <is>
-          <t>As frozen</t>
-        </is>
-      </c>
-      <c r="D14" s="41" t="inlineStr">
-        <is>
-          <t>Option 1 (park)</t>
-        </is>
-      </c>
-      <c r="E14" s="41" t="inlineStr">
-        <is>
-          <t>Option 2 (re-dispatch)</t>
-        </is>
-      </c>
-      <c r="F14" s="41" t="inlineStr"/>
-      <c r="G14" s="41" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
+      <c r="A14" s="42" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="B14" s="43" t="n">
+        <v>2311213</v>
+      </c>
+      <c r="C14" s="45" t="n">
+        <v>1.002223075069238</v>
+      </c>
+      <c r="D14" s="45" t="n">
+        <v>1.002223075069238</v>
+      </c>
+      <c r="E14" s="45" t="n">
+        <v>1.109456289835684</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="42" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>LIM-TOS</t>
         </is>
       </c>
       <c r="B15" s="43" t="n">
-        <v>2311213</v>
+        <v>996084</v>
       </c>
       <c r="C15" s="45" t="n">
-        <v>1.002223075069238</v>
+        <v>1.003960509354633</v>
       </c>
       <c r="D15" s="45" t="n">
-        <v>1.002223075069238</v>
+        <v>1.003960509354633</v>
       </c>
       <c r="E15" s="45" t="n">
-        <v>1.109456289835684</v>
+        <v>1.003960509354633</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="42" t="inlineStr">
         <is>
-          <t>LIM-TOS</t>
+          <t>LIM-LD</t>
         </is>
       </c>
       <c r="B16" s="43" t="n">
-        <v>996084</v>
+        <v>1973655</v>
       </c>
       <c r="C16" s="45" t="n">
-        <v>1.003960509354633</v>
+        <v>1.106990836797718</v>
       </c>
       <c r="D16" s="45" t="n">
-        <v>1.003960509354633</v>
+        <v>1.000482029580521</v>
       </c>
       <c r="E16" s="45" t="n">
-        <v>1.003960509354633</v>
+        <v>1.000482029580521</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="42" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
+      <c r="A17" s="60" t="inlineStr">
+        <is>
+          <t>TOTAL t/month</t>
         </is>
       </c>
       <c r="B17" s="43" t="n">
-        <v>1973655</v>
-      </c>
-      <c r="C17" s="45" t="n">
-        <v>1.106990836797718</v>
-      </c>
-      <c r="D17" s="45" t="n">
-        <v>1.000482029580521</v>
-      </c>
-      <c r="E17" s="45" t="n">
-        <v>1.000482029580521</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="60" t="inlineStr">
-        <is>
-          <t>TOTAL t/month</t>
-        </is>
-      </c>
-      <c r="B18" s="43" t="n">
         <v>5280952</v>
       </c>
-      <c r="C18" s="43" t="n">
+      <c r="C17" s="43" t="n">
         <v>5501198</v>
       </c>
-      <c r="D18" s="79" t="n">
+      <c r="D17" s="79" t="n">
         <v>5290986</v>
       </c>
-      <c r="E18" s="80" t="n">
+      <c r="E17" s="80" t="n">
         <v>5538825</v>
       </c>
     </row>
-    <row r="19"/>
+    <row r="19">
+      <c r="A19" s="81" t="inlineStr">
+        <is>
+          <t>Which trucks move (same 65 DT in both options)</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
-      <c r="A20" s="81" t="inlineStr">
-        <is>
-          <t>Which trucks move (same 65 DT in both options)</t>
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>Taken off (LIM-LD)</t>
+        </is>
+      </c>
+      <c r="B20" s="41" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="C20" s="41" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="D20" s="41" t="inlineStr"/>
+      <c r="E20" s="41" t="inlineStr">
+        <is>
+          <t>Option 2 sends them to</t>
+        </is>
+      </c>
+      <c r="F20" s="41" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="G20" s="41" t="inlineStr">
+        <is>
+          <t>DT</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="41" t="inlineStr">
-        <is>
-          <t>Taken off (LIM-LD)</t>
-        </is>
-      </c>
-      <c r="B21" s="41" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="C21" s="41" t="inlineStr">
-        <is>
-          <t>DT</t>
-        </is>
-      </c>
-      <c r="D21" s="41" t="inlineStr"/>
-      <c r="E21" s="41" t="inlineStr">
-        <is>
-          <t>Option 2 sends them to</t>
-        </is>
-      </c>
-      <c r="F21" s="41" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="G21" s="41" t="inlineStr">
-        <is>
-          <t>DT</t>
-        </is>
+      <c r="A21" s="82" t="inlineStr">
+        <is>
+          <t>TF&gt;HUAFEI</t>
+        </is>
+      </c>
+      <c r="B21" s="82" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C21" s="68" t="n">
+        <v>65</v>
+      </c>
+      <c r="D21" s="66" t="n"/>
+      <c r="E21" s="54" t="inlineStr">
+        <is>
+          <t>KR&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="F21" s="83" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="G21" s="61" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="82" t="inlineStr">
-        <is>
-          <t>TF&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B22" s="82" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C22" s="68" t="n">
-        <v>65</v>
-      </c>
+      <c r="A22" s="66" t="n"/>
+      <c r="B22" s="66" t="n"/>
+      <c r="C22" s="66" t="n"/>
       <c r="D22" s="66" t="n"/>
       <c r="E22" s="54" t="inlineStr">
         <is>
-          <t>KR&gt;FENI KM0</t>
+          <t>TF&gt;FENI KM0</t>
         </is>
       </c>
       <c r="F22" s="83" t="inlineStr">
@@ -2941,78 +2970,84 @@
         </is>
       </c>
       <c r="G22" s="61" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="66" t="n"/>
-      <c r="B23" s="66" t="n"/>
-      <c r="C23" s="66" t="n"/>
-      <c r="D23" s="66" t="n"/>
-      <c r="E23" s="54" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="F23" s="83" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="G23" s="61" t="n">
         <v>32</v>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25"/>
+    <row r="25">
+      <c r="A25" s="40" t="inlineStr">
+        <is>
+          <t>Scenario 3.0.2 — December</t>
+        </is>
+      </c>
+    </row>
     <row r="26">
-      <c r="A26" s="40" t="inlineStr">
-        <is>
-          <t>Scenario 3.0.2 — December</t>
+      <c r="A26" s="41" t="inlineStr"/>
+      <c r="B26" s="41" t="inlineStr">
+        <is>
+          <t>Fleet DT</t>
+        </is>
+      </c>
+      <c r="C26" s="41" t="inlineStr">
+        <is>
+          <t>SAP t/mo</t>
+        </is>
+      </c>
+      <c r="D26" s="41" t="inlineStr">
+        <is>
+          <t>LIM-TOS t/mo</t>
+        </is>
+      </c>
+      <c r="E26" s="41" t="inlineStr">
+        <is>
+          <t>LIM-LD t/mo</t>
+        </is>
+      </c>
+      <c r="F26" s="41" t="inlineStr">
+        <is>
+          <t>TOTAL t/mo</t>
+        </is>
+      </c>
+      <c r="G26" s="41" t="inlineStr">
+        <is>
+          <t>What happens</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="41" t="inlineStr"/>
-      <c r="B27" s="41" t="inlineStr">
-        <is>
-          <t>Fleet DT</t>
-        </is>
-      </c>
-      <c r="C27" s="41" t="inlineStr">
-        <is>
-          <t>SAP t/mo</t>
-        </is>
-      </c>
-      <c r="D27" s="41" t="inlineStr">
-        <is>
-          <t>LIM-TOS t/mo</t>
-        </is>
-      </c>
-      <c r="E27" s="41" t="inlineStr">
-        <is>
-          <t>LIM-LD t/mo</t>
-        </is>
-      </c>
-      <c r="F27" s="41" t="inlineStr">
-        <is>
-          <t>TOTAL t/mo</t>
-        </is>
-      </c>
-      <c r="G27" s="41" t="inlineStr">
-        <is>
-          <t>What happens</t>
+      <c r="A27" s="42" t="inlineStr">
+        <is>
+          <t>AS FROZEN</t>
+        </is>
+      </c>
+      <c r="B27" s="47" t="n">
+        <v>1281</v>
+      </c>
+      <c r="C27" s="43" t="n">
+        <v>2316134</v>
+      </c>
+      <c r="D27" s="43" t="n">
+        <v>1001827</v>
+      </c>
+      <c r="E27" s="68" t="n">
+        <v>2370849</v>
+      </c>
+      <c r="F27" s="47" t="n">
+        <v>5688810</v>
+      </c>
+      <c r="G27" s="76" t="inlineStr">
+        <is>
+          <t>LD runs 120% of its 1,973,655 t line — surplus fleet piles onto LD</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="42" t="inlineStr">
         <is>
-          <t>AS FROZEN</t>
-        </is>
-      </c>
-      <c r="B28" s="47" t="n">
-        <v>1281</v>
+          <t>OPTION 1 · park 101 DT</t>
+        </is>
+      </c>
+      <c r="B28" s="52" t="n">
+        <v>1180</v>
       </c>
       <c r="C28" s="43" t="n">
         <v>2316134</v>
@@ -3020,29 +3055,29 @@
       <c r="D28" s="43" t="n">
         <v>1001827</v>
       </c>
-      <c r="E28" s="68" t="n">
-        <v>2370849</v>
-      </c>
-      <c r="F28" s="47" t="n">
-        <v>5688810</v>
-      </c>
-      <c r="G28" s="76" t="inlineStr">
-        <is>
-          <t>LD runs 120% of its 1,973,655 t line — surplus fleet piles onto LD</t>
+      <c r="E28" s="47" t="n">
+        <v>1974352</v>
+      </c>
+      <c r="F28" s="52" t="n">
+        <v>5292313</v>
+      </c>
+      <c r="G28" s="77" t="inlineStr">
+        <is>
+          <t>LD → 100.0% · 396,497 t NOT hauled · 101 trucks idle</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="42" t="inlineStr">
         <is>
-          <t>OPTION 1 · park 101 DT</t>
-        </is>
-      </c>
-      <c r="B29" s="52" t="n">
-        <v>1180</v>
-      </c>
-      <c r="C29" s="43" t="n">
-        <v>2316134</v>
+          <t>OPTION 2 · re-dispatch 101 DT</t>
+        </is>
+      </c>
+      <c r="B29" s="61" t="n">
+        <v>1281</v>
+      </c>
+      <c r="C29" s="61" t="n">
+        <v>2701018</v>
       </c>
       <c r="D29" s="43" t="n">
         <v>1001827</v>
@@ -3050,974 +3085,874 @@
       <c r="E29" s="47" t="n">
         <v>1974352</v>
       </c>
-      <c r="F29" s="52" t="n">
-        <v>5292313</v>
-      </c>
-      <c r="G29" s="77" t="inlineStr">
-        <is>
-          <t>LD → 100.0% · 396,497 t NOT hauled · 101 trucks idle</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="42" t="inlineStr">
-        <is>
-          <t>OPTION 2 · re-dispatch 101 DT</t>
-        </is>
-      </c>
-      <c r="B30" s="61" t="n">
-        <v>1281</v>
-      </c>
-      <c r="C30" s="61" t="n">
-        <v>2701018</v>
-      </c>
-      <c r="D30" s="43" t="n">
-        <v>1001827</v>
-      </c>
-      <c r="E30" s="47" t="n">
-        <v>1974352</v>
-      </c>
-      <c r="F30" s="61" t="n">
+      <c r="F29" s="61" t="n">
         <v>5677196</v>
       </c>
-      <c r="G30" s="78" t="inlineStr">
+      <c r="G29" s="78" t="inlineStr">
         <is>
           <t>LD → 100.0% · +384,884 t SAP stock at FeNi KM0 · no truck idle</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="87" t="inlineStr">
-        <is>
-          <t>RECLAIMING (IWIP own fleet)</t>
-        </is>
-      </c>
-      <c r="B31" s="88" t="n">
-        <v>178</v>
-      </c>
-      <c r="C31" s="89" t="n"/>
-      <c r="D31" s="89" t="n"/>
-      <c r="E31" s="89" t="n"/>
-      <c r="F31" s="88" t="n">
-        <v>1476499</v>
-      </c>
-      <c r="G31" s="90" t="inlineStr">
-        <is>
-          <t>WMT hauled back out of the stockpiles: POS 12 130,944 t · POS 14 63,364 t · POS 6 1,282,191 t. Same in all three options — it follows what the plan tips IN, not which option we pick.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32"/>
+      <c r="A31" s="41" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="B31" s="41" t="inlineStr">
+        <is>
+          <t>December TARGET t</t>
+        </is>
+      </c>
+      <c r="C31" s="41" t="inlineStr">
+        <is>
+          <t>As frozen</t>
+        </is>
+      </c>
+      <c r="D31" s="41" t="inlineStr">
+        <is>
+          <t>Option 1 (park)</t>
+        </is>
+      </c>
+      <c r="E31" s="41" t="inlineStr">
+        <is>
+          <t>Option 2 (re-dispatch)</t>
+        </is>
+      </c>
+      <c r="F31" s="41" t="inlineStr"/>
+      <c r="G31" s="41" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="42" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="B32" s="43" t="n">
+        <v>2311213</v>
+      </c>
+      <c r="C32" s="45" t="n">
+        <v>1.002129184977758</v>
+      </c>
+      <c r="D32" s="45" t="n">
+        <v>1.002129184977758</v>
+      </c>
+      <c r="E32" s="45" t="n">
+        <v>1.168658016374951</v>
+      </c>
+    </row>
     <row r="33">
-      <c r="A33" s="41" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B33" s="41" t="inlineStr">
-        <is>
-          <t>December TARGET t</t>
-        </is>
-      </c>
-      <c r="C33" s="41" t="inlineStr">
-        <is>
-          <t>As frozen</t>
-        </is>
-      </c>
-      <c r="D33" s="41" t="inlineStr">
-        <is>
-          <t>Option 1 (park)</t>
-        </is>
-      </c>
-      <c r="E33" s="41" t="inlineStr">
-        <is>
-          <t>Option 2 (re-dispatch)</t>
-        </is>
-      </c>
-      <c r="F33" s="41" t="inlineStr"/>
-      <c r="G33" s="41" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
+      <c r="A33" s="42" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="B33" s="43" t="n">
+        <v>996084</v>
+      </c>
+      <c r="C33" s="45" t="n">
+        <v>1.005765578003462</v>
+      </c>
+      <c r="D33" s="45" t="n">
+        <v>1.005765578003462</v>
+      </c>
+      <c r="E33" s="45" t="n">
+        <v>1.005765578003462</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="42" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>LIM-LD</t>
         </is>
       </c>
       <c r="B34" s="43" t="n">
-        <v>2311213</v>
+        <v>1973655</v>
       </c>
       <c r="C34" s="45" t="n">
-        <v>1.002129184977758</v>
+        <v>1.201247938469489</v>
       </c>
       <c r="D34" s="45" t="n">
-        <v>1.002129184977758</v>
+        <v>1.000353079511291</v>
       </c>
       <c r="E34" s="45" t="n">
-        <v>1.168658016374951</v>
+        <v>1.000353079511291</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="42" t="inlineStr">
-        <is>
-          <t>LIM-TOS</t>
+      <c r="A35" s="60" t="inlineStr">
+        <is>
+          <t>TOTAL t/month</t>
         </is>
       </c>
       <c r="B35" s="43" t="n">
-        <v>996084</v>
-      </c>
-      <c r="C35" s="45" t="n">
-        <v>1.005765578003462</v>
-      </c>
-      <c r="D35" s="45" t="n">
-        <v>1.005765578003462</v>
-      </c>
-      <c r="E35" s="45" t="n">
-        <v>1.005765578003462</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="42" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="B36" s="43" t="n">
-        <v>1973655</v>
-      </c>
-      <c r="C36" s="45" t="n">
-        <v>1.201247938469489</v>
-      </c>
-      <c r="D36" s="45" t="n">
-        <v>1.000353079511291</v>
-      </c>
-      <c r="E36" s="45" t="n">
-        <v>1.000353079511291</v>
+        <v>5280952</v>
+      </c>
+      <c r="C35" s="43" t="n">
+        <v>5688810</v>
+      </c>
+      <c r="D35" s="79" t="n">
+        <v>5292313</v>
+      </c>
+      <c r="E35" s="80" t="n">
+        <v>5677196</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="60" t="inlineStr">
-        <is>
-          <t>TOTAL t/month</t>
-        </is>
-      </c>
-      <c r="B37" s="43" t="n">
-        <v>5280952</v>
-      </c>
-      <c r="C37" s="43" t="n">
-        <v>5688810</v>
-      </c>
-      <c r="D37" s="79" t="n">
-        <v>5292313</v>
-      </c>
-      <c r="E37" s="80" t="n">
-        <v>5677196</v>
-      </c>
-    </row>
-    <row r="38"/>
+      <c r="A37" s="81" t="inlineStr">
+        <is>
+          <t>Which trucks move (same 101 DT in both options)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="41" t="inlineStr">
+        <is>
+          <t>Taken off (LIM-LD)</t>
+        </is>
+      </c>
+      <c r="B38" s="41" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="C38" s="41" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="D38" s="41" t="inlineStr"/>
+      <c r="E38" s="41" t="inlineStr">
+        <is>
+          <t>Option 2 sends them to</t>
+        </is>
+      </c>
+      <c r="F38" s="41" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="G38" s="41" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+    </row>
     <row r="39">
-      <c r="A39" s="81" t="inlineStr">
-        <is>
-          <t>Which trucks move (same 101 DT in both options)</t>
-        </is>
+      <c r="A39" s="82" t="inlineStr">
+        <is>
+          <t>TF&gt;POS 6</t>
+        </is>
+      </c>
+      <c r="B39" s="82" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C39" s="68" t="n">
+        <v>101</v>
+      </c>
+      <c r="D39" s="66" t="n"/>
+      <c r="E39" s="54" t="inlineStr">
+        <is>
+          <t>KR&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="F39" s="83" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="G39" s="61" t="n">
+        <v>51</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="41" t="inlineStr">
-        <is>
-          <t>Taken off (LIM-LD)</t>
-        </is>
-      </c>
-      <c r="B40" s="41" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="C40" s="41" t="inlineStr">
-        <is>
-          <t>DT</t>
-        </is>
-      </c>
-      <c r="D40" s="41" t="inlineStr"/>
-      <c r="E40" s="41" t="inlineStr">
-        <is>
-          <t>Option 2 sends them to</t>
-        </is>
-      </c>
-      <c r="F40" s="41" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="G40" s="41" t="inlineStr">
-        <is>
-          <t>DT</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="82" t="inlineStr">
-        <is>
-          <t>TF&gt;POS 6</t>
-        </is>
-      </c>
-      <c r="B41" s="82" t="inlineStr">
+      <c r="A40" s="66" t="n"/>
+      <c r="B40" s="66" t="n"/>
+      <c r="C40" s="66" t="n"/>
+      <c r="D40" s="66" t="n"/>
+      <c r="E40" s="54" t="inlineStr">
+        <is>
+          <t>TF&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="F40" s="83" t="inlineStr">
         <is>
           <t>RIM</t>
         </is>
       </c>
-      <c r="C41" s="68" t="n">
-        <v>101</v>
-      </c>
-      <c r="D41" s="66" t="n"/>
-      <c r="E41" s="54" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="F41" s="83" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="G41" s="61" t="n">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="66" t="n"/>
-      <c r="B42" s="66" t="n"/>
-      <c r="C42" s="66" t="n"/>
-      <c r="D42" s="66" t="n"/>
-      <c r="E42" s="54" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="F42" s="83" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="G42" s="61" t="n">
+      <c r="G40" s="61" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="43"/>
-    <row r="44"/>
+    <row r="43">
+      <c r="A43" s="40" t="inlineStr">
+        <is>
+          <t>Scenario 3.1.1 — December</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="41" t="inlineStr"/>
+      <c r="B44" s="41" t="inlineStr">
+        <is>
+          <t>Fleet DT</t>
+        </is>
+      </c>
+      <c r="C44" s="41" t="inlineStr">
+        <is>
+          <t>SAP t/mo</t>
+        </is>
+      </c>
+      <c r="D44" s="41" t="inlineStr">
+        <is>
+          <t>LIM-TOS t/mo</t>
+        </is>
+      </c>
+      <c r="E44" s="41" t="inlineStr">
+        <is>
+          <t>LIM-LD t/mo</t>
+        </is>
+      </c>
+      <c r="F44" s="41" t="inlineStr">
+        <is>
+          <t>TOTAL t/mo</t>
+        </is>
+      </c>
+      <c r="G44" s="41" t="inlineStr">
+        <is>
+          <t>What happens</t>
+        </is>
+      </c>
+    </row>
     <row r="45">
-      <c r="A45" s="40" t="inlineStr">
-        <is>
-          <t>Scenario 3.1.1 — December</t>
+      <c r="A45" s="42" t="inlineStr">
+        <is>
+          <t>AS FROZEN</t>
+        </is>
+      </c>
+      <c r="B45" s="47" t="n">
+        <v>1281</v>
+      </c>
+      <c r="C45" s="43" t="n">
+        <v>2308694</v>
+      </c>
+      <c r="D45" s="43" t="n">
+        <v>1328877</v>
+      </c>
+      <c r="E45" s="68" t="n">
+        <v>2049937</v>
+      </c>
+      <c r="F45" s="47" t="n">
+        <v>5687508</v>
+      </c>
+      <c r="G45" s="76" t="inlineStr">
+        <is>
+          <t>LD runs 121% of its 1,696,393 t line — surplus fleet piles onto LD</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="41" t="inlineStr"/>
-      <c r="B46" s="41" t="inlineStr">
-        <is>
-          <t>Fleet DT</t>
-        </is>
-      </c>
-      <c r="C46" s="41" t="inlineStr">
-        <is>
-          <t>SAP t/mo</t>
-        </is>
-      </c>
-      <c r="D46" s="41" t="inlineStr">
-        <is>
-          <t>LIM-TOS t/mo</t>
-        </is>
-      </c>
-      <c r="E46" s="41" t="inlineStr">
-        <is>
-          <t>LIM-LD t/mo</t>
-        </is>
-      </c>
-      <c r="F46" s="41" t="inlineStr">
-        <is>
-          <t>TOTAL t/mo</t>
-        </is>
-      </c>
-      <c r="G46" s="41" t="inlineStr">
-        <is>
-          <t>What happens</t>
+      <c r="A46" s="42" t="inlineStr">
+        <is>
+          <t>OPTION 1 · park 109 DT</t>
+        </is>
+      </c>
+      <c r="B46" s="52" t="n">
+        <v>1172</v>
+      </c>
+      <c r="C46" s="43" t="n">
+        <v>2308694</v>
+      </c>
+      <c r="D46" s="43" t="n">
+        <v>1328877</v>
+      </c>
+      <c r="E46" s="47" t="n">
+        <v>1697274</v>
+      </c>
+      <c r="F46" s="52" t="n">
+        <v>5334845</v>
+      </c>
+      <c r="G46" s="77" t="inlineStr">
+        <is>
+          <t>LD → 100.0% · 352,663 t NOT hauled · 109 trucks idle</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="42" t="inlineStr">
         <is>
-          <t>AS FROZEN</t>
-        </is>
-      </c>
-      <c r="B47" s="47" t="n">
+          <t>OPTION 2 · re-dispatch 109 DT</t>
+        </is>
+      </c>
+      <c r="B47" s="61" t="n">
         <v>1281</v>
       </c>
-      <c r="C47" s="43" t="n">
-        <v>2308694</v>
+      <c r="C47" s="61" t="n">
+        <v>2724032</v>
       </c>
       <c r="D47" s="43" t="n">
         <v>1328877</v>
       </c>
-      <c r="E47" s="68" t="n">
-        <v>2049937</v>
-      </c>
-      <c r="F47" s="47" t="n">
+      <c r="E47" s="47" t="n">
+        <v>1697274</v>
+      </c>
+      <c r="F47" s="61" t="n">
+        <v>5750183</v>
+      </c>
+      <c r="G47" s="78" t="inlineStr">
+        <is>
+          <t>LD → 100.0% · +415,338 t SAP stock at FeNi KM0 · no truck idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="41" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="B49" s="41" t="inlineStr">
+        <is>
+          <t>December TARGET t</t>
+        </is>
+      </c>
+      <c r="C49" s="41" t="inlineStr">
+        <is>
+          <t>As frozen</t>
+        </is>
+      </c>
+      <c r="D49" s="41" t="inlineStr">
+        <is>
+          <t>Option 1 (park)</t>
+        </is>
+      </c>
+      <c r="E49" s="41" t="inlineStr">
+        <is>
+          <t>Option 2 (re-dispatch)</t>
+        </is>
+      </c>
+      <c r="F49" s="41" t="inlineStr"/>
+      <c r="G49" s="41" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="42" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="B50" s="43" t="n">
+        <v>2311213</v>
+      </c>
+      <c r="C50" s="84" t="n">
+        <v>0.9989100961270121</v>
+      </c>
+      <c r="D50" s="84" t="n">
+        <v>0.9989100961270121</v>
+      </c>
+      <c r="E50" s="45" t="n">
+        <v>1.178615731219927</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="42" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="B51" s="43" t="n">
+        <v>1326082</v>
+      </c>
+      <c r="C51" s="45" t="n">
+        <v>1.002107712796041</v>
+      </c>
+      <c r="D51" s="45" t="n">
+        <v>1.002107712796041</v>
+      </c>
+      <c r="E51" s="45" t="n">
+        <v>1.002107712796041</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="42" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="B52" s="43" t="n">
+        <v>1696393</v>
+      </c>
+      <c r="C52" s="45" t="n">
+        <v>1.20840925422352</v>
+      </c>
+      <c r="D52" s="45" t="n">
+        <v>1.000519511201352</v>
+      </c>
+      <c r="E52" s="45" t="n">
+        <v>1.000519511201352</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="60" t="inlineStr">
+        <is>
+          <t>TOTAL t/month</t>
+        </is>
+      </c>
+      <c r="B53" s="43" t="n">
+        <v>5333688</v>
+      </c>
+      <c r="C53" s="43" t="n">
         <v>5687508</v>
       </c>
-      <c r="G47" s="76" t="inlineStr">
-        <is>
-          <t>LD runs 121% of its 1,696,393 t line — surplus fleet piles onto LD</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="42" t="inlineStr">
-        <is>
-          <t>OPTION 1 · park 109 DT</t>
-        </is>
-      </c>
-      <c r="B48" s="52" t="n">
-        <v>1172</v>
-      </c>
-      <c r="C48" s="43" t="n">
+      <c r="D53" s="79" t="n">
+        <v>5334845</v>
+      </c>
+      <c r="E53" s="80" t="n">
+        <v>5750183</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="81" t="inlineStr">
+        <is>
+          <t>Which trucks move (same 109 DT in both options)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="41" t="inlineStr">
+        <is>
+          <t>Taken off (LIM-LD)</t>
+        </is>
+      </c>
+      <c r="B56" s="41" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="C56" s="41" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="D56" s="41" t="inlineStr"/>
+      <c r="E56" s="41" t="inlineStr">
+        <is>
+          <t>Option 2 sends them to</t>
+        </is>
+      </c>
+      <c r="F56" s="41" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="G56" s="41" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="82" t="inlineStr">
+        <is>
+          <t>TF&gt;HUAFEI</t>
+        </is>
+      </c>
+      <c r="B57" s="82" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C57" s="68" t="n">
+        <v>109</v>
+      </c>
+      <c r="D57" s="66" t="n"/>
+      <c r="E57" s="54" t="inlineStr">
+        <is>
+          <t>KR&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="F57" s="83" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="G57" s="61" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="66" t="n"/>
+      <c r="B58" s="66" t="n"/>
+      <c r="C58" s="66" t="n"/>
+      <c r="D58" s="66" t="n"/>
+      <c r="E58" s="54" t="inlineStr">
+        <is>
+          <t>TF&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="F58" s="83" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="G58" s="61" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="40" t="inlineStr">
+        <is>
+          <t>Scenario 3.1.2 — December</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="41" t="inlineStr"/>
+      <c r="B62" s="41" t="inlineStr">
+        <is>
+          <t>Fleet DT</t>
+        </is>
+      </c>
+      <c r="C62" s="41" t="inlineStr">
+        <is>
+          <t>SAP t/mo</t>
+        </is>
+      </c>
+      <c r="D62" s="41" t="inlineStr">
+        <is>
+          <t>LIM-TOS t/mo</t>
+        </is>
+      </c>
+      <c r="E62" s="41" t="inlineStr">
+        <is>
+          <t>LIM-LD t/mo</t>
+        </is>
+      </c>
+      <c r="F62" s="41" t="inlineStr">
+        <is>
+          <t>TOTAL t/mo</t>
+        </is>
+      </c>
+      <c r="G62" s="41" t="inlineStr">
+        <is>
+          <t>What happens</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="42" t="inlineStr">
+        <is>
+          <t>AS FROZEN</t>
+        </is>
+      </c>
+      <c r="B63" s="47" t="n">
+        <v>1281</v>
+      </c>
+      <c r="C63" s="43" t="n">
         <v>2308694</v>
       </c>
-      <c r="D48" s="43" t="n">
-        <v>1328877</v>
-      </c>
-      <c r="E48" s="47" t="n">
-        <v>1697274</v>
-      </c>
-      <c r="F48" s="52" t="n">
-        <v>5334845</v>
-      </c>
-      <c r="G48" s="77" t="inlineStr">
-        <is>
-          <t>LD → 100.0% · 352,663 t NOT hauled · 109 trucks idle</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="42" t="inlineStr">
-        <is>
-          <t>OPTION 2 · re-dispatch 109 DT</t>
-        </is>
-      </c>
-      <c r="B49" s="61" t="n">
+      <c r="D63" s="43" t="n">
+        <v>1330830</v>
+      </c>
+      <c r="E63" s="68" t="n">
+        <v>2222731</v>
+      </c>
+      <c r="F63" s="47" t="n">
+        <v>5862255</v>
+      </c>
+      <c r="G63" s="76" t="inlineStr">
+        <is>
+          <t>LD runs 131% of its 1,696,393 t line — surplus fleet piles onto LD</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="42" t="inlineStr">
+        <is>
+          <t>OPTION 1 · park 134 DT</t>
+        </is>
+      </c>
+      <c r="B64" s="52" t="n">
+        <v>1147</v>
+      </c>
+      <c r="C64" s="43" t="n">
+        <v>2308694</v>
+      </c>
+      <c r="D64" s="43" t="n">
+        <v>1330830</v>
+      </c>
+      <c r="E64" s="47" t="n">
+        <v>1696615</v>
+      </c>
+      <c r="F64" s="52" t="n">
+        <v>5336139</v>
+      </c>
+      <c r="G64" s="77" t="inlineStr">
+        <is>
+          <t>LD → 100.0% · 526,116 t NOT hauled · 134 trucks idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="42" t="inlineStr">
+        <is>
+          <t>OPTION 2 · re-dispatch 134 DT</t>
+        </is>
+      </c>
+      <c r="B65" s="61" t="n">
         <v>1281</v>
       </c>
-      <c r="C49" s="61" t="n">
-        <v>2724032</v>
-      </c>
-      <c r="D49" s="43" t="n">
-        <v>1328877</v>
-      </c>
-      <c r="E49" s="47" t="n">
-        <v>1697274</v>
-      </c>
-      <c r="F49" s="61" t="n">
-        <v>5750183</v>
-      </c>
-      <c r="G49" s="78" t="inlineStr">
-        <is>
-          <t>LD → 100.0% · +415,338 t SAP stock at FeNi KM0 · no truck idle</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="87" t="inlineStr">
-        <is>
-          <t>RECLAIMING (IWIP own fleet)</t>
-        </is>
-      </c>
-      <c r="B50" s="88" t="n">
-        <v>28</v>
-      </c>
-      <c r="C50" s="89" t="n"/>
-      <c r="D50" s="89" t="n"/>
-      <c r="E50" s="89" t="n"/>
-      <c r="F50" s="88" t="n">
-        <v>188449</v>
-      </c>
-      <c r="G50" s="90" t="inlineStr">
-        <is>
-          <t>WMT hauled back out of the stockpiles: POS 12 125,116 t · POS 14 63,333 t. Same in all three options — it follows what the plan tips IN, not which option we pick.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51"/>
-    <row r="52">
-      <c r="A52" s="41" t="inlineStr">
+      <c r="C65" s="61" t="n">
+        <v>2819118</v>
+      </c>
+      <c r="D65" s="43" t="n">
+        <v>1330830</v>
+      </c>
+      <c r="E65" s="47" t="n">
+        <v>1696615</v>
+      </c>
+      <c r="F65" s="61" t="n">
+        <v>5846563</v>
+      </c>
+      <c r="G65" s="78" t="inlineStr">
+        <is>
+          <t>LD → 100.0% · +510,424 t SAP stock at FeNi KM0 · no truck idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="41" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="B52" s="41" t="inlineStr">
+      <c r="B67" s="41" t="inlineStr">
         <is>
           <t>December TARGET t</t>
         </is>
       </c>
-      <c r="C52" s="41" t="inlineStr">
+      <c r="C67" s="41" t="inlineStr">
         <is>
           <t>As frozen</t>
         </is>
       </c>
-      <c r="D52" s="41" t="inlineStr">
+      <c r="D67" s="41" t="inlineStr">
         <is>
           <t>Option 1 (park)</t>
         </is>
       </c>
-      <c r="E52" s="41" t="inlineStr">
+      <c r="E67" s="41" t="inlineStr">
         <is>
           <t>Option 2 (re-dispatch)</t>
         </is>
       </c>
-      <c r="F52" s="41" t="inlineStr"/>
-      <c r="G52" s="41" t="inlineStr">
+      <c r="F67" s="41" t="inlineStr"/>
+      <c r="G67" s="41" t="inlineStr">
         <is>
           <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="42" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="B53" s="43" t="n">
-        <v>2311213</v>
-      </c>
-      <c r="C53" s="84" t="n">
-        <v>0.9989100961270121</v>
-      </c>
-      <c r="D53" s="84" t="n">
-        <v>0.9989100961270121</v>
-      </c>
-      <c r="E53" s="45" t="n">
-        <v>1.178615731219927</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="42" t="inlineStr">
-        <is>
-          <t>LIM-TOS</t>
-        </is>
-      </c>
-      <c r="B54" s="43" t="n">
-        <v>1326082</v>
-      </c>
-      <c r="C54" s="45" t="n">
-        <v>1.002107712796041</v>
-      </c>
-      <c r="D54" s="45" t="n">
-        <v>1.002107712796041</v>
-      </c>
-      <c r="E54" s="45" t="n">
-        <v>1.002107712796041</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="42" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="B55" s="43" t="n">
-        <v>1696393</v>
-      </c>
-      <c r="C55" s="45" t="n">
-        <v>1.20840925422352</v>
-      </c>
-      <c r="D55" s="45" t="n">
-        <v>1.000519511201352</v>
-      </c>
-      <c r="E55" s="45" t="n">
-        <v>1.000519511201352</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="60" t="inlineStr">
-        <is>
-          <t>TOTAL t/month</t>
-        </is>
-      </c>
-      <c r="B56" s="43" t="n">
-        <v>5333688</v>
-      </c>
-      <c r="C56" s="43" t="n">
-        <v>5687508</v>
-      </c>
-      <c r="D56" s="79" t="n">
-        <v>5334845</v>
-      </c>
-      <c r="E56" s="80" t="n">
-        <v>5750183</v>
-      </c>
-    </row>
-    <row r="57"/>
-    <row r="58">
-      <c r="A58" s="81" t="inlineStr">
-        <is>
-          <t>Which trucks move (same 109 DT in both options)</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="41" t="inlineStr">
-        <is>
-          <t>Taken off (LIM-LD)</t>
-        </is>
-      </c>
-      <c r="B59" s="41" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="C59" s="41" t="inlineStr">
-        <is>
-          <t>DT</t>
-        </is>
-      </c>
-      <c r="D59" s="41" t="inlineStr"/>
-      <c r="E59" s="41" t="inlineStr">
-        <is>
-          <t>Option 2 sends them to</t>
-        </is>
-      </c>
-      <c r="F59" s="41" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="G59" s="41" t="inlineStr">
-        <is>
-          <t>DT</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="82" t="inlineStr">
-        <is>
-          <t>TF&gt;HUAFEI</t>
-        </is>
-      </c>
-      <c r="B60" s="82" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C60" s="68" t="n">
-        <v>109</v>
-      </c>
-      <c r="D60" s="66" t="n"/>
-      <c r="E60" s="54" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="F60" s="83" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="G60" s="61" t="n">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="66" t="n"/>
-      <c r="B61" s="66" t="n"/>
-      <c r="C61" s="66" t="n"/>
-      <c r="D61" s="66" t="n"/>
-      <c r="E61" s="54" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="F61" s="83" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="G61" s="61" t="n">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64">
-      <c r="A64" s="40" t="inlineStr">
-        <is>
-          <t>Scenario 3.1.2 — December</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="41" t="inlineStr"/>
-      <c r="B65" s="41" t="inlineStr">
-        <is>
-          <t>Fleet DT</t>
-        </is>
-      </c>
-      <c r="C65" s="41" t="inlineStr">
-        <is>
-          <t>SAP t/mo</t>
-        </is>
-      </c>
-      <c r="D65" s="41" t="inlineStr">
-        <is>
-          <t>LIM-TOS t/mo</t>
-        </is>
-      </c>
-      <c r="E65" s="41" t="inlineStr">
-        <is>
-          <t>LIM-LD t/mo</t>
-        </is>
-      </c>
-      <c r="F65" s="41" t="inlineStr">
-        <is>
-          <t>TOTAL t/mo</t>
-        </is>
-      </c>
-      <c r="G65" s="41" t="inlineStr">
-        <is>
-          <t>What happens</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="42" t="inlineStr">
-        <is>
-          <t>AS FROZEN</t>
-        </is>
-      </c>
-      <c r="B66" s="47" t="n">
-        <v>1281</v>
-      </c>
-      <c r="C66" s="43" t="n">
-        <v>2308694</v>
-      </c>
-      <c r="D66" s="43" t="n">
-        <v>1330830</v>
-      </c>
-      <c r="E66" s="68" t="n">
-        <v>2222731</v>
-      </c>
-      <c r="F66" s="47" t="n">
-        <v>5862255</v>
-      </c>
-      <c r="G66" s="76" t="inlineStr">
-        <is>
-          <t>LD runs 131% of its 1,696,393 t line — surplus fleet piles onto LD</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="42" t="inlineStr">
-        <is>
-          <t>OPTION 1 · park 134 DT</t>
-        </is>
-      </c>
-      <c r="B67" s="52" t="n">
-        <v>1147</v>
-      </c>
-      <c r="C67" s="43" t="n">
-        <v>2308694</v>
-      </c>
-      <c r="D67" s="43" t="n">
-        <v>1330830</v>
-      </c>
-      <c r="E67" s="47" t="n">
-        <v>1696615</v>
-      </c>
-      <c r="F67" s="52" t="n">
-        <v>5336139</v>
-      </c>
-      <c r="G67" s="77" t="inlineStr">
-        <is>
-          <t>LD → 100.0% · 526,116 t NOT hauled · 134 trucks idle</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="42" t="inlineStr">
         <is>
-          <t>OPTION 2 · re-dispatch 134 DT</t>
-        </is>
-      </c>
-      <c r="B68" s="61" t="n">
-        <v>1281</v>
-      </c>
-      <c r="C68" s="61" t="n">
-        <v>2819118</v>
-      </c>
-      <c r="D68" s="43" t="n">
-        <v>1330830</v>
-      </c>
-      <c r="E68" s="47" t="n">
-        <v>1696615</v>
-      </c>
-      <c r="F68" s="61" t="n">
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="B68" s="43" t="n">
+        <v>2311213</v>
+      </c>
+      <c r="C68" s="84" t="n">
+        <v>0.9989100961270121</v>
+      </c>
+      <c r="D68" s="84" t="n">
+        <v>0.9989100961270121</v>
+      </c>
+      <c r="E68" s="45" t="n">
+        <v>1.219757028019486</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="42" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="B69" s="43" t="n">
+        <v>1326082</v>
+      </c>
+      <c r="C69" s="45" t="n">
+        <v>1.003580472399143</v>
+      </c>
+      <c r="D69" s="45" t="n">
+        <v>1.003580472399143</v>
+      </c>
+      <c r="E69" s="45" t="n">
+        <v>1.003580472399143</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="42" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="B70" s="43" t="n">
+        <v>1696393</v>
+      </c>
+      <c r="C70" s="45" t="n">
+        <v>1.310268905849057</v>
+      </c>
+      <c r="D70" s="45" t="n">
+        <v>1.000130919236398</v>
+      </c>
+      <c r="E70" s="45" t="n">
+        <v>1.000130919236398</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="60" t="inlineStr">
+        <is>
+          <t>TOTAL t/month</t>
+        </is>
+      </c>
+      <c r="B71" s="43" t="n">
+        <v>5333688</v>
+      </c>
+      <c r="C71" s="43" t="n">
+        <v>5862255</v>
+      </c>
+      <c r="D71" s="79" t="n">
+        <v>5336139</v>
+      </c>
+      <c r="E71" s="80" t="n">
         <v>5846563</v>
       </c>
-      <c r="G68" s="78" t="inlineStr">
-        <is>
-          <t>LD → 100.0% · +510,424 t SAP stock at FeNi KM0 · no truck idle</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="87" t="inlineStr">
-        <is>
-          <t>RECLAIMING (IWIP own fleet)</t>
-        </is>
-      </c>
-      <c r="B69" s="88" t="n">
-        <v>167</v>
-      </c>
-      <c r="C69" s="89" t="n"/>
-      <c r="D69" s="89" t="n"/>
-      <c r="E69" s="89" t="n"/>
-      <c r="F69" s="88" t="n">
-        <v>1389141</v>
-      </c>
-      <c r="G69" s="90" t="inlineStr">
-        <is>
-          <t>WMT hauled back out of the stockpiles: POS 12 125,116 t · POS 14 63,333 t · POS 6 1,200,692 t. Same in all three options — it follows what the plan tips IN, not which option we pick.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70"/>
-    <row r="71">
-      <c r="A71" s="41" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B71" s="41" t="inlineStr">
-        <is>
-          <t>December TARGET t</t>
-        </is>
-      </c>
-      <c r="C71" s="41" t="inlineStr">
-        <is>
-          <t>As frozen</t>
-        </is>
-      </c>
-      <c r="D71" s="41" t="inlineStr">
-        <is>
-          <t>Option 1 (park)</t>
-        </is>
-      </c>
-      <c r="E71" s="41" t="inlineStr">
-        <is>
-          <t>Option 2 (re-dispatch)</t>
-        </is>
-      </c>
-      <c r="F71" s="41" t="inlineStr"/>
-      <c r="G71" s="41" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="42" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="B72" s="43" t="n">
-        <v>2311213</v>
-      </c>
-      <c r="C72" s="84" t="n">
-        <v>0.9989100961270121</v>
-      </c>
-      <c r="D72" s="84" t="n">
-        <v>0.9989100961270121</v>
-      </c>
-      <c r="E72" s="45" t="n">
-        <v>1.219757028019486</v>
-      </c>
     </row>
     <row r="73">
-      <c r="A73" s="42" t="inlineStr">
-        <is>
-          <t>LIM-TOS</t>
-        </is>
-      </c>
-      <c r="B73" s="43" t="n">
-        <v>1326082</v>
-      </c>
-      <c r="C73" s="45" t="n">
-        <v>1.003580472399143</v>
-      </c>
-      <c r="D73" s="45" t="n">
-        <v>1.003580472399143</v>
-      </c>
-      <c r="E73" s="45" t="n">
-        <v>1.003580472399143</v>
+      <c r="A73" s="81" t="inlineStr">
+        <is>
+          <t>Which trucks move (same 134 DT in both options)</t>
+        </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="42" t="inlineStr">
-        <is>
-          <t>LIM-LD</t>
-        </is>
-      </c>
-      <c r="B74" s="43" t="n">
-        <v>1696393</v>
-      </c>
-      <c r="C74" s="45" t="n">
-        <v>1.310268905849057</v>
-      </c>
-      <c r="D74" s="45" t="n">
-        <v>1.000130919236398</v>
-      </c>
-      <c r="E74" s="45" t="n">
-        <v>1.000130919236398</v>
+      <c r="A74" s="41" t="inlineStr">
+        <is>
+          <t>Taken off (LIM-LD)</t>
+        </is>
+      </c>
+      <c r="B74" s="41" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="C74" s="41" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="D74" s="41" t="inlineStr"/>
+      <c r="E74" s="41" t="inlineStr">
+        <is>
+          <t>Option 2 sends them to</t>
+        </is>
+      </c>
+      <c r="F74" s="41" t="inlineStr">
+        <is>
+          <t>Contractor</t>
+        </is>
+      </c>
+      <c r="G74" s="41" t="inlineStr">
+        <is>
+          <t>DT</t>
+        </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="60" t="inlineStr">
-        <is>
-          <t>TOTAL t/month</t>
-        </is>
-      </c>
-      <c r="B75" s="43" t="n">
-        <v>5333688</v>
-      </c>
-      <c r="C75" s="43" t="n">
-        <v>5862255</v>
-      </c>
-      <c r="D75" s="79" t="n">
-        <v>5336139</v>
-      </c>
-      <c r="E75" s="80" t="n">
-        <v>5846563</v>
-      </c>
-    </row>
-    <row r="76"/>
+      <c r="A75" s="82" t="inlineStr">
+        <is>
+          <t>TF&gt;POS 6</t>
+        </is>
+      </c>
+      <c r="B75" s="82" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="C75" s="68" t="n">
+        <v>133</v>
+      </c>
+      <c r="D75" s="66" t="n"/>
+      <c r="E75" s="54" t="inlineStr">
+        <is>
+          <t>KR&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="F75" s="83" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="G75" s="61" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="82" t="inlineStr">
+        <is>
+          <t>TF&gt;POS 6</t>
+        </is>
+      </c>
+      <c r="B76" s="82" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="C76" s="68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" s="66" t="n"/>
+      <c r="E76" s="54" t="inlineStr">
+        <is>
+          <t>TF&gt;FENI KM0</t>
+        </is>
+      </c>
+      <c r="F76" s="83" t="inlineStr">
+        <is>
+          <t>RIM</t>
+        </is>
+      </c>
+      <c r="G76" s="61" t="n">
+        <v>66</v>
+      </c>
+    </row>
     <row r="77">
-      <c r="A77" s="81" t="inlineStr">
-        <is>
-          <t>Which trucks move (same 134 DT in both options)</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="41" t="inlineStr">
-        <is>
-          <t>Taken off (LIM-LD)</t>
-        </is>
-      </c>
-      <c r="B78" s="41" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="C78" s="41" t="inlineStr">
-        <is>
-          <t>DT</t>
-        </is>
-      </c>
-      <c r="D78" s="41" t="inlineStr"/>
-      <c r="E78" s="41" t="inlineStr">
-        <is>
-          <t>Option 2 sends them to</t>
-        </is>
-      </c>
-      <c r="F78" s="41" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="G78" s="41" t="inlineStr">
-        <is>
-          <t>DT</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="82" t="inlineStr">
-        <is>
-          <t>TF&gt;POS 6</t>
-        </is>
-      </c>
-      <c r="B79" s="82" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C79" s="68" t="n">
-        <v>133</v>
-      </c>
-      <c r="D79" s="66" t="n"/>
-      <c r="E79" s="54" t="inlineStr">
+      <c r="A77" s="66" t="n"/>
+      <c r="B77" s="66" t="n"/>
+      <c r="C77" s="66" t="n"/>
+      <c r="D77" s="66" t="n"/>
+      <c r="E77" s="54" t="inlineStr">
         <is>
           <t>KR&gt;FENI KM0</t>
         </is>
       </c>
-      <c r="F79" s="83" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="G79" s="61" t="n">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="82" t="inlineStr">
-        <is>
-          <t>TF&gt;POS 6</t>
-        </is>
-      </c>
-      <c r="B80" s="82" t="inlineStr">
+      <c r="F77" s="83" t="inlineStr">
         <is>
           <t>SMA</t>
         </is>
       </c>
-      <c r="C80" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="D80" s="66" t="n"/>
-      <c r="E80" s="54" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="F80" s="83" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="G80" s="61" t="n">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="66" t="n"/>
-      <c r="B81" s="66" t="n"/>
-      <c r="C81" s="66" t="n"/>
-      <c r="D81" s="66" t="n"/>
-      <c r="E81" s="54" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="F81" s="83" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="G81" s="61" t="n">
+      <c r="G77" s="61" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4038,6 +3973,874 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="73" t="inlineStr">
+        <is>
+          <t>Reaching 17 Mt — two kinds of adjustment</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="75" t="inlineStr">
+        <is>
+          <t>THE CONSTRAINTS: the fleet is fixed at 580 / 930 / 1,280 / 1,280 DT (Sep-Dec) and must NOT shrink. SAP cannot exceed its line — it is fixed per scenario. So only LIM-TOS and LIM-LD can move, and only by changing WHERE the trucks drive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="91" t="inlineStr">
+        <is>
+          <t>ADJUSTMENT A — fewer trucks in Nov/Dec: park the DT that push a month over its line. REJECTED by the owner: we do not want the DT number to go down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="92" t="inlineStr">
+        <is>
+          <t>ADJUSTMENT B — same trucks, different trip length: keep every DT working and move them between LD destinations. TF&gt;POS 6 yields 121.4 t/DT/day, TF&gt;HUAFEI 104.8 — so moving one truck from HUAFEI to POS 6 buys +16.6 t/day. This is the only lever left once the fleet and SAP are fixed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="50" t="inlineStr">
+        <is>
+          <t>Where each scenario stands against its lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B8" s="41" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="C8" s="41" t="inlineStr">
+        <is>
+          <t>Fleet DT</t>
+        </is>
+      </c>
+      <c r="D8" s="41" t="inlineStr">
+        <is>
+          <t>LIM-LD predicted</t>
+        </is>
+      </c>
+      <c r="E8" s="41" t="inlineStr">
+        <is>
+          <t>LIM-LD target</t>
+        </is>
+      </c>
+      <c r="F8" s="41" t="inlineStr">
+        <is>
+          <t>LD gap t</t>
+        </is>
+      </c>
+      <c r="G8" s="41" t="inlineStr">
+        <is>
+          <t>Month gap t</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="42" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="B9" s="42" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="C9" s="43" t="n">
+        <v>581</v>
+      </c>
+      <c r="D9" s="43" t="n">
+        <v>851940</v>
+      </c>
+      <c r="E9" s="43" t="n">
+        <v>890366</v>
+      </c>
+      <c r="F9" s="93" t="n">
+        <v>-38426</v>
+      </c>
+      <c r="G9" s="52" t="n">
+        <v>-50907</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="42" t="inlineStr"/>
+      <c r="B10" s="42" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="C10" s="43" t="n">
+        <v>931</v>
+      </c>
+      <c r="D10" s="43" t="n">
+        <v>1814864</v>
+      </c>
+      <c r="E10" s="43" t="n">
+        <v>2072629</v>
+      </c>
+      <c r="F10" s="93" t="n">
+        <v>-257765</v>
+      </c>
+      <c r="G10" s="52" t="n">
+        <v>-202025</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="42" t="inlineStr"/>
+      <c r="B11" s="42" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="C11" s="43" t="n">
+        <v>1280</v>
+      </c>
+      <c r="D11" s="43" t="n">
+        <v>2464530</v>
+      </c>
+      <c r="E11" s="43" t="n">
+        <v>2697656</v>
+      </c>
+      <c r="F11" s="93" t="n">
+        <v>-233126</v>
+      </c>
+      <c r="G11" s="52" t="n">
+        <v>-172448</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="42" t="inlineStr"/>
+      <c r="B12" s="42" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="C12" s="43" t="n">
+        <v>1281</v>
+      </c>
+      <c r="D12" s="43" t="n">
+        <v>2184849</v>
+      </c>
+      <c r="E12" s="43" t="n">
+        <v>1973655</v>
+      </c>
+      <c r="F12" s="94" t="n">
+        <v>211194</v>
+      </c>
+      <c r="G12" s="61" t="n">
+        <v>160195</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="60" t="inlineStr">
+        <is>
+          <t>3.0.1 YEAR</t>
+        </is>
+      </c>
+      <c r="B13" s="42" t="inlineStr">
+        <is>
+          <t>Sep–Dec</t>
+        </is>
+      </c>
+      <c r="D13" s="43" t="n">
+        <v>16738008</v>
+      </c>
+      <c r="E13" s="43" t="n">
+        <v>17003193</v>
+      </c>
+      <c r="G13" s="93" t="n">
+        <v>-265185</v>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="42" t="inlineStr">
+        <is>
+          <t>3.0.2</t>
+        </is>
+      </c>
+      <c r="B15" s="42" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="C15" s="43" t="n">
+        <v>581</v>
+      </c>
+      <c r="D15" s="43" t="n">
+        <v>851940</v>
+      </c>
+      <c r="E15" s="43" t="n">
+        <v>890366</v>
+      </c>
+      <c r="F15" s="93" t="n">
+        <v>-38426</v>
+      </c>
+      <c r="G15" s="52" t="n">
+        <v>-50907</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="42" t="inlineStr"/>
+      <c r="B16" s="42" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="C16" s="43" t="n">
+        <v>931</v>
+      </c>
+      <c r="D16" s="43" t="n">
+        <v>1965741</v>
+      </c>
+      <c r="E16" s="43" t="n">
+        <v>2072629</v>
+      </c>
+      <c r="F16" s="93" t="n">
+        <v>-106888</v>
+      </c>
+      <c r="G16" s="52" t="n">
+        <v>-48812</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="42" t="inlineStr"/>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="C17" s="43" t="n">
+        <v>1280</v>
+      </c>
+      <c r="D17" s="43" t="n">
+        <v>2672880</v>
+      </c>
+      <c r="E17" s="43" t="n">
+        <v>2697656</v>
+      </c>
+      <c r="F17" s="93" t="n">
+        <v>-24776</v>
+      </c>
+      <c r="G17" s="61" t="n">
+        <v>37007</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="42" t="inlineStr"/>
+      <c r="B18" s="42" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="C18" s="43" t="n">
+        <v>1281</v>
+      </c>
+      <c r="D18" s="43" t="n">
+        <v>2369919</v>
+      </c>
+      <c r="E18" s="43" t="n">
+        <v>1973655</v>
+      </c>
+      <c r="F18" s="94" t="n">
+        <v>396264</v>
+      </c>
+      <c r="G18" s="61" t="n">
+        <v>346837</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="60" t="inlineStr">
+        <is>
+          <t>3.0.2 YEAR</t>
+        </is>
+      </c>
+      <c r="B19" s="42" t="inlineStr">
+        <is>
+          <t>Sep–Dec</t>
+        </is>
+      </c>
+      <c r="D19" s="43" t="n">
+        <v>17287318</v>
+      </c>
+      <c r="E19" s="43" t="n">
+        <v>17003193</v>
+      </c>
+      <c r="G19" s="94" t="n">
+        <v>284125</v>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="42" t="inlineStr">
+        <is>
+          <t>3.1.1</t>
+        </is>
+      </c>
+      <c r="B21" s="42" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="C21" s="43" t="n">
+        <v>581</v>
+      </c>
+      <c r="D21" s="43" t="n">
+        <v>851940</v>
+      </c>
+      <c r="E21" s="43" t="n">
+        <v>840444</v>
+      </c>
+      <c r="F21" s="94" t="n">
+        <v>11496</v>
+      </c>
+      <c r="G21" s="61" t="n">
+        <v>20112</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="42" t="inlineStr"/>
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="C22" s="43" t="n">
+        <v>931</v>
+      </c>
+      <c r="D22" s="43" t="n">
+        <v>1675736</v>
+      </c>
+      <c r="E22" s="43" t="n">
+        <v>1786681</v>
+      </c>
+      <c r="F22" s="93" t="n">
+        <v>-110945</v>
+      </c>
+      <c r="G22" s="52" t="n">
+        <v>-78928</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="42" t="inlineStr"/>
+      <c r="B23" s="42" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="C23" s="43" t="n">
+        <v>1280</v>
+      </c>
+      <c r="D23" s="43" t="n">
+        <v>2324910</v>
+      </c>
+      <c r="E23" s="43" t="n">
+        <v>2320788</v>
+      </c>
+      <c r="F23" s="94" t="n">
+        <v>4122</v>
+      </c>
+      <c r="G23" s="61" t="n">
+        <v>34487</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="42" t="inlineStr"/>
+      <c r="B24" s="42" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="C24" s="43" t="n">
+        <v>1281</v>
+      </c>
+      <c r="D24" s="43" t="n">
+        <v>2049937</v>
+      </c>
+      <c r="E24" s="43" t="n">
+        <v>1696393</v>
+      </c>
+      <c r="F24" s="94" t="n">
+        <v>353544</v>
+      </c>
+      <c r="G24" s="61" t="n">
+        <v>317465</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="60" t="inlineStr">
+        <is>
+          <t>3.1.1 YEAR</t>
+        </is>
+      </c>
+      <c r="B25" s="42" t="inlineStr">
+        <is>
+          <t>Sep–Dec</t>
+        </is>
+      </c>
+      <c r="D25" s="43" t="n">
+        <v>17296329</v>
+      </c>
+      <c r="E25" s="43" t="n">
+        <v>17003193</v>
+      </c>
+      <c r="G25" s="94" t="n">
+        <v>293136</v>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="42" t="inlineStr">
+        <is>
+          <t>3.1.2</t>
+        </is>
+      </c>
+      <c r="B27" s="42" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="C27" s="43" t="n">
+        <v>581</v>
+      </c>
+      <c r="D27" s="43" t="n">
+        <v>851940</v>
+      </c>
+      <c r="E27" s="43" t="n">
+        <v>840444</v>
+      </c>
+      <c r="F27" s="94" t="n">
+        <v>11496</v>
+      </c>
+      <c r="G27" s="61" t="n">
+        <v>20112</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="42" t="inlineStr"/>
+      <c r="B28" s="42" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="C28" s="43" t="n">
+        <v>931</v>
+      </c>
+      <c r="D28" s="43" t="n">
+        <v>1808447</v>
+      </c>
+      <c r="E28" s="43" t="n">
+        <v>1786681</v>
+      </c>
+      <c r="F28" s="94" t="n">
+        <v>21766</v>
+      </c>
+      <c r="G28" s="61" t="n">
+        <v>59284</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="42" t="inlineStr"/>
+      <c r="B29" s="42" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="C29" s="43" t="n">
+        <v>1280</v>
+      </c>
+      <c r="D29" s="43" t="n">
+        <v>2520240</v>
+      </c>
+      <c r="E29" s="43" t="n">
+        <v>2320788</v>
+      </c>
+      <c r="F29" s="94" t="n">
+        <v>199452</v>
+      </c>
+      <c r="G29" s="61" t="n">
+        <v>237094</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="42" t="inlineStr"/>
+      <c r="B30" s="42" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="C30" s="43" t="n">
+        <v>1281</v>
+      </c>
+      <c r="D30" s="43" t="n">
+        <v>2218732</v>
+      </c>
+      <c r="E30" s="43" t="n">
+        <v>1696393</v>
+      </c>
+      <c r="F30" s="94" t="n">
+        <v>522339</v>
+      </c>
+      <c r="G30" s="61" t="n">
+        <v>491883</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="60" t="inlineStr">
+        <is>
+          <t>3.1.2 YEAR</t>
+        </is>
+      </c>
+      <c r="B31" s="42" t="inlineStr">
+        <is>
+          <t>Sep–Dec</t>
+        </is>
+      </c>
+      <c r="D31" s="43" t="n">
+        <v>17811566</v>
+      </c>
+      <c r="E31" s="43" t="n">
+        <v>17003193</v>
+      </c>
+      <c r="G31" s="94" t="n">
+        <v>808373</v>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="50" t="inlineStr">
+        <is>
+          <t>ADJUSTMENT B — how far the trip-length lever actually reaches</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="49" t="inlineStr">
+        <is>
+          <t>For each SHORT month: how many LD trucks would have to move from TF&gt;HUAFEI to TF&gt;POS 6 to close the gap, and how many LD trucks that month actually has. If the shift needed exceeds the fleet on the route, the gap cannot be closed by route mix alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="41" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B35" s="41" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="C35" s="41" t="inlineStr">
+        <is>
+          <t>Gap to close t</t>
+        </is>
+      </c>
+      <c r="D35" s="41" t="inlineStr">
+        <is>
+          <t>DT to shift HUAFEI→POS 6</t>
+        </is>
+      </c>
+      <c r="E35" s="41" t="inlineStr">
+        <is>
+          <t>LD DT available</t>
+        </is>
+      </c>
+      <c r="F35" s="41" t="inlineStr">
+        <is>
+          <t>Feasible?</t>
+        </is>
+      </c>
+      <c r="G35" s="41" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="42" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="B36" s="42" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="C36" s="43" t="n">
+        <v>38426</v>
+      </c>
+      <c r="D36" s="59" t="n">
+        <v>77</v>
+      </c>
+      <c r="E36" s="43" t="n">
+        <v>268</v>
+      </c>
+      <c r="F36" s="95" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G36" s="76" t="inlineStr">
+        <is>
+          <t>shift 77 of 268 LD trucks to the longer POS 6 haul</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="42" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="B37" s="42" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="C37" s="43" t="n">
+        <v>257765</v>
+      </c>
+      <c r="D37" s="59" t="n">
+        <v>501</v>
+      </c>
+      <c r="E37" s="43" t="n">
+        <v>557</v>
+      </c>
+      <c r="F37" s="95" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G37" s="76" t="inlineStr">
+        <is>
+          <t>shift 501 of 557 LD trucks to the longer POS 6 haul</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="42" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="B38" s="42" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="C38" s="43" t="n">
+        <v>233126</v>
+      </c>
+      <c r="D38" s="59" t="n">
+        <v>468</v>
+      </c>
+      <c r="E38" s="43" t="n">
+        <v>788</v>
+      </c>
+      <c r="F38" s="95" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G38" s="76" t="inlineStr">
+        <is>
+          <t>shift 468 of 788 LD trucks to the longer POS 6 haul</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="42" t="inlineStr">
+        <is>
+          <t>3.0.2</t>
+        </is>
+      </c>
+      <c r="B39" s="42" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="C39" s="43" t="n">
+        <v>38426</v>
+      </c>
+      <c r="D39" s="59" t="n">
+        <v>77</v>
+      </c>
+      <c r="E39" s="43" t="n">
+        <v>268</v>
+      </c>
+      <c r="F39" s="95" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G39" s="76" t="inlineStr">
+        <is>
+          <t>shift 77 of 268 LD trucks to the longer POS 6 haul</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="42" t="inlineStr">
+        <is>
+          <t>3.0.2</t>
+        </is>
+      </c>
+      <c r="B40" s="42" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="C40" s="43" t="n">
+        <v>106888</v>
+      </c>
+      <c r="D40" s="59" t="n">
+        <v>208</v>
+      </c>
+      <c r="E40" s="43" t="n">
+        <v>278</v>
+      </c>
+      <c r="F40" s="95" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G40" s="76" t="inlineStr">
+        <is>
+          <t>shift 208 of 278 LD trucks to the longer POS 6 haul</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="42" t="inlineStr">
+        <is>
+          <t>3.0.2</t>
+        </is>
+      </c>
+      <c r="B41" s="42" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="C41" s="43" t="n">
+        <v>24776</v>
+      </c>
+      <c r="D41" s="59" t="n">
+        <v>50</v>
+      </c>
+      <c r="E41" s="43" t="n">
+        <v>394</v>
+      </c>
+      <c r="F41" s="95" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G41" s="76" t="inlineStr">
+        <is>
+          <t>shift 50 of 394 LD trucks to the longer POS 6 haul</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="42" t="inlineStr">
+        <is>
+          <t>3.1.1</t>
+        </is>
+      </c>
+      <c r="B42" s="42" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="C42" s="43" t="n">
+        <v>110945</v>
+      </c>
+      <c r="D42" s="59" t="n">
+        <v>216</v>
+      </c>
+      <c r="E42" s="43" t="n">
+        <v>514</v>
+      </c>
+      <c r="F42" s="95" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G42" s="76" t="inlineStr">
+        <is>
+          <t>shift 216 of 514 LD trucks to the longer POS 6 haul</t>
+        </is>
+      </c>
+    </row>
+    <row r="43"/>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="96" t="inlineStr">
+        <is>
+          <t>READING: every short month CAN be closed by route mix — the shift needed is always smaller than the LD fleet on HUAFEI that month (3.0.1 Oct needs 501 of 557; Nov 468 of 788). But in 3.0.1 and 3.1.1 that means opening a POS 6 leg those scenarios do not have by definition, which turns them into .2 scenarios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="26" customHeight="1">
+      <c r="A45" s="96" t="inlineStr">
+        <is>
+          <t>The .2 scenarios already run the split, which is why they clear the line (+284 kt and +808 kt) with only small October/November gaps left. 3.0.1 is the only scenario that stays short overall (-265 kt).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="26" customHeight="1">
+      <c r="A46" s="96" t="inlineStr">
+        <is>
+          <t>CONCLUSION: adjustment B is feasible and needs no extra trucks — but it IS the POS 6 split. Choosing a .2 scenario applies the same lever as policy instead of month by month, and lands 17.29-17.81 Mt with the fleet untouched at 580/930/1,280/1,281 DT. December still finishes over its LD line, which is what Options 1 and 2 are for.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A44:G44"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A46:G46"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Comparison workbook: Fleet levelling sheet replaces the old adjustment sheet
The side workbook still carried the pre-levelling numbers. Its middle
sheet is now 'Fleet levelling': a summary row per scenario (fleet to
own, Nov run, Dec run, DT parked, LIM-LD year before and after, Together
year), then a per-scenario block with Fleet available / PARKED / RUNNING
by month and the Sep-Dec year result.

  3.0.1  no change      (LIM-LD year 95.8%, under its line)
  3.0.2  own 1,244 DT   park 73   year 100.3%
  3.1.1  own 1,239 DT   park 83   year 100.2%
  3.1.2  own 1,161 DT   park 239  year 100.3%
Workbook is Compare / Fleet levelling / Insights.
</commit_message>
<xml_diff>
--- a/reports/scenario_comparison_dec_options.xlsx
+++ b/reports/scenario_comparison_dec_options.xlsx
@@ -7,7 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Compare" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Year adjustment" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fleet levelling" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Insights" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -22,7 +22,7 @@
     <numFmt numFmtId="165" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="166" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="58">
+  <fonts count="59">
     <font>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -406,6 +406,12 @@
       <b val="1"/>
       <color rgb="000F4C81"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001B7A41"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="43">
@@ -940,7 +946,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1151,6 +1157,13 @@
     <xf numFmtId="3" fontId="47" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="45" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="49" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2468,276 +2481,296 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>Bringing the YEAR to 100% — how many trucks we do not need</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="40" customHeight="1">
+          <t>Fleet levelling — one running level all year</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
       <c r="A3" s="40" t="inlineStr">
         <is>
-          <t>THE TARGET IS THE YEAR, not each month. SAP and LIM-TOS already land on their year lines; LIM-LD is the one running over (3.0.2 103.0%, 3.1.1 103.9%, 3.1.2 111.4%). We remove only enough LIM-LD to bring the YEAR to 100%, so a single month may still sit above its own line — that is fine, and it is why far fewer trucks are freed than a month-by-month fix would demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="40" customHeight="1">
+          <t>The fleet grows through the year (581 · 931 · 1,280 · 1,281 DT). Running every truck flat out overshoots the LIM-LD year line, so some must stand down. Parking a different number each month would force them to BUY for the peak and leave those trucks idle a month later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="40" t="inlineStr">
         <is>
-          <t>RULES STILL HOLD IN EVERY MONTH: no month is pushed BELOW its own line, a truck never changes contractor, RIM works BLB and TF only and SMA works KR and TF only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="40" t="inlineStr">
-        <is>
-          <t>THE FREED TRUCKS ARE OPTIONAL CAPACITY. First we try to keep them working by moving SAP onto LONGER hauls (KM15 to KM0, POS 12 to KM0) — the same tonnage over a longer distance needs more trucks. Only what no haul can take is reported as trucks we simply do not need.</t>
+          <t>Instead we hold ONE running level all year: the highest level every month can keep while the YEAR still lands on its line. That level is the fleet they actually need to own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="44" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B6" s="44" t="inlineStr">
+        <is>
+          <t>FLEET TO OWN</t>
+        </is>
+      </c>
+      <c r="C6" s="44" t="inlineStr">
+        <is>
+          <t>Nov run</t>
+        </is>
+      </c>
+      <c r="D6" s="44" t="inlineStr">
+        <is>
+          <t>Dec run</t>
+        </is>
+      </c>
+      <c r="E6" s="44" t="inlineStr">
+        <is>
+          <t>DT parked</t>
+        </is>
+      </c>
+      <c r="F6" s="44" t="inlineStr">
+        <is>
+          <t>LIM-LD year was</t>
+        </is>
+      </c>
+      <c r="G6" s="44" t="inlineStr">
+        <is>
+          <t>LIM-LD year now</t>
+        </is>
+      </c>
+      <c r="H6" s="44" t="inlineStr">
+        <is>
+          <t>Together year</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="41" t="inlineStr">
-        <is>
-          <t>THE ANSWER — trucks not needed, per scenario</t>
-        </is>
+      <c r="A7" s="67" t="inlineStr">
+        <is>
+          <t>3.0.1</t>
+        </is>
+      </c>
+      <c r="B7" s="56" t="inlineStr">
+        <is>
+          <t>no change</t>
+        </is>
+      </c>
+      <c r="C7" s="46" t="n">
+        <v>1280</v>
+      </c>
+      <c r="D7" s="46" t="n">
+        <v>1281</v>
+      </c>
+      <c r="E7" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="80" t="n">
+        <v>0.9583298075817238</v>
+      </c>
+      <c r="G7" s="50" t="n">
+        <v>0.9583298075817238</v>
+      </c>
+      <c r="H7" s="50" t="n">
+        <v>0.9844039283917985</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="44" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="B8" s="44" t="inlineStr">
-        <is>
-          <t>LIM-LD year now</t>
-        </is>
-      </c>
-      <c r="C8" s="44" t="inlineStr">
-        <is>
-          <t>Year line</t>
-        </is>
-      </c>
-      <c r="D8" s="44" t="inlineStr">
-        <is>
-          <t>Now %</t>
-        </is>
-      </c>
-      <c r="E8" s="44" t="inlineStr">
-        <is>
-          <t>Trucks freed</t>
-        </is>
-      </c>
-      <c r="F8" s="44" t="inlineStr">
-        <is>
-          <t>Kept working (longer hauls)</t>
-        </is>
-      </c>
-      <c r="G8" s="44" t="inlineStr">
-        <is>
-          <t>NOT NEEDED</t>
-        </is>
-      </c>
-      <c r="H8" s="44" t="inlineStr">
-        <is>
-          <t>Year LD after</t>
-        </is>
+      <c r="A8" s="67" t="inlineStr">
+        <is>
+          <t>3.0.2</t>
+        </is>
+      </c>
+      <c r="B8" s="58" t="n">
+        <v>1244</v>
+      </c>
+      <c r="C8" s="46" t="n">
+        <v>1244</v>
+      </c>
+      <c r="D8" s="46" t="n">
+        <v>1244</v>
+      </c>
+      <c r="E8" s="79" t="n">
+        <v>73</v>
+      </c>
+      <c r="F8" s="81" t="n">
+        <v>1.029626006607542</v>
+      </c>
+      <c r="G8" s="50" t="n">
+        <v>0.9994156617947111</v>
+      </c>
+      <c r="H8" s="50" t="n">
+        <v>1.00314440861065</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="67" t="inlineStr">
         <is>
-          <t>3.0.1</t>
-        </is>
-      </c>
-      <c r="B9" s="46" t="n">
-        <v>7316183</v>
+          <t>3.1.1</t>
+        </is>
+      </c>
+      <c r="B9" s="58" t="n">
+        <v>1239</v>
       </c>
       <c r="C9" s="46" t="n">
-        <v>7634306</v>
-      </c>
-      <c r="D9" s="68" t="n">
-        <v>0.9583298075817238</v>
-      </c>
-      <c r="E9" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="58" t="n">
-        <v>0</v>
+        <v>1239</v>
+      </c>
+      <c r="D9" s="46" t="n">
+        <v>1239</v>
+      </c>
+      <c r="E9" s="79" t="n">
+        <v>83</v>
+      </c>
+      <c r="F9" s="81" t="n">
+        <v>1.038862900053068</v>
+      </c>
+      <c r="G9" s="50" t="n">
+        <v>0.9991867558336038</v>
       </c>
       <c r="H9" s="50" t="n">
-        <v>0.9583298075817238</v>
+        <v>1.001733413065755</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="67" t="inlineStr">
         <is>
-          <t>3.0.2</t>
-        </is>
-      </c>
-      <c r="B10" s="46" t="n">
-        <v>7860480</v>
+          <t>3.1.2</t>
+        </is>
+      </c>
+      <c r="B10" s="58" t="n">
+        <v>1161</v>
       </c>
       <c r="C10" s="46" t="n">
-        <v>7634306</v>
-      </c>
-      <c r="D10" s="70" t="n">
-        <v>1.029626006607542</v>
-      </c>
-      <c r="E10" s="71" t="n">
-        <v>70</v>
-      </c>
-      <c r="F10" s="58" t="n">
-        <v>70</v>
-      </c>
-      <c r="G10" s="58" t="n">
+        <v>1161</v>
+      </c>
+      <c r="D10" s="46" t="n">
+        <v>1161</v>
+      </c>
+      <c r="E10" s="79" t="n">
+        <v>239</v>
+      </c>
+      <c r="F10" s="81" t="n">
+        <v>1.113639106928549</v>
+      </c>
+      <c r="G10" s="50" t="n">
+        <v>0.999877543964426</v>
+      </c>
+      <c r="H10" s="50" t="n">
+        <v>1.003088441366754</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>Scenario 3.0.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="72" t="inlineStr">
+        <is>
+          <t>LIM-LD year is 95.8% — under its line. No parking, no levelling needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>Scenario 3.0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="82" t="inlineStr">
+        <is>
+          <t>Fleet to own: 1244 DT, held every month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="44" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t>Fleet available</t>
+        </is>
+      </c>
+      <c r="C18" s="44" t="inlineStr">
+        <is>
+          <t>PARKED</t>
+        </is>
+      </c>
+      <c r="D18" s="44" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="E18" s="44" t="inlineStr"/>
+      <c r="F18" s="44" t="inlineStr"/>
+      <c r="G18" s="44" t="inlineStr"/>
+      <c r="H18" s="44" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="67" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="B19" s="46" t="n">
+        <v>581</v>
+      </c>
+      <c r="C19" s="69" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="50" t="n">
-        <v>1.0000909696791</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="67" t="inlineStr">
-        <is>
-          <t>3.1.1</t>
-        </is>
-      </c>
-      <c r="B11" s="46" t="n">
-        <v>6902523</v>
-      </c>
-      <c r="C11" s="46" t="n">
-        <v>6644306</v>
-      </c>
-      <c r="D11" s="70" t="n">
-        <v>1.038862900053068</v>
-      </c>
-      <c r="E11" s="71" t="n">
-        <v>79</v>
-      </c>
-      <c r="F11" s="58" t="n">
-        <v>79</v>
-      </c>
-      <c r="G11" s="58" t="n">
+      <c r="D19" s="58" t="n">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="67" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="B20" s="46" t="n">
+        <v>931</v>
+      </c>
+      <c r="C20" s="69" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="50" t="n">
-        <v>1.000408890947364</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="67" t="inlineStr">
-        <is>
-          <t>3.1.2</t>
-        </is>
-      </c>
-      <c r="B12" s="46" t="n">
-        <v>7399359</v>
-      </c>
-      <c r="C12" s="46" t="n">
-        <v>6644306</v>
-      </c>
-      <c r="D12" s="70" t="n">
-        <v>1.113639106928549</v>
-      </c>
-      <c r="E12" s="71" t="n">
-        <v>234</v>
-      </c>
-      <c r="F12" s="58" t="n">
-        <v>163</v>
-      </c>
-      <c r="G12" s="53" t="n">
-        <v>71</v>
-      </c>
-      <c r="H12" s="50" t="n">
-        <v>1.001169677059233</v>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="42" t="inlineStr">
-        <is>
-          <t>Reading: 3.0.1 needs no change — its year LIM-LD is already 95.8%, under the line. The other three each free trucks, and in 3.0.2 and 3.1.1 EVERY freed truck stays working on a longer haul, so nothing is wasted. Only 3.1.2, which runs 11.4% over, ends with trucks it genuinely does not need.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="41" t="inlineStr">
-        <is>
-          <t>Scenario 3.0.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="72" t="inlineStr">
-        <is>
-          <t>Year LIM-LD is 95.8% — already at or under the line. No adjustment needed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="41" t="inlineStr">
-        <is>
-          <t>Scenario 3.0.2</t>
-        </is>
+      <c r="D20" s="58" t="n">
+        <v>931</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="44" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
-      <c r="B21" s="44" t="inlineStr">
-        <is>
-          <t>LIM-LD before</t>
-        </is>
-      </c>
-      <c r="C21" s="44" t="inlineStr">
-        <is>
-          <t>LIM-LD after</t>
-        </is>
-      </c>
-      <c r="D21" s="44" t="inlineStr">
-        <is>
-          <t>Tonnes removed</t>
-        </is>
-      </c>
-      <c r="E21" s="44" t="inlineStr">
-        <is>
-          <t>DT freed</t>
-        </is>
-      </c>
-      <c r="F21" s="44" t="inlineStr">
-        <is>
-          <t>Kept working</t>
-        </is>
-      </c>
-      <c r="G21" s="44" t="inlineStr">
-        <is>
-          <t>Not needed</t>
-        </is>
-      </c>
-      <c r="H21" s="44" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
+      <c r="A21" s="67" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="B21" s="46" t="n">
+        <v>1280</v>
+      </c>
+      <c r="C21" s="53" t="n">
+        <v>36</v>
+      </c>
+      <c r="D21" s="58" t="n">
+        <v>1244</v>
       </c>
     </row>
     <row r="22">
@@ -2746,209 +2779,124 @@
           <t>Dec</t>
         </is>
       </c>
-      <c r="B22" s="70" t="n">
-        <v>1.200776731495626</v>
-      </c>
-      <c r="C22" s="50" t="n">
-        <v>1.086532089127519</v>
-      </c>
-      <c r="D22" s="46" t="n">
-        <v>225480</v>
-      </c>
-      <c r="E22" s="71" t="n">
-        <v>70</v>
-      </c>
-      <c r="F22" s="73" t="n">
-        <v>70</v>
-      </c>
-      <c r="G22" s="73" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="74" t="inlineStr">
-        <is>
-          <t>from RIM 61 DT + SMA 9 DT · stays above its own line, the YEAR is what lands on 100%</t>
-        </is>
+      <c r="B22" s="46" t="n">
+        <v>1281</v>
+      </c>
+      <c r="C22" s="53" t="n">
+        <v>37</v>
+      </c>
+      <c r="D22" s="58" t="n">
+        <v>1244</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="75" t="inlineStr">
         <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="D23" s="48" t="n">
-        <v>225480</v>
-      </c>
-      <c r="E23" s="71" t="n">
-        <v>70</v>
-      </c>
-      <c r="F23" s="73" t="n">
-        <v>70</v>
-      </c>
-      <c r="G23" s="73" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="76" t="inlineStr">
-        <is>
-          <t>year LIM-LD 103.0% -&gt; 100.0%</t>
-        </is>
+          <t>TOTAL parked</t>
+        </is>
+      </c>
+      <c r="C23" s="79" t="n">
+        <v>73</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="77" t="inlineStr">
-        <is>
-          <t>Where the kept trucks work — same SAP tonnage, longer haul</t>
-        </is>
-      </c>
+      <c r="A25" s="44" t="inlineStr">
+        <is>
+          <t>Sep–Dec year</t>
+        </is>
+      </c>
+      <c r="B25" s="44" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="C25" s="44" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="D25" s="44" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="E25" s="44" t="inlineStr">
+        <is>
+          <t>Together</t>
+        </is>
+      </c>
+      <c r="F25" s="44" t="inlineStr"/>
+      <c r="G25" s="44" t="inlineStr"/>
+      <c r="H25" s="44" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="44" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
-      <c r="B26" s="44" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="C26" s="44" t="inlineStr">
-        <is>
-          <t>Moved from</t>
-        </is>
-      </c>
-      <c r="D26" s="44" t="inlineStr">
-        <is>
-          <t>Moved to</t>
-        </is>
-      </c>
-      <c r="E26" s="44" t="inlineStr">
-        <is>
-          <t>SAP t/day shifted</t>
-        </is>
-      </c>
-      <c r="F26" s="44" t="inlineStr">
-        <is>
-          <t>DT off</t>
-        </is>
-      </c>
-      <c r="G26" s="44" t="inlineStr">
-        <is>
-          <t>DT on</t>
-        </is>
-      </c>
-      <c r="H26" s="44" t="inlineStr">
-        <is>
-          <t>Extra DT used</t>
-        </is>
+      <c r="A26" s="67" t="inlineStr">
+        <is>
+          <t>Sales line t</t>
+        </is>
+      </c>
+      <c r="B26" s="46" t="n">
+        <v>5718685</v>
+      </c>
+      <c r="C26" s="46" t="n">
+        <v>3650201</v>
+      </c>
+      <c r="D26" s="46" t="n">
+        <v>7634306</v>
+      </c>
+      <c r="E26" s="48" t="n">
+        <v>17003192</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="45" t="inlineStr">
-        <is>
-          <t>Dec</t>
-        </is>
-      </c>
-      <c r="B27" s="67" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C27" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="D27" s="56" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E27" s="46" t="n">
-        <v>14384</v>
-      </c>
-      <c r="F27" s="78" t="n">
-        <v>136</v>
-      </c>
-      <c r="G27" s="73" t="n">
-        <v>183</v>
-      </c>
-      <c r="H27" s="58" t="n">
-        <v>47</v>
+      <c r="A27" s="67" t="inlineStr">
+        <is>
+          <t>Year predicted</t>
+        </is>
+      </c>
+      <c r="B27" s="48" t="n">
+        <v>5754365</v>
+      </c>
+      <c r="C27" s="48" t="n">
+        <v>3672447</v>
+      </c>
+      <c r="D27" s="48" t="n">
+        <v>7629845</v>
+      </c>
+      <c r="E27" s="48" t="n">
+        <v>17056657</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="45" t="inlineStr">
-        <is>
-          <t>Dec</t>
-        </is>
-      </c>
-      <c r="B28" s="67" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C28" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;POS 12</t>
-        </is>
-      </c>
-      <c r="D28" s="56" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E28" s="46" t="n">
-        <v>1992</v>
-      </c>
-      <c r="F28" s="78" t="n">
-        <v>18</v>
-      </c>
-      <c r="G28" s="73" t="n">
-        <v>32</v>
-      </c>
-      <c r="H28" s="58" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="45" t="inlineStr">
-        <is>
-          <t>Dec</t>
-        </is>
-      </c>
-      <c r="B29" s="67" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C29" s="51" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="D29" s="56" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E29" s="46" t="n">
-        <v>2563</v>
-      </c>
-      <c r="F29" s="78" t="n">
-        <v>16</v>
-      </c>
-      <c r="G29" s="73" t="n">
-        <v>25</v>
-      </c>
-      <c r="H29" s="58" t="n">
-        <v>9</v>
+      <c r="A28" s="67" t="inlineStr">
+        <is>
+          <t>YEAR % of target</t>
+        </is>
+      </c>
+      <c r="B28" s="50" t="n">
+        <v>1.006239196598519</v>
+      </c>
+      <c r="C28" s="50" t="n">
+        <v>1.006094458907879</v>
+      </c>
+      <c r="D28" s="50" t="n">
+        <v>0.9994156617947111</v>
+      </c>
+      <c r="E28" s="50" t="n">
+        <v>1.00314440861065</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="41" t="inlineStr">
+        <is>
+          <t>Scenario 3.1.1</t>
+        </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="41" t="inlineStr">
-        <is>
-          <t>Scenario 3.1.1</t>
+      <c r="A32" s="82" t="inlineStr">
+        <is>
+          <t>Fleet to own: 1239 DT, held every month.</t>
         </is>
       </c>
     </row>
@@ -2960,833 +2908,390 @@
       </c>
       <c r="B33" s="44" t="inlineStr">
         <is>
-          <t>LIM-LD before</t>
+          <t>Fleet available</t>
         </is>
       </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
-          <t>LIM-LD after</t>
+          <t>PARKED</t>
         </is>
       </c>
       <c r="D33" s="44" t="inlineStr">
         <is>
-          <t>Tonnes removed</t>
-        </is>
-      </c>
-      <c r="E33" s="44" t="inlineStr">
-        <is>
-          <t>DT freed</t>
-        </is>
-      </c>
-      <c r="F33" s="44" t="inlineStr">
-        <is>
-          <t>Kept working</t>
-        </is>
-      </c>
-      <c r="G33" s="44" t="inlineStr">
-        <is>
-          <t>Not needed</t>
-        </is>
-      </c>
-      <c r="H33" s="44" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="E33" s="44" t="inlineStr"/>
+      <c r="F33" s="44" t="inlineStr"/>
+      <c r="G33" s="44" t="inlineStr"/>
+      <c r="H33" s="44" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="67" t="inlineStr">
         <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="B34" s="46" t="n">
+        <v>581</v>
+      </c>
+      <c r="C34" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="58" t="n">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="67" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="B35" s="46" t="n">
+        <v>931</v>
+      </c>
+      <c r="C35" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="58" t="n">
+        <v>931</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="67" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="B36" s="46" t="n">
+        <v>1280</v>
+      </c>
+      <c r="C36" s="53" t="n">
+        <v>41</v>
+      </c>
+      <c r="D36" s="58" t="n">
+        <v>1239</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="67" t="inlineStr">
+        <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="B34" s="70" t="n">
-        <v>1.20840925422352</v>
-      </c>
-      <c r="C34" s="50" t="n">
-        <v>1.057795449860331</v>
-      </c>
-      <c r="D34" s="46" t="n">
-        <v>255500</v>
-      </c>
-      <c r="E34" s="71" t="n">
-        <v>79</v>
-      </c>
-      <c r="F34" s="73" t="n">
-        <v>79</v>
-      </c>
-      <c r="G34" s="73" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" s="74" t="inlineStr">
-        <is>
-          <t>from RIM 61 DT + SMA 18 DT · stays above its own line, the YEAR is what lands on 100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="75" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="D35" s="48" t="n">
-        <v>255500</v>
-      </c>
-      <c r="E35" s="71" t="n">
-        <v>79</v>
-      </c>
-      <c r="F35" s="73" t="n">
-        <v>79</v>
-      </c>
-      <c r="G35" s="73" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="76" t="inlineStr">
-        <is>
-          <t>year LIM-LD 103.9% -&gt; 100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="77" t="inlineStr">
-        <is>
-          <t>Where the kept trucks work — same SAP tonnage, longer haul</t>
-        </is>
+      <c r="B37" s="46" t="n">
+        <v>1281</v>
+      </c>
+      <c r="C37" s="53" t="n">
+        <v>42</v>
+      </c>
+      <c r="D37" s="58" t="n">
+        <v>1239</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="44" t="inlineStr">
+      <c r="A38" s="75" t="inlineStr">
+        <is>
+          <t>TOTAL parked</t>
+        </is>
+      </c>
+      <c r="C38" s="79" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="44" t="inlineStr">
+        <is>
+          <t>Sep–Dec year</t>
+        </is>
+      </c>
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="C40" s="44" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="D40" s="44" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="E40" s="44" t="inlineStr">
+        <is>
+          <t>Together</t>
+        </is>
+      </c>
+      <c r="F40" s="44" t="inlineStr"/>
+      <c r="G40" s="44" t="inlineStr"/>
+      <c r="H40" s="44" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="67" t="inlineStr">
+        <is>
+          <t>Sales line t</t>
+        </is>
+      </c>
+      <c r="B41" s="46" t="n">
+        <v>5718685</v>
+      </c>
+      <c r="C41" s="46" t="n">
+        <v>4640202</v>
+      </c>
+      <c r="D41" s="46" t="n">
+        <v>6644306</v>
+      </c>
+      <c r="E41" s="48" t="n">
+        <v>17003193</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="67" t="inlineStr">
+        <is>
+          <t>Year predicted</t>
+        </is>
+      </c>
+      <c r="B42" s="48" t="n">
+        <v>5740906</v>
+      </c>
+      <c r="C42" s="48" t="n">
+        <v>4652858</v>
+      </c>
+      <c r="D42" s="48" t="n">
+        <v>6638903</v>
+      </c>
+      <c r="E42" s="48" t="n">
+        <v>17032667</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="67" t="inlineStr">
+        <is>
+          <t>YEAR % of target</t>
+        </is>
+      </c>
+      <c r="B43" s="50" t="n">
+        <v>1.003885683509408</v>
+      </c>
+      <c r="C43" s="50" t="n">
+        <v>1.002727467468011</v>
+      </c>
+      <c r="D43" s="50" t="n">
+        <v>0.9991867558336038</v>
+      </c>
+      <c r="E43" s="50" t="n">
+        <v>1.001733413065755</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="41" t="inlineStr">
+        <is>
+          <t>Scenario 3.1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="82" t="inlineStr">
+        <is>
+          <t>Fleet to own: 1161 DT, held every month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="44" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B38" s="44" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="C38" s="44" t="inlineStr">
-        <is>
-          <t>Moved from</t>
-        </is>
-      </c>
-      <c r="D38" s="44" t="inlineStr">
-        <is>
-          <t>Moved to</t>
-        </is>
-      </c>
-      <c r="E38" s="44" t="inlineStr">
-        <is>
-          <t>SAP t/day shifted</t>
-        </is>
-      </c>
-      <c r="F38" s="44" t="inlineStr">
-        <is>
-          <t>DT off</t>
-        </is>
-      </c>
-      <c r="G38" s="44" t="inlineStr">
-        <is>
-          <t>DT on</t>
-        </is>
-      </c>
-      <c r="H38" s="44" t="inlineStr">
-        <is>
-          <t>Extra DT used</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="45" t="inlineStr">
-        <is>
-          <t>Dec</t>
-        </is>
-      </c>
-      <c r="B39" s="67" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C39" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="D39" s="56" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E39" s="46" t="n">
-        <v>14384</v>
-      </c>
-      <c r="F39" s="78" t="n">
-        <v>136</v>
-      </c>
-      <c r="G39" s="73" t="n">
-        <v>183</v>
-      </c>
-      <c r="H39" s="58" t="n">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="45" t="inlineStr">
-        <is>
-          <t>Dec</t>
-        </is>
-      </c>
-      <c r="B40" s="67" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C40" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;POS 12</t>
-        </is>
-      </c>
-      <c r="D40" s="56" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E40" s="46" t="n">
-        <v>1992</v>
-      </c>
-      <c r="F40" s="78" t="n">
-        <v>18</v>
-      </c>
-      <c r="G40" s="73" t="n">
-        <v>32</v>
-      </c>
-      <c r="H40" s="58" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="45" t="inlineStr">
-        <is>
-          <t>Dec</t>
-        </is>
-      </c>
-      <c r="B41" s="67" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C41" s="51" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="D41" s="56" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E41" s="46" t="n">
-        <v>5125</v>
-      </c>
-      <c r="F41" s="78" t="n">
-        <v>32</v>
-      </c>
-      <c r="G41" s="73" t="n">
-        <v>50</v>
-      </c>
-      <c r="H41" s="58" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="41" t="inlineStr">
-        <is>
-          <t>Scenario 3.1.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="44" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
-      <c r="B45" s="44" t="inlineStr">
-        <is>
-          <t>LIM-LD before</t>
-        </is>
-      </c>
-      <c r="C45" s="44" t="inlineStr">
-        <is>
-          <t>LIM-LD after</t>
-        </is>
-      </c>
-      <c r="D45" s="44" t="inlineStr">
-        <is>
-          <t>Tonnes removed</t>
-        </is>
-      </c>
-      <c r="E45" s="44" t="inlineStr">
-        <is>
-          <t>DT freed</t>
-        </is>
-      </c>
-      <c r="F45" s="44" t="inlineStr">
-        <is>
-          <t>Kept working</t>
-        </is>
-      </c>
-      <c r="G45" s="44" t="inlineStr">
-        <is>
-          <t>Not needed</t>
-        </is>
-      </c>
-      <c r="H45" s="44" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="67" t="inlineStr">
-        <is>
-          <t>Dec</t>
-        </is>
-      </c>
-      <c r="B46" s="70" t="n">
-        <v>1.307911551155894</v>
-      </c>
-      <c r="C46" s="50" t="n">
-        <v>1.001860148915527</v>
-      </c>
-      <c r="D46" s="46" t="n">
-        <v>519183</v>
-      </c>
-      <c r="E46" s="71" t="n">
-        <v>161</v>
-      </c>
-      <c r="F46" s="73" t="n">
-        <v>94</v>
-      </c>
-      <c r="G46" s="79" t="n">
-        <v>67</v>
-      </c>
-      <c r="H46" s="74" t="inlineStr">
-        <is>
-          <t>from RIM 128 DT + SMA 33 DT · stays above its own line, the YEAR is what lands on 100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="67" t="inlineStr">
-        <is>
-          <t>Nov</t>
-        </is>
-      </c>
-      <c r="B47" s="70" t="n">
-        <v>1.085941499180451</v>
-      </c>
-      <c r="C47" s="50" t="n">
-        <v>1.000181011689175</v>
-      </c>
-      <c r="D47" s="46" t="n">
-        <v>199032</v>
-      </c>
-      <c r="E47" s="71" t="n">
-        <v>64</v>
-      </c>
-      <c r="F47" s="73" t="n">
-        <v>60</v>
-      </c>
-      <c r="G47" s="79" t="n">
-        <v>4</v>
-      </c>
-      <c r="H47" s="74" t="inlineStr">
-        <is>
-          <t>from RIM 43 DT + SMA 21 DT · stays above its own line, the YEAR is what lands on 100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="67" t="inlineStr">
-        <is>
-          <t>Sep</t>
-        </is>
-      </c>
-      <c r="B48" s="70" t="n">
-        <v>1.013678484229764</v>
-      </c>
-      <c r="C48" s="50" t="n">
-        <v>1.002329219968693</v>
-      </c>
-      <c r="D48" s="46" t="n">
-        <v>9538</v>
-      </c>
-      <c r="E48" s="71" t="n">
-        <v>3</v>
-      </c>
-      <c r="F48" s="73" t="n">
-        <v>3</v>
-      </c>
-      <c r="G48" s="73" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="74" t="inlineStr">
-        <is>
-          <t>from RIM 3 DT · stays above its own line, the YEAR is what lands on 100%</t>
-        </is>
-      </c>
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>Fleet available</t>
+        </is>
+      </c>
+      <c r="C48" s="44" t="inlineStr">
+        <is>
+          <t>PARKED</t>
+        </is>
+      </c>
+      <c r="D48" s="44" t="inlineStr">
+        <is>
+          <t>RUNNING</t>
+        </is>
+      </c>
+      <c r="E48" s="44" t="inlineStr"/>
+      <c r="F48" s="44" t="inlineStr"/>
+      <c r="G48" s="44" t="inlineStr"/>
+      <c r="H48" s="44" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="67" t="inlineStr">
         <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="B49" s="46" t="n">
+        <v>581</v>
+      </c>
+      <c r="C49" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="58" t="n">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="67" t="inlineStr">
+        <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="B49" s="70" t="n">
-        <v>1.012182364954908</v>
-      </c>
-      <c r="C49" s="50" t="n">
-        <v>1.001252870546001</v>
-      </c>
-      <c r="D49" s="46" t="n">
-        <v>19528</v>
-      </c>
-      <c r="E49" s="71" t="n">
-        <v>6</v>
-      </c>
-      <c r="F49" s="73" t="n">
-        <v>6</v>
-      </c>
-      <c r="G49" s="73" t="n">
+      <c r="B50" s="46" t="n">
+        <v>931</v>
+      </c>
+      <c r="C50" s="69" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="74" t="inlineStr">
-        <is>
-          <t>from RIM 6 DT · stays above its own line, the YEAR is what lands on 100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="75" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="D50" s="48" t="n">
-        <v>747281</v>
-      </c>
-      <c r="E50" s="71" t="n">
-        <v>234</v>
-      </c>
-      <c r="F50" s="73" t="n">
-        <v>163</v>
-      </c>
-      <c r="G50" s="79" t="n">
-        <v>71</v>
-      </c>
-      <c r="H50" s="76" t="inlineStr">
-        <is>
-          <t>year LIM-LD 111.4% -&gt; 100.1%</t>
-        </is>
+      <c r="D50" s="58" t="n">
+        <v>931</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="67" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="B51" s="46" t="n">
+        <v>1280</v>
+      </c>
+      <c r="C51" s="53" t="n">
+        <v>119</v>
+      </c>
+      <c r="D51" s="58" t="n">
+        <v>1161</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="77" t="inlineStr">
-        <is>
-          <t>Where the kept trucks work — same SAP tonnage, longer haul</t>
-        </is>
+      <c r="A52" s="67" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="B52" s="46" t="n">
+        <v>1281</v>
+      </c>
+      <c r="C52" s="53" t="n">
+        <v>120</v>
+      </c>
+      <c r="D52" s="58" t="n">
+        <v>1161</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="44" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
-      <c r="B53" s="44" t="inlineStr">
-        <is>
-          <t>Contractor</t>
-        </is>
-      </c>
-      <c r="C53" s="44" t="inlineStr">
-        <is>
-          <t>Moved from</t>
-        </is>
-      </c>
-      <c r="D53" s="44" t="inlineStr">
-        <is>
-          <t>Moved to</t>
-        </is>
-      </c>
-      <c r="E53" s="44" t="inlineStr">
-        <is>
-          <t>SAP t/day shifted</t>
-        </is>
-      </c>
-      <c r="F53" s="44" t="inlineStr">
-        <is>
-          <t>DT off</t>
-        </is>
-      </c>
-      <c r="G53" s="44" t="inlineStr">
-        <is>
-          <t>DT on</t>
-        </is>
-      </c>
-      <c r="H53" s="44" t="inlineStr">
-        <is>
-          <t>Extra DT used</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="45" t="inlineStr">
-        <is>
-          <t>Dec</t>
-        </is>
-      </c>
-      <c r="B54" s="67" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C54" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="D54" s="56" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E54" s="46" t="n">
-        <v>14384</v>
-      </c>
-      <c r="F54" s="78" t="n">
-        <v>136</v>
-      </c>
-      <c r="G54" s="73" t="n">
-        <v>183</v>
-      </c>
-      <c r="H54" s="58" t="n">
-        <v>47</v>
+      <c r="A53" s="75" t="inlineStr">
+        <is>
+          <t>TOTAL parked</t>
+        </is>
+      </c>
+      <c r="C53" s="79" t="n">
+        <v>239</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="45" t="inlineStr">
-        <is>
-          <t>Dec</t>
-        </is>
-      </c>
-      <c r="B55" s="67" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C55" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;POS 12</t>
-        </is>
-      </c>
-      <c r="D55" s="56" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E55" s="46" t="n">
-        <v>1992</v>
-      </c>
-      <c r="F55" s="78" t="n">
-        <v>18</v>
-      </c>
-      <c r="G55" s="73" t="n">
-        <v>32</v>
-      </c>
-      <c r="H55" s="58" t="n">
-        <v>14</v>
-      </c>
+      <c r="A55" s="44" t="inlineStr">
+        <is>
+          <t>Sep–Dec year</t>
+        </is>
+      </c>
+      <c r="B55" s="44" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="C55" s="44" t="inlineStr">
+        <is>
+          <t>LIM-TOS</t>
+        </is>
+      </c>
+      <c r="D55" s="44" t="inlineStr">
+        <is>
+          <t>LIM-LD</t>
+        </is>
+      </c>
+      <c r="E55" s="44" t="inlineStr">
+        <is>
+          <t>Together</t>
+        </is>
+      </c>
+      <c r="F55" s="44" t="inlineStr"/>
+      <c r="G55" s="44" t="inlineStr"/>
+      <c r="H55" s="44" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="45" t="inlineStr">
-        <is>
-          <t>Dec</t>
-        </is>
-      </c>
-      <c r="B56" s="67" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C56" s="51" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="D56" s="56" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E56" s="46" t="n">
-        <v>7688</v>
-      </c>
-      <c r="F56" s="78" t="n">
-        <v>48</v>
-      </c>
-      <c r="G56" s="73" t="n">
-        <v>75</v>
-      </c>
-      <c r="H56" s="58" t="n">
-        <v>27</v>
+      <c r="A56" s="67" t="inlineStr">
+        <is>
+          <t>Sales line t</t>
+        </is>
+      </c>
+      <c r="B56" s="46" t="n">
+        <v>5718685</v>
+      </c>
+      <c r="C56" s="46" t="n">
+        <v>4640202</v>
+      </c>
+      <c r="D56" s="46" t="n">
+        <v>6644306</v>
+      </c>
+      <c r="E56" s="48" t="n">
+        <v>17003193</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="45" t="inlineStr">
-        <is>
-          <t>Dec</t>
-        </is>
-      </c>
-      <c r="B57" s="67" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C57" s="51" t="inlineStr">
-        <is>
-          <t>KR&gt;POS 12</t>
-        </is>
-      </c>
-      <c r="D57" s="56" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E57" s="46" t="n">
-        <v>1779</v>
-      </c>
-      <c r="F57" s="78" t="n">
-        <v>9</v>
-      </c>
-      <c r="G57" s="73" t="n">
-        <v>15</v>
-      </c>
-      <c r="H57" s="58" t="n">
-        <v>6</v>
+      <c r="A57" s="67" t="inlineStr">
+        <is>
+          <t>Year predicted</t>
+        </is>
+      </c>
+      <c r="B57" s="48" t="n">
+        <v>5753327</v>
+      </c>
+      <c r="C57" s="48" t="n">
+        <v>4658887</v>
+      </c>
+      <c r="D57" s="48" t="n">
+        <v>6643492</v>
+      </c>
+      <c r="E57" s="48" t="n">
+        <v>17055706</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="45" t="inlineStr">
-        <is>
-          <t>Nov</t>
-        </is>
-      </c>
-      <c r="B58" s="67" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C58" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="D58" s="56" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E58" s="46" t="n">
-        <v>7651</v>
-      </c>
-      <c r="F58" s="78" t="n">
-        <v>73</v>
-      </c>
-      <c r="G58" s="73" t="n">
-        <v>98</v>
-      </c>
-      <c r="H58" s="58" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="45" t="inlineStr">
-        <is>
-          <t>Nov</t>
-        </is>
-      </c>
-      <c r="B59" s="67" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C59" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;POS 12</t>
-        </is>
-      </c>
-      <c r="D59" s="56" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E59" s="46" t="n">
-        <v>1992</v>
-      </c>
-      <c r="F59" s="78" t="n">
-        <v>18</v>
-      </c>
-      <c r="G59" s="73" t="n">
-        <v>32</v>
-      </c>
-      <c r="H59" s="58" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="45" t="inlineStr">
-        <is>
-          <t>Nov</t>
-        </is>
-      </c>
-      <c r="B60" s="67" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C60" s="51" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="D60" s="56" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E60" s="46" t="n">
-        <v>3986</v>
-      </c>
-      <c r="F60" s="78" t="n">
-        <v>25</v>
-      </c>
-      <c r="G60" s="73" t="n">
-        <v>39</v>
-      </c>
-      <c r="H60" s="58" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="45" t="inlineStr">
-        <is>
-          <t>Nov</t>
-        </is>
-      </c>
-      <c r="B61" s="67" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="C61" s="51" t="inlineStr">
-        <is>
-          <t>KR&gt;POS 12</t>
-        </is>
-      </c>
-      <c r="D61" s="56" t="inlineStr">
-        <is>
-          <t>KR&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E61" s="46" t="n">
-        <v>2075</v>
-      </c>
-      <c r="F61" s="78" t="n">
-        <v>10</v>
-      </c>
-      <c r="G61" s="73" t="n">
-        <v>17</v>
-      </c>
-      <c r="H61" s="58" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="45" t="inlineStr">
-        <is>
-          <t>Sep</t>
-        </is>
-      </c>
-      <c r="B62" s="67" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C62" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="D62" s="56" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E62" s="46" t="n">
-        <v>918</v>
-      </c>
-      <c r="F62" s="78" t="n">
-        <v>9</v>
-      </c>
-      <c r="G62" s="73" t="n">
-        <v>12</v>
-      </c>
-      <c r="H62" s="58" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="45" t="inlineStr">
-        <is>
-          <t>Oct</t>
-        </is>
-      </c>
-      <c r="B63" s="67" t="inlineStr">
-        <is>
-          <t>RIM</t>
-        </is>
-      </c>
-      <c r="C63" s="51" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM15</t>
-        </is>
-      </c>
-      <c r="D63" s="56" t="inlineStr">
-        <is>
-          <t>TF&gt;FENI KM0</t>
-        </is>
-      </c>
-      <c r="E63" s="46" t="n">
-        <v>1836</v>
-      </c>
-      <c r="F63" s="78" t="n">
-        <v>17</v>
-      </c>
-      <c r="G63" s="73" t="n">
-        <v>23</v>
-      </c>
-      <c r="H63" s="58" t="n">
-        <v>6</v>
+      <c r="A58" s="67" t="inlineStr">
+        <is>
+          <t>YEAR % of target</t>
+        </is>
+      </c>
+      <c r="B58" s="50" t="n">
+        <v>1.00605768633873</v>
+      </c>
+      <c r="C58" s="50" t="n">
+        <v>1.004026764352069</v>
+      </c>
+      <c r="D58" s="50" t="n">
+        <v>0.999877543964426</v>
+      </c>
+      <c r="E58" s="50" t="n">
+        <v>1.003088441366754</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="2">
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A5:H5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>